<commit_message>
Mise à jour des annonces — 2026-07-14 08:06
</commit_message>
<xml_diff>
--- a/annonces.xlsx
+++ b/annonces.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Annonces" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -576,32 +576,32 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Condo 3 chambres, 1100 pi², 2 balcons – Centre-Sud, près métro Frontenac</t>
+          <t>Grand 4 1/2 avec balcon, wifi et électros neufs inclus – Hochelaga</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Centre-Sud</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2553 Avenue Gascon, Montréal, QC H2K 2W5</t>
+          <t>Montréal, QC H1W 3N5</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2090</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Frontenac</t>
+          <t>Joliette ou Pie-IX</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>quelques min (estimé)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-1100pc-3ch-pres-metro-et-plateau/1740479448</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-4-1-2-avec-balcon-wifi-electros-inclus/1740319117</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>3 chambres fermées + bureau, 2 balcons, planchers bois franc, grande fenestration, animaux acceptés, dispo 1er août 2026, bail 1 an, secteur vivant à la frontière Plateau/Hochelaga (rue Ontario), aucun stationnement inclus</t>
+          <t>2 chambres fermées + den, grand balcon arrière vue jardin, wifi et électroménagers neufs inclus (laveuse-sécheuse, lave-vaisselle, thermopompe/climatisation), salle de bain rénovée 2025, non-fumeur, pas d'animaux, dispo 1er août 2026 (possibilité plus tôt), bail 1 an</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/6c/6c93d656-ed7d-413a-ac8b-986e4f7f2eda?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/20/2040a77c-67f8-4d3c-8b23-22071ed8ca1b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>4 1/2 (2 chambres), 900 pi², balcon, tout inclus – Rosemont (rue Dandurand)</t>
+          <t>Condo 5½ meublé, balcon vue sur parc – Angus/Rosemont, près métro Joliette</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -673,17 +673,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>3320 Rue Dandurand, Montréal, QC H1X 1M6</t>
+          <t>3439 Rue William-Tremblay, Montréal</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -698,136 +698,128 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Iberville</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>5 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-a-louer-2-chambres-rosemont-petite-patrie-tout-inclus/1739170766</t>
+          <t>https://www.logisquebec.com/condo-a-louer-rosemont_la-petite-patrie-l353563</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Construit 2012, tout inclus (chauffage, hydro, eau, wifi, climatisation), semi-meublé (électros + meubles salon/cuisine, matelas non inclus), animaux limités, dispo 1er juillet 2026, à 5-10 min à pied des commerces/restos de la rue Masson</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ba/bacee7d5-1abf-4a36-80b6-12877aa40971?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>Unité de coin entièrement meublée (TV, lit, sofa, climatiseur portatif, électros inclus), vue sur parc, arrêt de bus à 1 min vers le métro, électricité et internet en sus (~70$/mois chacun), dispo 1er août ou 1er sept 2026, secteur Angus vivant (écoles, parcs, commerces à pied)</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>vu</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>6 et demi avec cour arrière privative - Villeray - 1er juillet!</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Villeray</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>8413 rue Saint-Hubert, Montréal, QC H2P 1Z6</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>1950</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>NOUVEAU</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Condo 4½ neuf sur 2 étages, semi-meublé, balcon – Plateau/Centre-Sud, près métro Préfontaine</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2484 Rue Marie-Anne Est, Montréal</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2075</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>Jarry</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Préfontaine</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N4" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/6-et-demi-avec-cour-arriere-privative-villeray-1er-juillet/1734943312</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="P4" s="6" t="inlineStr">
-        <is>
-          <t>Dispo 1er juillet 2026, prix promo 12 mois (régulier 2050$), RDC + sous-sol aménagé, cour arrière privée, lave-vaisselle inclus, option 4 électros +100$/mois, 1 chat ou petit chien accepté</t>
-        </is>
-      </c>
-      <c r="Q4" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8a/8a62cfb1-09e6-4e8b-bc96-fe68a77e35b2?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>LogisQuébec</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.logisquebec.com/condo-a-louer-le-plateau-mont-royal-l353552</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Condo construit en 2019, climatisation centrale, système d'alarme, entrées laveuse-sécheuse, dispo 1er sept 2026, station Frontenac aussi accessible à 12 min</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -837,32 +829,32 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Beau 6 1/2 ensoleillé - proche metro - Hochelaga</t>
+          <t>Condo 3 chambres, 1100 pi², 2 balcons – Centre-Sud, près métro Frontenac</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Centre-Sud</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H1W 1M3</t>
+          <t>2553 Avenue Gascon, Montréal, QC H2K 2W5</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2090</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -872,7 +864,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Frontenac</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -882,7 +874,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
@@ -892,29 +884,29 @@
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/beau-6-1-2-ensoleille-proche-metro-hochelaga/1738000997</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-1100pc-3ch-pres-metro-et-plateau/1740479448</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er juin 2026, eau incluse, 4 électros inclus (frigo cuisinière laveuse sécheuse), 2e étage, plafonds hauts, animaux limités, près Promenade Ontario</t>
+          <t>3 chambres fermées + bureau, 2 balcons, planchers bois franc, grande fenestration, animaux acceptés, dispo 1er août 2026, bail 1 an, secteur vivant à la frontière Plateau/Hochelaga (rue Ontario), aucun stationnement inclus</t>
         </is>
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/77/77a71464-4b91-4435-bf29-e86a1a84a6a8?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/6c/6c93d656-ed7d-413a-ac8b-986e4f7f2eda?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -924,32 +916,32 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Grand 6 1/2 Villeray, metro Jarry</t>
+          <t>4 1/2 (2 chambres), 900 pi², balcon, tout inclus – Rosemont (rue Dandurand)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H2R 2E8</t>
+          <t>3320 Rue Dandurand, Montréal, QC H1X 1M6</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>1999</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>1250</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -959,17 +951,17 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Iberville</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5 (estimé)</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
@@ -979,22 +971,22 @@
       </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-6-1-2-villeray-metro-jarry/1740222569</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-a-louer-2-chambres-rosemont-petite-patrie-tout-inclus/1739170766</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er août 2026 (ou 1er juillet), 2 balcons (avant + grand arrière), 3 chambres fermées, électros non inclus mais négociable, pas d'animaux, non-fumeur, chauffage/électricité aux frais du locataire</t>
+          <t>Construit 2012, tout inclus (chauffage, hydro, eau, wifi, climatisation), semi-meublé (électros + meubles salon/cuisine, matelas non inclus), animaux limités, dispo 1er juillet 2026, à 5-10 min à pied des commerces/restos de la rue Masson</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/41/41b6a01a-67b3-4d74-8966-ac23a1a991aa?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ba/bacee7d5-1abf-4a36-80b6-12877aa40971?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1011,32 +1003,32 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 rénové, grand balcon, près métro Joliette/Pie-IX</t>
+          <t>6 et demi avec cour arrière privative - Villeray - 1er juillet!</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>1695 Avenue Bourbonnière, Montréal</t>
+          <t>8413 rue Saint-Hubert, Montréal, QC H2P 1Z6</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1046,42 +1038,42 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Joliette/Pie-IX</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/mercier-hochelaga-maisonneuve/4-1-2-a-louer/hab-1695-avenue-bourbonniere-1135855</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/6-et-demi-avec-cour-arriere-privative-villeray-1er-juillet/1734943312</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>2 ch fermées (1 grande chambre double) + salle d'eau, grand balcon arrière sur jardin paisible, dispo 1er août 2026 (ou 18 juillet), à 1 min du Metro épicerie, 3 min boulangerie Arhoma, Promenade Ontario et Place Simon-Valois à pied</t>
+          <t>Dispo 1er juillet 2026, prix promo 12 mois (régulier 2050$), RDC + sous-sol aménagé, cour arrière privée, lave-vaisselle inclus, option 4 électros +100$/mois, 1 chat ou petit chien accepté</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135855/mercier-hochelaga-maisonneuve-600-15749477.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8a/8a62cfb1-09e6-4e8b-bc96-fe68a77e35b2?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1098,32 +1090,32 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 balcon, 1200 pi² – Rosemont</t>
+          <t>Beau 6 1/2 ensoleillé - proche metro - Hochelaga</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>6885 43e Avenue, Montréal, QC H1T 2R9</t>
+          <t>Montréal, QC H1W 1M3</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1133,17 +1125,17 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Mary Two-Axe Earley (à vérifier)</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
@@ -1153,22 +1145,22 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-bedroom-apartment-for-rent-in-rosemont/1739297378</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/beau-6-1-2-ensoleille-proche-metro-hochelaga/1738000997</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>Animaux permis, eau chaude incluse, électricité et internet à la charge du locataire, libre 16 juin 2026, nom de station à vérifier</t>
+          <t>Dispo 1er juin 2026, eau incluse, 4 électros inclus (frigo cuisinière laveuse sécheuse), 2e étage, plafonds hauts, animaux limités, près Promenade Ontario</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2efd08ab-2014-42f0-bde7-3afc97ccb893?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/77/77a71464-4b91-4435-bf29-e86a1a84a6a8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1185,27 +1177,27 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 style condo, 2 balcons – Rosemont (Promenade Masson)</t>
+          <t>Grand 6 1/2 Villeray, metro Jarry</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1Y 1Y3, secteur Promenade Masson)</t>
+          <t>Montréal, QC H2R 2E8</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>1925</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1250</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1220,7 +1212,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Laurier</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -1230,7 +1222,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>n/d (bus ~20 min)</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
@@ -1240,22 +1232,22 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cessation-de-bail-5-style-condo-promenade-masson-rosemont/1739478440</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-6-1-2-villeray-metro-jarry/1740222569</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>Chiens et chats acceptés, chauffage non inclus, Walk Score 99, très proche des commerces de la Promenade Masson</t>
+          <t>Dispo 1er août 2026 (ou 1er juillet), 2 balcons (avant + grand arrière), 3 chambres fermées, électros non inclus mais négociable, pas d'animaux, non-fumeur, chauffage/électricité aux frais du locataire</t>
         </is>
       </c>
       <c r="Q9" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/21/219d597c-7a1f-471a-9c6c-a7768c42324c?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/41/41b6a01a-67b3-4d74-8966-ac23a1a991aa?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1272,32 +1264,32 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 1000 pi², balcon – Rosemont/Beaubien</t>
+          <t>4 1/2 rénové, grand balcon, près métro Joliette/Pie-IX</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Rue de Normanville, Montréal, QC H2S 2B5</t>
+          <t>1695 Avenue Bourbonnière, Montréal</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1307,27 +1299,27 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Rosemont/Beaubien</t>
+          <t>Joliette/Pie-IX</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appart-5-1-2-a-louer-3-bed-apartment-for-rent-la-petite-patrie/1740477077</t>
+          <t>https://duproprio.com/fr/location/montreal/mercier-hochelaga-maisonneuve/4-1-2-a-louer/hab-1695-avenue-bourbonniere-1135855</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1337,10 +1329,14 @@
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>1 mois gratuit 1ère année (régulier 2160$), animaux non acceptés, près du parc Père-Marquette, libre 12 juillet 2026</t>
-        </is>
-      </c>
-      <c r="Q10" s="5" t="inlineStr"/>
+          <t>2 ch fermées (1 grande chambre double) + salle d'eau, grand balcon arrière sur jardin paisible, dispo 1er août 2026 (ou 18 juillet), à 1 min du Metro épicerie, 3 min boulangerie Arhoma, Promenade Ontario et Place Simon-Valois à pied</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135855/mercier-hochelaga-maisonneuve-600-15749477.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1355,22 +1351,22 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Appartement 3 chambres, jardin, parking, Hochelaga</t>
+          <t>5 1/2 balcon, 1200 pi² – Rosemont</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H1W 3A8</t>
+          <t>6885 43e Avenue, Montréal, QC H1T 2R9</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>2135</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -1385,22 +1381,22 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Mary Two-Axe Earley (à vérifier)</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>Joliette</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
@@ -1410,7 +1406,7 @@
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-3-chambres-jardin-parking-hochelaga/1739953364</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-bedroom-apartment-for-rent-in-rosemont/1739297378</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
@@ -1420,12 +1416,12 @@
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail jusqu'au 1er juillet 2027, dispo 1er sept 2026, cour privée, stationnement, rangement au sous-sol, lave-vaisselle inclus, animaux limités, enquête de crédit</t>
+          <t>Animaux permis, eau chaude incluse, électricité et internet à la charge du locataire, libre 16 juin 2026, nom de station à vérifier</t>
         </is>
       </c>
       <c r="Q11" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/43/4348c9c2-4f70-41ce-a65d-9ed5490935cd?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2efd08ab-2014-42f0-bde7-3afc97ccb893?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1442,32 +1438,32 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>5½ meublé tout inclus à 3 min du métro Joliette</t>
+          <t>5 1/2 style condo, 2 balcons – Rosemont (Promenade Masson)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>3602 rue de Rouen, Montréal</t>
+          <t>n/d (Montréal, QC H1Y 1Y3, secteur Promenade Masson)</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>1925</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -1477,27 +1473,27 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>n/d (bus ~20 min)</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-mercier_hochelaga-maisonneuve-l353091</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cessation-de-bail-5-style-condo-promenade-masson-rosemont/1739478440</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -1507,10 +1503,14 @@
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>5½ 900 pi² meublé, chauffé, wifi et tout inclus, grande terrasse arrière 100 pi², métro Joliette à 287 m, disponible 11 octobre 2026, bail min 3 mois, pas d'animaux</t>
-        </is>
-      </c>
-      <c r="Q12" s="5" t="inlineStr"/>
+          <t>Chiens et chats acceptés, chauffage non inclus, Walk Score 99, très proche des commerces de la Promenade Masson</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/21/219d597c-7a1f-471a-9c6c-a7768c42324c?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1525,27 +1525,27 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 + annexe rénové près du métro Beaubien</t>
+          <t>5 1/2, 1000 pi², balcon – Rosemont/Beaubien</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>La Petite-Patrie</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>secteur métro Beaubien, H2S 2J5</t>
+          <t>Rue de Normanville, Montréal, QC H2S 2B5</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>1064</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Rosemont/Beaubien</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-annexe-renove-pres-du-metro-beaubien/1735720589</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appart-5-1-2-a-louer-3-bed-apartment-for-rent-la-petite-patrie/1740477077</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -1590,14 +1590,10 @@
       </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées + annexe (ancien solarium), rénové récemment, 2 grands balcons, entrées laveuse-sécheuse et lave-vaisselle, climatisation, dispo 1er sept 2026, rue Beaubien et commerces à pied, non-fumeur, pas d'animaux</t>
-        </is>
-      </c>
-      <c r="Q13" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ca/ca9a1937-a625-413b-ba4b-233b3a0e900b?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>1 mois gratuit 1ère année (régulier 2160$), animaux non acceptés, près du parc Père-Marquette, libre 12 juillet 2026</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1612,27 +1608,27 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Magnifique 5 1/2 sur le plateau mont-royal</t>
+          <t>Appartement 3 chambres, jardin, parking, Hochelaga</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>rue Marie-Anne, H2H 1M9</t>
+          <t>Montréal, QC H1W 3A8</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>2135</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1642,22 +1638,22 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
@@ -1667,7 +1663,7 @@
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/magnifique-5-1-2-sur-le-plateau-mont-royal/1734803750</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-3-chambres-jardin-parking-hochelaga/1739953364</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -1677,12 +1673,12 @@
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées, cuisine rénovée comptoirs quartz, planchers bois franc d'origine, laveuse-sécheuse dans l'unité, balcon privé, animaux acceptés, bail au mois, avenue Mont-Royal et ses commerces à pied, chauffage/électricité en sus</t>
+          <t>Cession de bail jusqu'au 1er juillet 2027, dispo 1er sept 2026, cour privée, stationnement, rangement au sous-sol, lave-vaisselle inclus, animaux limités, enquête de crédit</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/38/389e0d3d-7bcf-42a9-8fe4-8a27fa531359?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/43/4348c9c2-4f70-41ce-a65d-9ed5490935cd?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1695,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Unité neuve 3 chambres 1120 pi2 projet boutique</t>
+          <t>5½ meublé tout inclus à 3 min du métro Joliette</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1709,32 +1705,32 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>2017, avenue Letourneux, app. 101, Montréal</t>
+          <t>3602 rue de Rouen, Montréal</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>1120</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Pie-IX</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -1744,17 +1740,17 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/27359064</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-mercier_hochelaga-maisonneuve-l353091</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
@@ -1764,14 +1760,10 @@
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>Construction neuve 2026, 6 pièces, 3 chambres en demi-sous-sol, terrasse commune sur le toit, semi-meublé, internet inclus, 1 mois gratuit bail 24 mois, dispo 1er juillet 2026</t>
-        </is>
-      </c>
-      <c r="Q15" s="5" t="inlineStr">
-        <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15A15CDDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
-        </is>
-      </c>
+          <t>5½ 900 pi² meublé, chauffé, wifi et tout inclus, grande terrasse arrière 100 pi², métro Joliette à 287 m, disponible 11 octobre 2026, bail min 3 mois, pas d'animaux</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1786,27 +1778,27 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Plateau - Superbe 5 1/2 de 3 Chambres - Disponible le 1er Juillet</t>
+          <t>5 1/2 + annexe rénové près du métro Beaubien</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>La Petite-Patrie</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>3477 rue Saint-Dominique, H2X 2X5</t>
+          <t>secteur métro Beaubien, H2S 2J5</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1064</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1821,7 +1813,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Sherbrooke</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -1831,7 +1823,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
@@ -1841,7 +1833,7 @@
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/plateau-superbe-5-1-2-de-3-chambres-disponible-le-1er-juillet/1740256791</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-annexe-renove-pres-du-metro-beaubien/1735720589</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -1851,19 +1843,19 @@
       </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées, 2e étage, laveuse-sécheuse dans l'unité, climatisation, balcon arrière, boul. Saint-Laurent et ses commerces à 1 rue, secteur sud du Plateau (limite Milton-Parc), métro Sherbrooke ou Saint-Laurent à pied, dispo 1er juillet 2026, animaux limités, prix à la limite haute du budget</t>
+          <t>3 ch fermées + annexe (ancien solarium), rénové récemment, 2 grands balcons, entrées laveuse-sécheuse et lave-vaisselle, climatisation, dispo 1er sept 2026, rue Beaubien et commerces à pied, non-fumeur, pas d'animaux</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8d/8d95567f-3a46-42b2-bcd6-c8ea29c0a1ff?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ca/ca9a1937-a625-413b-ba4b-233b3a0e900b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1873,7 +1865,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Appartement 2 chambres fermées, 974 pi², balcon – Plateau (Gilford/Chambord)</t>
+          <t>Magnifique 5 1/2 sur le plateau mont-royal</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1883,22 +1875,22 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2J 3L2, coin Gilford/Chambord)</t>
+          <t>rue Marie-Anne, H2H 1M9</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>974</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -1908,7 +1900,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal ou Laurier</t>
+          <t>Mont-Royal</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -1918,7 +1910,7 @@
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="M17" s="5" t="inlineStr">
@@ -1928,22 +1920,22 @@
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-2-chambre-plateau-mont-royal/1739725006</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/magnifique-5-1-2-sur-le-plateau-mont-royal/1734803750</t>
         </is>
       </c>
       <c r="O17" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>Rez-de-jardin lumineux, sdb rénovée 2021, cuisine rénovée 2019, tous électros inclus + laveuse-sécheuse, à 2 min de l'avenue Mont-Royal, près parcs Lafontaine et Laurier, animaux limités, dispo 1er juillet ou août 2026</t>
+          <t>3 ch fermées, cuisine rénovée comptoirs quartz, planchers bois franc d'origine, laveuse-sécheuse dans l'unité, balcon privé, animaux acceptés, bail au mois, avenue Mont-Royal et ses commerces à pied, chauffage/électricité en sus</t>
         </is>
       </c>
       <c r="Q17" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/83/83da6eb9-3422-4702-b436-ed820032998c?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/38/389e0d3d-7bcf-42a9-8fe4-8a27fa531359?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1960,77 +1952,77 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 lumineux, 2 chambres fermées, 2 balcons – Rosemont, près Cinéma Beaubien</t>
+          <t>Unité neuve 3 chambres 1120 pi2 projet boutique</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2G 2S1)</t>
+          <t>2017, avenue Letourneux, app. 101, Montréal</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>946</t>
+          <t>1120</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Pie-IX</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-lumineux-2-ch-fermees-renove-rosemont-petite-patrie/1739560132</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/27359064</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>Animaux limités, 3e étage, buanderie et lave-vaisselle inclus, à deux pas du Cinéma Beaubien, libre 1er juillet 2026</t>
+          <t>Construction neuve 2026, 6 pièces, 3 chambres en demi-sous-sol, terrasse commune sur le toit, semi-meublé, internet inclus, 1 mois gratuit bail 24 mois, dispo 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q18" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c1/c15d7c88-4278-46b2-b504-86cd39d6404b?rule=kijijica-960-jpg</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15A15CDDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -2047,22 +2039,22 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Appartement lumineux sur la plaza</t>
+          <t>Plateau - Superbe 5 1/2 de 3 Chambres - Disponible le 1er Juillet</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>rue Saint-Hubert, H2S 2L9</t>
+          <t>3477 rue Saint-Dominique, H2X 2X5</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -2072,7 +2064,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -2082,7 +2074,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Sherbrooke</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -2092,7 +2084,7 @@
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
@@ -2102,29 +2094,29 @@
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-lumineux-sur-la-plaza/1739853332</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/plateau-superbe-5-1-2-de-3-chambres-disponible-le-1er-juillet/1740256791</t>
         </is>
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>2 ch fermées + boudoir avec grand placard, Plaza St-Hubert au pied de l'immeuble (quartier très vivant), laveuse-sécheuse dans l'unité, clim, 1 stationnement, grand balcon, métro Beaubien à 2 min selon l'annonce, dispo 15 juillet 2026, animaux limités</t>
+          <t>3 ch fermées, 2e étage, laveuse-sécheuse dans l'unité, climatisation, balcon arrière, boul. Saint-Laurent et ses commerces à 1 rue, secteur sud du Plateau (limite Milton-Parc), métro Sherbrooke ou Saint-Laurent à pied, dispo 1er juillet 2026, animaux limités, prix à la limite haute du budget</t>
         </is>
       </c>
       <c r="Q19" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/29/29f42067-d07c-42c9-9127-b218f6f690f8?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8d/8d95567f-3a46-42b2-bcd6-c8ea29c0a1ff?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -2134,27 +2126,27 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Condo 4½ rénové avec stationnement</t>
+          <t>Appartement 2 chambres fermées, 974 pi², balcon – Plateau (Gilford/Chambord)</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Rosemont/La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>6855, rue d'Iberville, Montréal</t>
+          <t>n/d (Montréal, QC H2J 3L2, coin Gilford/Chambord)</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>1010</t>
+          <t>974</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -2169,27 +2161,27 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>D'Iberville</t>
+          <t>Mont-Royal ou Laurier</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/4-1-2-a-louer/hab-6855-diberville-1136946</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-2-chambre-plateau-mont-royal/1739725006</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr">
@@ -2199,12 +2191,12 @@
       </c>
       <c r="P20" s="6" t="inlineStr">
         <is>
-          <t>2 chambres fermées, cuisine et sdb modernes, climatisé, stationnement, rangement ext., animaux acceptés, dispo 16 juillet 2026</t>
+          <t>Rez-de-jardin lumineux, sdb rénovée 2021, cuisine rénovée 2019, tous électros inclus + laveuse-sécheuse, à 2 min de l'avenue Mont-Royal, près parcs Lafontaine et Laurier, animaux limités, dispo 1er juillet ou août 2026</t>
         </is>
       </c>
       <c r="Q20" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202607/1136946/4-1-2-rosemont-petite-patrie-600-15776920.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/83/83da6eb9-3422-4702-b436-ed820032998c?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2221,32 +2213,32 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>6 1/2, balcon et terrasse, animaux acceptés – Hochelaga</t>
+          <t>5 1/2 lumineux, 2 chambres fermées, 2 balcons – Rosemont, près Cinéma Beaubien</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>1841 Rue Saint-Germain, Montréal</t>
+          <t>n/d (Montréal, QC H2G 2S1)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>946</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -2256,27 +2248,27 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Préfontaine</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>https://centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/25697495</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-lumineux-2-ch-fermees-renove-rosemont-petite-patrie/1739560132</t>
         </is>
       </c>
       <c r="O21" s="5" t="inlineStr">
@@ -2286,12 +2278,12 @@
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, animaux acceptés sous conditions (chiens ok), 1 stationnement, libre 7 jours après acceptation du bail, vérification de crédit requise</t>
+          <t>Animaux limités, 3e étage, buanderie et lave-vaisselle inclus, à deux pas du Cinéma Beaubien, libre 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q21" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA16F1EEDDDDDDDDDD4&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c1/c15d7c88-4278-46b2-b504-86cd39d6404b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2308,32 +2300,32 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail – Grand 5 1/2 lumineux, balcon et terrasse – Hochelaga/Préfontaine</t>
+          <t>Appartement lumineux sur la plaza</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>La Petite-Patrie</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1V 2X2, secteur Préfontaine)</t>
+          <t>rue Saint-Hubert, H2S 2L9</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -2343,17 +2335,17 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Préfontaine</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
@@ -2363,7 +2355,7 @@
       </c>
       <c r="N22" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cession-de-bail-grand-5-1-2-lumineux-hochelaga-prefontaine/1739376269</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-lumineux-sur-la-plaza/1739853332</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -2373,12 +2365,12 @@
       </c>
       <c r="P22" s="6" t="inlineStr">
         <is>
-          <t>1er mois gratuit, animaux acceptés (même chiens), hydro et stationnement inclus, buanderie, bail jusqu'en juin 2027</t>
+          <t>2 ch fermées + boudoir avec grand placard, Plaza St-Hubert au pied de l'immeuble (quartier très vivant), laveuse-sécheuse dans l'unité, clim, 1 stationnement, grand balcon, métro Beaubien à 2 min selon l'annonce, dispo 15 juillet 2026, animaux limités</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/9b/9b7ac581-3ab1-482b-9f87-d703dcb6bcc3?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/29/29f42067-d07c-42c9-9127-b218f6f690f8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2395,27 +2387,27 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 Villeray . Christophe-Colomb.</t>
+          <t>Condo 4½ rénové avec stationnement</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Rosemont/La Petite-Patrie</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Jarry/Christophe-Colomb, Montréal, QC H2P 0C3</t>
+          <t>6855, rue d'Iberville, Montréal</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>2305</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>1054</t>
+          <t>1010</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2430,27 +2422,27 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>D'Iberville</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
+          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/4-1-2-a-louer/hab-6855-diberville-1136946</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">
@@ -2460,19 +2452,19 @@
       </c>
       <c r="P23" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er sept 2026, internet et clim inclus, tous électros inclus (four frigo lave-vaisselle laveuse-sécheuse), animaux acceptés, immeuble béton insonorisé avec gym/ascenseur/concierge, grand balcon-terrasse privé</t>
+          <t>2 chambres fermées, cuisine et sdb modernes, climatisé, stationnement, rangement ext., animaux acceptés, dispo 16 juillet 2026</t>
         </is>
       </c>
       <c r="Q23" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202607/1136946/4-1-2-rosemont-petite-patrie-600-15776920.jpg</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2482,22 +2474,22 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 sur 2 étages, condo neuf « Joseph », balcon, près métro Joliette</t>
+          <t>6 1/2, balcon et terrasse, animaux acceptés – Hochelaga</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>3420 boul. Saint-Joseph Est, Montréal, QC H1X 0A6</t>
+          <t>1841 Rue Saint-Germain, Montréal</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -2507,7 +2499,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2517,7 +2509,7 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Préfontaine</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -2527,32 +2519,32 @@
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N24" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-sur-2-etages-condo-appartement-a-louer-rosemont-joseph/1727979165</t>
+          <t>https://centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/25697495</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>Condo neuf « Joseph » sur 2 étages, face au parc Lafond, eau chaude et climatisation incluses, électros neufs (laveuse-sécheuse inclus), piscine extérieure/gym/stationnement intérieur payant, animaux acceptés, superficie non précisée, près Stade olympique et Jardin botanique</t>
+          <t>Semi-meublé, animaux acceptés sous conditions (chiens ok), 1 stationnement, libre 7 jours après acceptation du bail, vérification de crédit requise</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/2a/2a378c4c-30df-42fd-8c0d-515e4ee71bc4?rule=kijijica-960-jpg</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA16F1EEDDDDDDDDDD4&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2561,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 RDC rénové avec cour – Hochelaga, près Pie-IX</t>
+          <t>Cession de bail – Grand 5 1/2 lumineux, balcon et terrasse – Hochelaga/Préfontaine</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -2579,32 +2571,32 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>1711 Avenue d'Orléans, Montréal, QC H1W 3R4</t>
+          <t>n/d (Montréal, QC H1V 2X2, secteur Préfontaine)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Pie-IX</t>
+          <t>Préfontaine</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
@@ -2614,7 +2606,7 @@
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
@@ -2624,22 +2616,22 @@
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/hochelaga-superbe-5-1-2-renove-au-rez-de-chaussee-avec-cour/1740256793</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cession-de-bail-grand-5-1-2-lumineux-hochelaga-prefontaine/1739376269</t>
         </is>
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>Animaux limités, stationnement inclus, cour arrière privée, climatisation, libre 1er juillet 2026</t>
+          <t>1er mois gratuit, animaux acceptés (même chiens), hydro et stationnement inclus, buanderie, bail jusqu'en juin 2027</t>
         </is>
       </c>
       <c r="Q25" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/d0/d0d75179-15a9-4d6e-a66c-024195759d32?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/9b/9b7ac581-3ab1-482b-9f87-d703dcb6bcc3?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2656,27 +2648,27 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 avec garage, grande cour – Hochelaga (Place Valois)</t>
+          <t>4 1/2 Villeray . Christophe-Colomb.</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1W 3N6, angle Bourbonnière/Ontario)</t>
+          <t>Jarry/Christophe-Colomb, Montréal, QC H2P 0C3</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2305</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>1054</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -2686,22 +2678,22 @@
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>n/d (grande cour arrière privée)</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>9 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
@@ -2711,29 +2703,29 @@
       </c>
       <c r="N26" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-avec-garage-a-louer-dans-hochelaga-mainsonneuve/1739944242</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P26" s="6" t="inlineStr">
         <is>
-          <t>Chauffage et climatisation centrale inclus, chats seulement (pas de chiens), 2 places de stationnement + 1 garage, libre 1er août 2026, près Place Valois</t>
+          <t>Dispo 1er sept 2026, internet et clim inclus, tous électros inclus (four frigo lave-vaisselle laveuse-sécheuse), animaux acceptés, immeuble béton insonorisé avec gym/ascenseur/concierge, grand balcon-terrasse privé</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/3e/3efd086c-a651-43a1-8291-a49f0c1d38d5?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -2743,27 +2735,27 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Grand 5 1/2 lumineux, à 200m du métro Laurier – Plateau</t>
+          <t>4 1/2 sur 2 étages, condo neuf « Joseph », balcon, près métro Joliette</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2J 2Y3)</t>
+          <t>3420 boul. Saint-Joseph Est, Montréal, QC H1X 0A6</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -2773,22 +2765,22 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>oui (petit balcon cuisine)</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Laurier</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -2798,7 +2790,7 @@
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-51-2-lumineux-sur-plateau-mont-royal/1738318103</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-sur-2-etages-condo-appartement-a-louer-rosemont-joseph/1727979165</t>
         </is>
       </c>
       <c r="O27" s="5" t="inlineStr">
@@ -2808,12 +2800,12 @@
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>Chauffage inclus, animaux limités, walk-in dans chambre principale, libre 1er juillet 2026</t>
+          <t>Condo neuf « Joseph » sur 2 étages, face au parc Lafond, eau chaude et climatisation incluses, électros neufs (laveuse-sécheuse inclus), piscine extérieure/gym/stationnement intérieur payant, animaux acceptés, superficie non précisée, près Stade olympique et Jardin botanique</t>
         </is>
       </c>
       <c r="Q27" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/d0/d0ca9a85-dbf8-4673-a89d-264708952626?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/2a/2a378c4c-30df-42fd-8c0d-515e4ee71bc4?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2830,62 +2822,62 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Grand 5½ meublé et entièrement rénové</t>
+          <t>5 1/2 RDC rénové avec cour – Hochelaga, près Pie-IX</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>13e Avenue, Montréal (près métro Saint-Michel)</t>
+          <t>1711 Avenue d'Orléans, Montréal, QC H1W 3R4</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>2265</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>Saint-Michel</t>
+          <t>Pie-IX</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353226</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/hochelaga-superbe-5-1-2-renove-au-rez-de-chaussee-avec-cour/1740256793</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -2895,10 +2887,14 @@
       </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>5½ 3 chambres, meublé, laveuse-sécheuse, comptoirs quartz, balcon + terrasse, métro Saint-Michel à 394 m, cession de bail jusqu'au 30 juin 2027, pas d'animaux, limite est de Villeray</t>
-        </is>
-      </c>
-      <c r="Q28" s="5" t="inlineStr"/>
+          <t>Animaux limités, stationnement inclus, cour arrière privée, climatisation, libre 1er juillet 2026</t>
+        </is>
+      </c>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/d0/d0d75179-15a9-4d6e-a66c-024195759d32?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2913,62 +2909,62 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>5½ 2e étage Jarry Est rénové</t>
+          <t>5 1/2 avec garage, grande cour – Hochelaga (Place Valois)</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>582 rue Jarry Est, Montréal</t>
+          <t>n/d (Montréal, QC H1W 3N6, angle Bourbonnière/Ontario)</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>950</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>n/d (grande cour arrière privée)</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9 (estimé)</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353442</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-avec-garage-a-louer-dans-hochelaga-mainsonneuve/1739944242</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
@@ -2978,10 +2974,14 @@
       </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>5½ 3 chambres fermées, rénové, climatisation murale, balcons avant et arrière, métro Jarry à 103 m, disponible immédiatement, enquête de crédit exigée</t>
-        </is>
-      </c>
-      <c r="Q29" s="5" t="inlineStr"/>
+          <t>Chauffage et climatisation centrale inclus, chats seulement (pas de chiens), 2 places de stationnement + 1 garage, libre 1er août 2026, près Place Valois</t>
+        </is>
+      </c>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/3e/3efd086c-a651-43a1-8291-a49f0c1d38d5?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 rénové, stationnement, patio – Plateau</t>
+          <t>Grand 5 1/2 lumineux, à 200m du métro Laurier – Plateau</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -3006,12 +3006,12 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>2181A Rue Marie-Anne, Montréal, QC H2H 1M9</t>
+          <t>n/d (Montréal, QC H2J 2Y3)</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -3026,22 +3026,22 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>oui (patio arrière)</t>
+          <t>oui (petit balcon cuisine)</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
@@ -3051,22 +3051,22 @@
       </c>
       <c r="N30" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-avec-stationnement-2-chambres-renove/1739130207</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-51-2-lumineux-sur-plateau-mont-royal/1738318103</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>Non chauffé, animaux limités, stationnement privé inclus, planchers bois franc, libre 15 juillet 2026</t>
+          <t>Chauffage inclus, animaux limités, walk-in dans chambre principale, libre 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2e8a22d5-2d29-437c-bd2c-a9be0878ff77?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/d0/d0ca9a85-dbf8-4673-a89d-264708952626?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 Villeray - 2 chambres - près du métro Jarry - 2050$</t>
+          <t>Grand 5½ meublé et entièrement rénové</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -3093,37 +3093,37 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H2R</t>
+          <t>13e Avenue, Montréal (près métro Saint-Michel)</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2265</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Saint-Michel</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
@@ -3133,29 +3133,25 @@
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-villeray-2-chambres-pres-du-metro-jarry-2050/1738384606</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353226</t>
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P31" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er juin 2026, rénové, 2 chambres + bureau, thermopompe (chauffage/clim), 5 électros inclus, cour-patio arrière, planchers bois franc refaits, pas d'animaux</t>
-        </is>
-      </c>
-      <c r="Q31" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cf44ffec-5a1f-4ffd-81e0-2eb0cfc316d8?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>5½ 3 chambres, meublé, laveuse-sécheuse, comptoirs quartz, balcon + terrasse, métro Saint-Michel à 394 m, cession de bail jusqu'au 30 juin 2027, pas d'animaux, limite est de Villeray</t>
+        </is>
+      </c>
+      <c r="Q31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -3170,27 +3166,27 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 rénové, 995 pi², près Promenade Masson – Rosemont</t>
+          <t>5½ 2e étage Jarry Est rénové</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>5472 1ere Avenue, Montréal</t>
+          <t>582 rue Jarry Est, Montréal</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -3200,54 +3196,50 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N32" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/5-1-2-a-louer/hab-5472-1ere-avenue-882773</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353442</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>Chauffage au plancher radiant, climatisation, cour privée avec remise, près Promenade Masson et parc Pélican, non-fumeurs</t>
-        </is>
-      </c>
-      <c r="Q32" s="5" t="inlineStr">
-        <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/201911/882773/5-1-2-plateau-mont-royal-1600-10690669.jpg</t>
-        </is>
-      </c>
+          <t>5½ 3 chambres fermées, rénové, climatisation murale, balcons avant et arrière, métro Jarry à 103 m, disponible immédiatement, enquête de crédit exigée</t>
+        </is>
+      </c>
+      <c r="Q32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -3257,7 +3249,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
+          <t>5 1/2 rénové, stationnement, patio – Plateau</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -3267,67 +3259,67 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
+          <t>2181A Rue Marie-Anne, Montréal, QC H2H 1M9</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>oui (patio arrière)</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
+      <c r="K33" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>Mont-Royal ou Papineau (à vérifier)</t>
-        </is>
-      </c>
-      <c r="K33" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>12 (estimé)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-avec-stationnement-2-chambres-renove/1739130207</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P33" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
+          <t>Non chauffé, animaux limités, stationnement privé inclus, planchers bois franc, libre 15 juillet 2026</t>
         </is>
       </c>
       <c r="Q33" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2e8a22d5-2d29-437c-bd2c-a9be0878ff77?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3344,42 +3336,42 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
+          <t>5 1/2 Villeray - 2 chambres - près du métro Jarry - 2050$</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>62 rue Rachel Est, Montréal</t>
+          <t>Montréal, QC H2R</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -3389,32 +3381,32 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-villeray-2-chambres-pres-du-metro-jarry-2050/1738384606</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
+          <t>Dispo 1er juin 2026, rénové, 2 chambres + bureau, thermopompe (chauffage/clim), 5 électros inclus, cour-patio arrière, planchers bois franc refaits, pas d'animaux</t>
         </is>
       </c>
       <c r="Q34" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cf44ffec-5a1f-4ffd-81e0-2eb0cfc316d8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3431,52 +3423,52 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
+          <t>5 1/2 rénové, 995 pi², près Promenade Masson – Rosemont</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>4275 Rue de Bordeaux, Montréal</t>
+          <t>5472 1ere Avenue, Montréal</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>2095</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
+          <t>995</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
+      <c r="J35" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J35" s="5" t="inlineStr">
-        <is>
-          <t>Mont-Royal</t>
-        </is>
-      </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
@@ -3486,114 +3478,375 @@
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
+          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/5-1-2-a-louer/hab-5472-1ere-avenue-882773</t>
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P35" s="6" t="inlineStr">
         <is>
-          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
+          <t>Chauffage au plancher radiant, climatisation, cour privée avec remise, près Promenade Masson et parc Pélican, non-fumeurs</t>
         </is>
       </c>
       <c r="Q35" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/201911/882773/5-1-2-plateau-mont-royal-1600-10690669.jpg</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>2150</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>Mont-Royal ou Papineau (à vérifier)</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>12 (estimé)</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N36" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P36" s="6" t="inlineStr">
+        <is>
+          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
+        </is>
+      </c>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>62 rue Rachel Est, Montréal</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>2195</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>8 (estimé)</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
+        </is>
+      </c>
+      <c r="O37" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P37" s="6" t="inlineStr">
+        <is>
+          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>4275 Rue de Bordeaux, Montréal</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>2095</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>Mont-Royal</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>10 (estimé)</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N38" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P38" s="6" t="inlineStr">
+        <is>
+          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
+        </is>
+      </c>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>1889 Rue des Carrières, Montréal</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>2375</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I36" s="5" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J36" s="5" t="inlineStr">
+      <c r="J39" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="K36" s="5" t="inlineStr">
+      <c r="K39" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="L36" s="5" t="inlineStr">
+      <c r="L39" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="M36" s="5" t="inlineStr">
+      <c r="M39" s="5" t="inlineStr">
         <is>
           <t>Centris</t>
         </is>
       </c>
-      <c r="N36" s="7" t="inlineStr">
+      <c r="N39" s="7" t="inlineStr">
         <is>
           <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
         </is>
       </c>
-      <c r="O36" s="5" t="inlineStr">
+      <c r="O39" s="5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="P36" s="6" t="inlineStr">
+      <c r="P39" s="6" t="inlineStr">
         <is>
           <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
         </is>
       </c>
-      <c r="Q36" s="5" t="inlineStr">
+      <c r="Q39" s="5" t="inlineStr">
         <is>
           <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE603764DDDDDDDDDDD&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q36"/>
+  <autoFilter ref="A1:Q39"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -3630,6 +3883,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour des annonces — 2026-07-14 17:04
</commit_message>
<xml_diff>
--- a/annonces.xlsx
+++ b/annonces.xlsx
@@ -36,7 +36,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -46,11 +46,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E5F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,19 +61,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -566,42 +552,42 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>NOUVEAU</t>
+          <t>vu</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Grand 4 1/2 avec balcon, wifi et électros neufs inclus – Hochelaga</t>
+          <t>Condo 3 chambres, 1100 pi², 2 balcons – Centre-Sud, près métro Frontenac</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Centre-Sud</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Montréal, QC H1W 3N5</t>
+          <t>2553 Avenue Gascon, Montréal, QC H2K 2W5</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>2090</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -611,7 +597,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Joliette ou Pie-IX</t>
+          <t>Frontenac</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -621,7 +607,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>quelques min (estimé)</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -631,64 +617,64 @@
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-4-1-2-avec-balcon-wifi-electros-inclus/1740319117</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-1100pc-3ch-pres-metro-et-plateau/1740479448</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>2 chambres fermées + den, grand balcon arrière vue jardin, wifi et électroménagers neufs inclus (laveuse-sécheuse, lave-vaisselle, thermopompe/climatisation), salle de bain rénovée 2025, non-fumeur, pas d'animaux, dispo 1er août 2026 (possibilité plus tôt), bail 1 an</t>
+          <t>3 chambres fermées + bureau, 2 balcons, planchers bois franc, grande fenestration, animaux acceptés, dispo 1er août 2026, bail 1 an, secteur vivant à la frontière Plateau/Hochelaga (rue Ontario), aucun stationnement inclus</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/20/2040a77c-67f8-4d3c-8b23-22071ed8ca1b?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/6c/6c93d656-ed7d-413a-ac8b-986e4f7f2eda?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>NOUVEAU</t>
+          <t>vu</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Condo 5½ meublé, balcon vue sur parc – Angus/Rosemont, près métro Joliette</t>
+          <t>6 et demi avec cour arrière privative - Villeray - 1er juillet!</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>3439 Rue William-Tremblay, Montréal</t>
+          <t>8413 rue Saint-Hubert, Montréal, QC H2P 1Z6</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -698,12 +684,12 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -713,3133 +699,3133 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/condo-a-louer-rosemont_la-petite-patrie-l353563</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/6-et-demi-avec-cour-arriere-privative-villeray-1er-juillet/1734943312</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Unité de coin entièrement meublée (TV, lit, sofa, climatiseur portatif, électros inclus), vue sur parc, arrêt de bus à 1 min vers le métro, électricité et internet en sus (~70$/mois chacun), dispo 1er août ou 1er sept 2026, secteur Angus vivant (écoles, parcs, commerces à pied)</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr"/>
+          <t>Dispo 1er juillet 2026, prix promo 12 mois (régulier 2050$), RDC + sous-sol aménagé, cour arrière privée, lave-vaisselle inclus, option 4 électros +100$/mois, 1 chat ou petit chien accepté</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8a/8a62cfb1-09e6-4e8b-bc96-fe68a77e35b2?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>NOUVEAU</t>
+          <t>vu</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Condo 4½ neuf sur 2 étages, semi-meublé, balcon – Plateau/Centre-Sud, près métro Préfontaine</t>
+          <t>Beau 6 1/2 ensoleillé - proche metro - Hochelaga</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2484 Rue Marie-Anne Est, Montréal</t>
+          <t>Montréal, QC H1W 1M3</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2075</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Joliette</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Préfontaine</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/condo-a-louer-le-plateau-mont-royal-l353552</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/beau-6-1-2-ensoleille-proche-metro-hochelaga/1738000997</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Condo construit en 2019, climatisation centrale, système d'alarme, entrées laveuse-sécheuse, dispo 1er sept 2026, station Frontenac aussi accessible à 12 min</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr"/>
+          <t>Dispo 1er juin 2026, eau incluse, 4 électros inclus (frigo cuisinière laveuse sécheuse), 2e étage, plafonds hauts, animaux limités, près Promenade Ontario</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/77/77a71464-4b91-4435-bf29-e86a1a84a6a8?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Condo 3 chambres, 1100 pi², 2 balcons – Centre-Sud, près métro Frontenac</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Centre-Sud</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>2553 Avenue Gascon, Montréal, QC H2K 2W5</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>2090</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>1100</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Grand 6 1/2 Villeray, metro Jarry</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Villeray</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Montréal, QC H2R 2E8</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>1250</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Frontenac</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>8 (estimé)</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Jarry</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-1100pc-3ch-pres-metro-et-plateau/1740479448</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="P5" s="6" t="inlineStr">
-        <is>
-          <t>3 chambres fermées + bureau, 2 balcons, planchers bois franc, grande fenestration, animaux acceptés, dispo 1er août 2026, bail 1 an, secteur vivant à la frontière Plateau/Hochelaga (rue Ontario), aucun stationnement inclus</t>
-        </is>
-      </c>
-      <c r="Q5" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/6c/6c93d656-ed7d-413a-ac8b-986e4f7f2eda?rule=kijijica-960-jpg</t>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-6-1-2-villeray-metro-jarry/1740222569</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>Dispo 1er août 2026 (ou 1er juillet), 2 balcons (avant + grand arrière), 3 chambres fermées, électros non inclus mais négociable, pas d'animaux, non-fumeur, chauffage/électricité aux frais du locataire</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/41/41b6a01a-67b3-4d74-8966-ac23a1a991aa?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>4 1/2 (2 chambres), 900 pi², balcon, tout inclus – Rosemont (rue Dandurand)</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Rosemont-La Petite-Patrie</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>3320 Rue Dandurand, Montréal, QC H1X 1M6</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>1999</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Grand 4 1/2 avec balcon, wifi et électros neufs inclus – Hochelaga</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Hochelaga-Maisonneuve</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Montréal, QC H1W 3N5</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1940</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>900</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>Iberville</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>bleue</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>5 (estimé)</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Joliette ou Pie-IX</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>quelques min (estimé)</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N6" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-a-louer-2-chambres-rosemont-petite-patrie-tout-inclus/1739170766</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="inlineStr">
-        <is>
-          <t>Construit 2012, tout inclus (chauffage, hydro, eau, wifi, climatisation), semi-meublé (électros + meubles salon/cuisine, matelas non inclus), animaux limités, dispo 1er juillet 2026, à 5-10 min à pied des commerces/restos de la rue Masson</t>
-        </is>
-      </c>
-      <c r="Q6" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ba/bacee7d5-1abf-4a36-80b6-12877aa40971?rule=kijijica-960-jpg</t>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-4-1-2-avec-balcon-wifi-electros-inclus/1740319117</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>2 chambres fermées + den, grand balcon arrière vue jardin, wifi et électroménagers neufs inclus (laveuse-sécheuse, lave-vaisselle, thermopompe/climatisation), salle de bain rénovée 2025, non-fumeur, pas d'animaux, dispo 1er août 2026 (possibilité plus tôt), bail 1 an</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/20/2040a77c-67f8-4d3c-8b23-22071ed8ca1b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>6 et demi avec cour arrière privative - Villeray - 1er juillet!</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Villeray</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>8413 rue Saint-Hubert, Montréal, QC H2P 1Z6</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>1950</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Condo 5½ meublé, balcon vue sur parc – Angus/Rosemont, près métro Joliette</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Rosemont-La Petite-Patrie</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>3439 Rue William-Tremblay, Montréal</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Jarry</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Joliette</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/6-et-demi-avec-cour-arriere-privative-villeray-1er-juillet/1734943312</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="inlineStr">
-        <is>
-          <t>Dispo 1er juillet 2026, prix promo 12 mois (régulier 2050$), RDC + sous-sol aménagé, cour arrière privée, lave-vaisselle inclus, option 4 électros +100$/mois, 1 chat ou petit chien accepté</t>
-        </is>
-      </c>
-      <c r="Q7" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8a/8a62cfb1-09e6-4e8b-bc96-fe68a77e35b2?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>LogisQuébec</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.logisquebec.com/condo-a-louer-rosemont_la-petite-patrie-l353563</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>Unité de coin entièrement meublée (TV, lit, sofa, climatiseur portatif, électros inclus), vue sur parc, arrêt de bus à 1 min vers le métro, électricité et internet en sus (~70$/mois chacun), dispo 1er août ou 1er sept 2026, secteur Angus vivant (écoles, parcs, commerces à pied)</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Beau 6 1/2 ensoleillé - proche metro - Hochelaga</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Hochelaga-Maisonneuve</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Montréal, QC H1W 1M3</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>2100</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>900</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Condo 4½ neuf sur 2 étages, semi-meublé, balcon – Plateau/Centre-Sud, près métro Préfontaine</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2484 Rue Marie-Anne Est, Montréal</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2075</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>Joliette</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Préfontaine</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>verte</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/beau-6-1-2-ensoleille-proche-metro-hochelaga/1738000997</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="P8" s="6" t="inlineStr">
-        <is>
-          <t>Dispo 1er juin 2026, eau incluse, 4 électros inclus (frigo cuisinière laveuse sécheuse), 2e étage, plafonds hauts, animaux limités, près Promenade Ontario</t>
-        </is>
-      </c>
-      <c r="Q8" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/77/77a71464-4b91-4435-bf29-e86a1a84a6a8?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>LogisQuébec</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.logisquebec.com/condo-a-louer-le-plateau-mont-royal-l353552</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>Condo construit en 2019, climatisation centrale, système d'alarme, entrées laveuse-sécheuse, dispo 1er sept 2026, station Frontenac aussi accessible à 12 min</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Grand 6 1/2 Villeray, metro Jarry</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Villeray</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Montréal, QC H2R 2E8</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>1250</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>4 1/2 rénové, grand balcon, près métro Joliette/Pie-IX</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Hochelaga-Maisonneuve</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>1695 Avenue Bourbonnière, Montréal</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>1940</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Jarry</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-6-1-2-villeray-metro-jarry/1740222569</t>
-        </is>
-      </c>
-      <c r="O9" s="5" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="P9" s="6" t="inlineStr">
-        <is>
-          <t>Dispo 1er août 2026 (ou 1er juillet), 2 balcons (avant + grand arrière), 3 chambres fermées, électros non inclus mais négociable, pas d'animaux, non-fumeur, chauffage/électricité aux frais du locataire</t>
-        </is>
-      </c>
-      <c r="Q9" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/41/41b6a01a-67b3-4d74-8966-ac23a1a991aa?rule=kijijica-960-jpg</t>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Joliette/Pie-IX</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/mercier-hochelaga-maisonneuve/4-1-2-a-louer/hab-1695-avenue-bourbonniere-1135855</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>2 ch fermées (1 grande chambre double) + salle d'eau, grand balcon arrière sur jardin paisible, dispo 1er août 2026 (ou 18 juillet), à 1 min du Metro épicerie, 3 min boulangerie Arhoma, Promenade Ontario et Place Simon-Valois à pied</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135855/mercier-hochelaga-maisonneuve-600-15749477.jpg</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>4 1/2 rénové, grand balcon, près métro Joliette/Pie-IX</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Hochelaga-Maisonneuve</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>1695 Avenue Bourbonnière, Montréal</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>1940</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>900</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>5 1/2 balcon, 1200 pi² – Rosemont</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Rosemont-La Petite-Patrie</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>6885 43e Avenue, Montréal, QC H1T 2R9</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>Joliette/Pie-IX</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>DuProprio</t>
-        </is>
-      </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>https://duproprio.com/fr/location/montreal/mercier-hochelaga-maisonneuve/4-1-2-a-louer/hab-1695-avenue-bourbonniere-1135855</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Mary Two-Axe Earley (à vérifier)</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Kijiji</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-bedroom-apartment-for-rent-in-rosemont/1739297378</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P10" s="6" t="inlineStr">
-        <is>
-          <t>2 ch fermées (1 grande chambre double) + salle d'eau, grand balcon arrière sur jardin paisible, dispo 1er août 2026 (ou 18 juillet), à 1 min du Metro épicerie, 3 min boulangerie Arhoma, Promenade Ontario et Place Simon-Valois à pied</t>
-        </is>
-      </c>
-      <c r="Q10" s="5" t="inlineStr">
-        <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135855/mercier-hochelaga-maisonneuve-600-15749477.jpg</t>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Animaux permis, eau chaude incluse, électricité et internet à la charge du locataire, libre 16 juin 2026, nom de station à vérifier</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2efd08ab-2014-42f0-bde7-3afc97ccb893?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>5 1/2 balcon, 1200 pi² – Rosemont</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>5 1/2 style condo, 2 balcons – Rosemont (Promenade Masson)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>6885 43e Avenue, Montréal, QC H1T 2R9</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>1900</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>n/d (Montréal, QC H1Y 1Y3, secteur Promenade Masson)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>1925</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>Mary Two-Axe Earley (à vérifier)</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Laurier</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>n/d (bus ~20 min)</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-bedroom-apartment-for-rent-in-rosemont/1739297378</t>
-        </is>
-      </c>
-      <c r="O11" s="5" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cessation-de-bail-5-style-condo-promenade-masson-rosemont/1739478440</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P11" s="6" t="inlineStr">
-        <is>
-          <t>Animaux permis, eau chaude incluse, électricité et internet à la charge du locataire, libre 16 juin 2026, nom de station à vérifier</t>
-        </is>
-      </c>
-      <c r="Q11" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2efd08ab-2014-42f0-bde7-3afc97ccb893?rule=kijijica-960-jpg</t>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>Chiens et chats acceptés, chauffage non inclus, Walk Score 99, très proche des commerces de la Promenade Masson</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/21/219d597c-7a1f-471a-9c6c-a7768c42324c?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>5 1/2 style condo, 2 balcons – Rosemont (Promenade Masson)</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>5 1/2, 1000 pi², balcon – Rosemont/Beaubien</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>n/d (Montréal, QC H1Y 1Y3, secteur Promenade Masson)</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>1925</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>1100</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Rue de Normanville, Montréal, QC H2S 2B5</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>1980</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>Laurier</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Rosemont/Beaubien</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>n/d (bus ~20 min)</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>10 (estimé)</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N12" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cessation-de-bail-5-style-condo-promenade-masson-rosemont/1739478440</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appart-5-1-2-a-louer-3-bed-apartment-for-rent-la-petite-patrie/1740477077</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P12" s="6" t="inlineStr">
-        <is>
-          <t>Chiens et chats acceptés, chauffage non inclus, Walk Score 99, très proche des commerces de la Promenade Masson</t>
-        </is>
-      </c>
-      <c r="Q12" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/21/219d597c-7a1f-471a-9c6c-a7768c42324c?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>1 mois gratuit 1ère année (régulier 2160$), animaux non acceptés, près du parc Père-Marquette, libre 12 juillet 2026</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>5 1/2, 1000 pi², balcon – Rosemont/Beaubien</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Rosemont-La Petite-Patrie</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Rue de Normanville, Montréal, QC H2S 2B5</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>1980</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Appartement 3 chambres, jardin, parking, Hochelaga</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Hochelaga-Maisonneuve</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Montréal, QC H1W 3A8</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2135</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>Rosemont/Beaubien</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>10 (estimé)</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Joliette</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appart-5-1-2-a-louer-3-bed-apartment-for-rent-la-petite-patrie/1740477077</t>
-        </is>
-      </c>
-      <c r="O13" s="5" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-3-chambres-jardin-parking-hochelaga/1739953364</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P13" s="6" t="inlineStr">
-        <is>
-          <t>1 mois gratuit 1ère année (régulier 2160$), animaux non acceptés, près du parc Père-Marquette, libre 12 juillet 2026</t>
-        </is>
-      </c>
-      <c r="Q13" s="5" t="inlineStr"/>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>Cession de bail jusqu'au 1er juillet 2027, dispo 1er sept 2026, cour privée, stationnement, rangement au sous-sol, lave-vaisselle inclus, animaux limités, enquête de crédit</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/43/4348c9c2-4f70-41ce-a65d-9ed5490935cd?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Appartement 3 chambres, jardin, parking, Hochelaga</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>5½ meublé tout inclus à 3 min du métro Joliette</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Montréal, QC H1W 3A8</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>2135</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>3602 rue de Rouen, Montréal</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2150</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Joliette</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>verte</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-3-chambres-jardin-parking-hochelaga/1739953364</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>LogisQuébec</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.logisquebec.com/appartement-a-louer-mercier_hochelaga-maisonneuve-l353091</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P14" s="6" t="inlineStr">
-        <is>
-          <t>Cession de bail jusqu'au 1er juillet 2027, dispo 1er sept 2026, cour privée, stationnement, rangement au sous-sol, lave-vaisselle inclus, animaux limités, enquête de crédit</t>
-        </is>
-      </c>
-      <c r="Q14" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/43/4348c9c2-4f70-41ce-a65d-9ed5490935cd?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>5½ 900 pi² meublé, chauffé, wifi et tout inclus, grande terrasse arrière 100 pi², métro Joliette à 287 m, disponible 11 octobre 2026, bail min 3 mois, pas d'animaux</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>5½ meublé tout inclus à 3 min du métro Joliette</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Hochelaga-Maisonneuve</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>3602 rue de Rouen, Montréal</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>2150</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>900</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>5 1/2 + annexe rénové près du métro Beaubien</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>La Petite-Patrie</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>secteur métro Beaubien, H2S 2J5</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>1064</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Joliette</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
-      <c r="L15" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
-        <is>
-          <t>LogisQuébec</t>
-        </is>
-      </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-mercier_hochelaga-maisonneuve-l353091</t>
-        </is>
-      </c>
-      <c r="O15" s="5" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Beaubien</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Kijiji</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-annexe-renove-pres-du-metro-beaubien/1735720589</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P15" s="6" t="inlineStr">
-        <is>
-          <t>5½ 900 pi² meublé, chauffé, wifi et tout inclus, grande terrasse arrière 100 pi², métro Joliette à 287 m, disponible 11 octobre 2026, bail min 3 mois, pas d'animaux</t>
-        </is>
-      </c>
-      <c r="Q15" s="5" t="inlineStr"/>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>3 ch fermées + annexe (ancien solarium), rénové récemment, 2 grands balcons, entrées laveuse-sécheuse et lave-vaisselle, climatisation, dispo 1er sept 2026, rue Beaubien et commerces à pied, non-fumeur, pas d'animaux</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ca/ca9a1937-a625-413b-ba4b-233b3a0e900b?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>5 1/2 + annexe rénové près du métro Beaubien</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>La Petite-Patrie</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>secteur métro Beaubien, H2S 2J5</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>1064</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Magnifique 5 1/2 sur le plateau mont-royal</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>rue Marie-Anne, H2H 1M9</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>2300</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>Beaubien</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Mont-Royal</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N16" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-annexe-renove-pres-du-metro-beaubien/1735720589</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/magnifique-5-1-2-sur-le-plateau-mont-royal/1734803750</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P16" s="6" t="inlineStr">
-        <is>
-          <t>3 ch fermées + annexe (ancien solarium), rénové récemment, 2 grands balcons, entrées laveuse-sécheuse et lave-vaisselle, climatisation, dispo 1er sept 2026, rue Beaubien et commerces à pied, non-fumeur, pas d'animaux</t>
-        </is>
-      </c>
-      <c r="Q16" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ca/ca9a1937-a625-413b-ba4b-233b3a0e900b?rule=kijijica-960-jpg</t>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>3 ch fermées, cuisine rénovée comptoirs quartz, planchers bois franc d'origine, laveuse-sécheuse dans l'unité, balcon privé, animaux acceptés, bail au mois, avenue Mont-Royal et ses commerces à pied, chauffage/électricité en sus</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/38/389e0d3d-7bcf-42a9-8fe4-8a27fa531359?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Magnifique 5 1/2 sur le plateau mont-royal</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Le Plateau-Mont-Royal</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>rue Marie-Anne, H2H 1M9</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>2300</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Unité neuve 3 chambres 1120 pi2 projet boutique</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Hochelaga-Maisonneuve</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2017, avenue Letourneux, app. 101, Montréal</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2395</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>1120</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Mont-Royal</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="M17" s="5" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N17" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/magnifique-5-1-2-sur-le-plateau-mont-royal/1734803750</t>
-        </is>
-      </c>
-      <c r="O17" s="5" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Pie-IX</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Centris</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/27359064</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P17" s="6" t="inlineStr">
-        <is>
-          <t>3 ch fermées, cuisine rénovée comptoirs quartz, planchers bois franc d'origine, laveuse-sécheuse dans l'unité, balcon privé, animaux acceptés, bail au mois, avenue Mont-Royal et ses commerces à pied, chauffage/électricité en sus</t>
-        </is>
-      </c>
-      <c r="Q17" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/38/389e0d3d-7bcf-42a9-8fe4-8a27fa531359?rule=kijijica-960-jpg</t>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>Construction neuve 2026, 6 pièces, 3 chambres en demi-sous-sol, terrasse commune sur le toit, semi-meublé, internet inclus, 1 mois gratuit bail 24 mois, dispo 1er juillet 2026</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15A15CDDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Unité neuve 3 chambres 1120 pi2 projet boutique</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Hochelaga-Maisonneuve</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>2017, avenue Letourneux, app. 101, Montréal</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>2395</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>1120</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Plateau - Superbe 5 1/2 de 3 Chambres - Disponible le 1er Juillet</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>3477 rue Saint-Dominique, H2X 2X5</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>Pie-IX</t>
-        </is>
-      </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M18" s="5" t="inlineStr">
-        <is>
-          <t>Centris</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/27359064</t>
-        </is>
-      </c>
-      <c r="O18" s="5" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Sherbrooke</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Kijiji</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/plateau-superbe-5-1-2-de-3-chambres-disponible-le-1er-juillet/1740256791</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="P18" s="6" t="inlineStr">
-        <is>
-          <t>Construction neuve 2026, 6 pièces, 3 chambres en demi-sous-sol, terrasse commune sur le toit, semi-meublé, internet inclus, 1 mois gratuit bail 24 mois, dispo 1er juillet 2026</t>
-        </is>
-      </c>
-      <c r="Q18" s="5" t="inlineStr">
-        <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15A15CDDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>3 ch fermées, 2e étage, laveuse-sécheuse dans l'unité, climatisation, balcon arrière, boul. Saint-Laurent et ses commerces à 1 rue, secteur sud du Plateau (limite Milton-Parc), métro Sherbrooke ou Saint-Laurent à pied, dispo 1er juillet 2026, animaux limités, prix à la limite haute du budget</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8d/8d95567f-3a46-42b2-bcd6-c8ea29c0a1ff?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Plateau - Superbe 5 1/2 de 3 Chambres - Disponible le 1er Juillet</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Le Plateau-Mont-Royal</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>3477 rue Saint-Dominique, H2X 2X5</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>2400</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>4 1/2 (2 chambres), 900 pi², balcon, tout inclus – Rosemont (rue Dandurand)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Rosemont-La Petite-Patrie</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>3320 Rue Dandurand, Montréal, QC H1X 1M6</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Sherbrooke</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Iberville</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>bleue</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>5 (estimé)</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Kijiji</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-a-louer-2-chambres-rosemont-petite-patrie-tout-inclus/1739170766</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/plateau-superbe-5-1-2-de-3-chambres-disponible-le-1er-juillet/1740256791</t>
-        </is>
-      </c>
-      <c r="O19" s="5" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="P19" s="6" t="inlineStr">
-        <is>
-          <t>3 ch fermées, 2e étage, laveuse-sécheuse dans l'unité, climatisation, balcon arrière, boul. Saint-Laurent et ses commerces à 1 rue, secteur sud du Plateau (limite Milton-Parc), métro Sherbrooke ou Saint-Laurent à pied, dispo 1er juillet 2026, animaux limités, prix à la limite haute du budget</t>
-        </is>
-      </c>
-      <c r="Q19" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8d/8d95567f-3a46-42b2-bcd6-c8ea29c0a1ff?rule=kijijica-960-jpg</t>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>Construit 2012, tout inclus (chauffage, hydro, eau, wifi, climatisation), semi-meublé (électros + meubles salon/cuisine, matelas non inclus), animaux limités, dispo 1er juillet 2026, à 5-10 min à pied des commerces/restos de la rue Masson</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ba/bacee7d5-1abf-4a36-80b6-12877aa40971?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Appartement 2 chambres fermées, 974 pi², balcon – Plateau (Gilford/Chambord)</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>n/d (Montréal, QC H2J 3L2, coin Gilford/Chambord)</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>2195</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>974</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Mont-Royal ou Laurier</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L20" s="5" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-2-chambre-plateau-mont-royal/1739725006</t>
         </is>
       </c>
-      <c r="O20" s="5" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P20" s="6" t="inlineStr">
+      <c r="P20" s="3" t="inlineStr">
         <is>
           <t>Rez-de-jardin lumineux, sdb rénovée 2021, cuisine rénovée 2019, tous électros inclus + laveuse-sécheuse, à 2 min de l'avenue Mont-Royal, près parcs Lafontaine et Laurier, animaux limités, dispo 1er juillet ou août 2026</t>
         </is>
       </c>
-      <c r="Q20" s="5" t="inlineStr">
+      <c r="Q20" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/83/83da6eb9-3422-4702-b436-ed820032998c?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>5 1/2 lumineux, 2 chambres fermées, 2 balcons – Rosemont, près Cinéma Beaubien</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>n/d (Montréal, QC H2G 2S1)</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>1950</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>946</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Beaubien</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>8 (estimé)</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-lumineux-2-ch-fermees-renove-rosemont-petite-patrie/1739560132</t>
         </is>
       </c>
-      <c r="O21" s="5" t="inlineStr">
+      <c r="O21" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P21" s="6" t="inlineStr">
+      <c r="P21" s="3" t="inlineStr">
         <is>
           <t>Animaux limités, 3e étage, buanderie et lave-vaisselle inclus, à deux pas du Cinéma Beaubien, libre 1er juillet 2026</t>
         </is>
       </c>
-      <c r="Q21" s="5" t="inlineStr">
+      <c r="Q21" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c1/c15d7c88-4278-46b2-b504-86cd39d6404b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Appartement lumineux sur la plaza</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>rue Saint-Hubert, H2S 2L9</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>1975</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Beaubien</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L22" s="5" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M22" s="5" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N22" s="7" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-lumineux-sur-la-plaza/1739853332</t>
         </is>
       </c>
-      <c r="O22" s="5" t="inlineStr">
+      <c r="O22" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P22" s="6" t="inlineStr">
+      <c r="P22" s="3" t="inlineStr">
         <is>
           <t>2 ch fermées + boudoir avec grand placard, Plaza St-Hubert au pied de l'immeuble (quartier très vivant), laveuse-sécheuse dans l'unité, clim, 1 stationnement, grand balcon, métro Beaubien à 2 min selon l'annonce, dispo 15 juillet 2026, animaux limités</t>
         </is>
       </c>
-      <c r="Q22" s="5" t="inlineStr">
+      <c r="Q22" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/29/29f42067-d07c-42c9-9127-b218f6f690f8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Condo 4½ rénové avec stationnement</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Rosemont/La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>6855, rue d'Iberville, Montréal</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>2100</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>1010</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>D'Iberville</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>bleue</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>DuProprio</t>
         </is>
       </c>
-      <c r="N23" s="7" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/4-1-2-a-louer/hab-6855-diberville-1136946</t>
         </is>
       </c>
-      <c r="O23" s="5" t="inlineStr">
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P23" s="6" t="inlineStr">
+      <c r="P23" s="3" t="inlineStr">
         <is>
           <t>2 chambres fermées, cuisine et sdb modernes, climatisé, stationnement, rangement ext., animaux acceptés, dispo 16 juillet 2026</t>
         </is>
       </c>
-      <c r="Q23" s="5" t="inlineStr">
+      <c r="Q23" s="2" t="inlineStr">
         <is>
           <t>https://photos.duproprio.com/photos/public/for_rent/202607/1136946/4-1-2-rosemont-petite-patrie-600-15776920.jpg</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>6 1/2, balcon et terrasse, animaux acceptés – Hochelaga</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>1841 Rue Saint-Germain, Montréal</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>2195</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Préfontaine</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>verte</t>
         </is>
       </c>
-      <c r="L24" s="5" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="M24" s="5" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Centris</t>
         </is>
       </c>
-      <c r="N24" s="7" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>https://centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/25697495</t>
         </is>
       </c>
-      <c r="O24" s="5" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P24" s="6" t="inlineStr">
+      <c r="P24" s="3" t="inlineStr">
         <is>
           <t>Semi-meublé, animaux acceptés sous conditions (chiens ok), 1 stationnement, libre 7 jours après acceptation du bail, vérification de crédit requise</t>
         </is>
       </c>
-      <c r="Q24" s="5" t="inlineStr">
+      <c r="Q24" s="2" t="inlineStr">
         <is>
           <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA16F1EEDDDDDDDDDD4&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Cession de bail – Grand 5 1/2 lumineux, balcon et terrasse – Hochelaga/Préfontaine</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>n/d (Montréal, QC H1V 2X2, secteur Préfontaine)</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>2195</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J25" s="5" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Préfontaine</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>verte</t>
         </is>
       </c>
-      <c r="L25" s="5" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="M25" s="5" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N25" s="7" t="inlineStr">
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cession-de-bail-grand-5-1-2-lumineux-hochelaga-prefontaine/1739376269</t>
         </is>
       </c>
-      <c r="O25" s="5" t="inlineStr">
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P25" s="6" t="inlineStr">
+      <c r="P25" s="3" t="inlineStr">
         <is>
           <t>1er mois gratuit, animaux acceptés (même chiens), hydro et stationnement inclus, buanderie, bail jusqu'en juin 2027</t>
         </is>
       </c>
-      <c r="Q25" s="5" t="inlineStr">
+      <c r="Q25" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/9b/9b7ac581-3ab1-482b-9f87-d703dcb6bcc3?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>4 1/2 Villeray . Christophe-Colomb.</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Villeray</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Jarry/Christophe-Colomb, Montréal, QC H2P 0C3</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>2305</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>1054</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J26" s="5" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Jarry</t>
         </is>
       </c>
-      <c r="K26" s="5" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="M26" s="5" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N26" s="7" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
         </is>
       </c>
-      <c r="O26" s="5" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="P26" s="6" t="inlineStr">
+      <c r="P26" s="3" t="inlineStr">
         <is>
           <t>Dispo 1er sept 2026, internet et clim inclus, tous électros inclus (four frigo lave-vaisselle laveuse-sécheuse), animaux acceptés, immeuble béton insonorisé avec gym/ascenseur/concierge, grand balcon-terrasse privé</t>
         </is>
       </c>
-      <c r="Q26" s="5" t="inlineStr">
+      <c r="Q26" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>4 1/2 sur 2 étages, condo neuf « Joseph », balcon, près métro Joliette</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>3420 boul. Saint-Joseph Est, Montréal, QC H1X 0A6</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>2150</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J27" s="5" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Joliette</t>
         </is>
       </c>
-      <c r="K27" s="5" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>verte</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>10 (estimé)</t>
         </is>
       </c>
-      <c r="M27" s="5" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N27" s="7" t="inlineStr">
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-sur-2-etages-condo-appartement-a-louer-rosemont-joseph/1727979165</t>
         </is>
       </c>
-      <c r="O27" s="5" t="inlineStr">
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="P27" s="6" t="inlineStr">
+      <c r="P27" s="3" t="inlineStr">
         <is>
           <t>Condo neuf « Joseph » sur 2 étages, face au parc Lafond, eau chaude et climatisation incluses, électros neufs (laveuse-sécheuse inclus), piscine extérieure/gym/stationnement intérieur payant, animaux acceptés, superficie non précisée, près Stade olympique et Jardin botanique</t>
         </is>
       </c>
-      <c r="Q27" s="5" t="inlineStr">
+      <c r="Q27" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/2a/2a378c4c-30df-42fd-8c0d-515e4ee71bc4?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>5 1/2 RDC rénové avec cour – Hochelaga, près Pie-IX</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>1711 Avenue d'Orléans, Montréal, QC H1W 3R4</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>1950</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>900</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Pie-IX</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>verte</t>
         </is>
       </c>
-      <c r="L28" s="5" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>10 (estimé)</t>
         </is>
       </c>
-      <c r="M28" s="5" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N28" s="7" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/hochelaga-superbe-5-1-2-renove-au-rez-de-chaussee-avec-cour/1740256793</t>
         </is>
       </c>
-      <c r="O28" s="5" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="P28" s="6" t="inlineStr">
+      <c r="P28" s="3" t="inlineStr">
         <is>
           <t>Animaux limités, stationnement inclus, cour arrière privée, climatisation, libre 1er juillet 2026</t>
         </is>
       </c>
-      <c r="Q28" s="5" t="inlineStr">
+      <c r="Q28" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/d0/d0d75179-15a9-4d6e-a66c-024195759d32?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>5 1/2 avec garage, grande cour – Hochelaga (Place Valois)</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>n/d (Montréal, QC H1W 3N6, angle Bourbonnière/Ontario)</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>1950</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>950</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>n/d (grande cour arrière privée)</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Joliette</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>verte</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>9 (estimé)</t>
         </is>
       </c>
-      <c r="M29" s="5" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N29" s="7" t="inlineStr">
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-avec-garage-a-louer-dans-hochelaga-mainsonneuve/1739944242</t>
         </is>
       </c>
-      <c r="O29" s="5" t="inlineStr">
+      <c r="O29" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="P29" s="6" t="inlineStr">
+      <c r="P29" s="3" t="inlineStr">
         <is>
           <t>Chauffage et climatisation centrale inclus, chats seulement (pas de chiens), 2 places de stationnement + 1 garage, libre 1er août 2026, près Place Valois</t>
         </is>
       </c>
-      <c r="Q29" s="5" t="inlineStr">
+      <c r="Q29" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/3e/3efd086c-a651-43a1-8291-a49f0c1d38d5?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Grand 5 1/2 lumineux, à 200m du métro Laurier – Plateau</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>n/d (Montréal, QC H2J 2Y3)</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>1100</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>oui (petit balcon cuisine)</t>
         </is>
       </c>
-      <c r="J30" s="5" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Laurier</t>
         </is>
       </c>
-      <c r="K30" s="5" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L30" s="5" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="M30" s="5" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N30" s="7" t="inlineStr">
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-51-2-lumineux-sur-plateau-mont-royal/1738318103</t>
         </is>
       </c>
-      <c r="O30" s="5" t="inlineStr">
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="P30" s="6" t="inlineStr">
+      <c r="P30" s="3" t="inlineStr">
         <is>
           <t>Chauffage inclus, animaux limités, walk-in dans chambre principale, libre 1er juillet 2026</t>
         </is>
       </c>
-      <c r="Q30" s="5" t="inlineStr">
+      <c r="Q30" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/d0/d0ca9a85-dbf8-4673-a89d-264708952626?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Grand 5½ meublé et entièrement rénové</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Villeray</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>13e Avenue, Montréal (près métro Saint-Michel)</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>2265</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J31" s="5" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Saint-Michel</t>
         </is>
       </c>
-      <c r="K31" s="5" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>bleue</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="M31" s="5" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>LogisQuébec</t>
         </is>
       </c>
-      <c r="N31" s="7" t="inlineStr">
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353226</t>
         </is>
       </c>
-      <c r="O31" s="5" t="inlineStr">
+      <c r="O31" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="P31" s="6" t="inlineStr">
+      <c r="P31" s="3" t="inlineStr">
         <is>
           <t>5½ 3 chambres, meublé, laveuse-sécheuse, comptoirs quartz, balcon + terrasse, métro Saint-Michel à 394 m, cession de bail jusqu'au 30 juin 2027, pas d'animaux, limite est de Villeray</t>
         </is>
       </c>
-      <c r="Q31" s="5" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>5½ 2e étage Jarry Est rénové</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Villeray</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>582 rue Jarry Est, Montréal</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>2300</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J32" s="5" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>Jarry</t>
         </is>
       </c>
-      <c r="K32" s="5" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L32" s="5" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M32" s="5" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>LogisQuébec</t>
         </is>
       </c>
-      <c r="N32" s="7" t="inlineStr">
+      <c r="N32" s="4" t="inlineStr">
         <is>
           <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353442</t>
         </is>
       </c>
-      <c r="O32" s="5" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="P32" s="6" t="inlineStr">
+      <c r="P32" s="3" t="inlineStr">
         <is>
           <t>5½ 3 chambres fermées, rénové, climatisation murale, balcons avant et arrière, métro Jarry à 103 m, disponible immédiatement, enquête de crédit exigée</t>
         </is>
       </c>
-      <c r="Q32" s="5" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>5 1/2 rénové, stationnement, patio – Plateau</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>2181A Rue Marie-Anne, Montréal, QC H2H 1M9</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>1995</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>1100</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>oui (patio arrière)</t>
         </is>
       </c>
-      <c r="J33" s="5" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="K33" s="5" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="L33" s="5" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="M33" s="5" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N33" s="7" t="inlineStr">
+      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-avec-stationnement-2-chambres-renove/1739130207</t>
         </is>
       </c>
-      <c r="O33" s="5" t="inlineStr">
+      <c r="O33" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="P33" s="6" t="inlineStr">
+      <c r="P33" s="3" t="inlineStr">
         <is>
           <t>Non chauffé, animaux limités, stationnement privé inclus, planchers bois franc, libre 15 juillet 2026</t>
         </is>
       </c>
-      <c r="Q33" s="5" t="inlineStr">
+      <c r="Q33" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2e8a22d5-2d29-437c-bd2c-a9be0878ff77?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>5 1/2 Villeray - 2 chambres - près du métro Jarry - 2050$</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Villeray</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Montréal, QC H2R</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I34" s="5" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="J34" s="5" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Jarry</t>
         </is>
       </c>
-      <c r="K34" s="5" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L34" s="5" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="M34" s="5" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N34" s="7" t="inlineStr">
+      <c r="N34" s="4" t="inlineStr">
         <is>
           <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-villeray-2-chambres-pres-du-metro-jarry-2050/1738384606</t>
         </is>
       </c>
-      <c r="O34" s="5" t="inlineStr">
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="P34" s="6" t="inlineStr">
+      <c r="P34" s="3" t="inlineStr">
         <is>
           <t>Dispo 1er juin 2026, rénové, 2 chambres + bureau, thermopompe (chauffage/clim), 5 électros inclus, cour-patio arrière, planchers bois franc refaits, pas d'animaux</t>
         </is>
       </c>
-      <c r="Q34" s="5" t="inlineStr">
+      <c r="Q34" s="2" t="inlineStr">
         <is>
           <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cf44ffec-5a1f-4ffd-81e0-2eb0cfc316d8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>5 1/2 rénové, 995 pi², près Promenade Masson – Rosemont</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>5472 1ere Avenue, Montréal</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>2200</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>995</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J35" s="5" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="K35" s="5" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="L35" s="5" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="M35" s="5" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>DuProprio</t>
         </is>
       </c>
-      <c r="N35" s="7" t="inlineStr">
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/5-1-2-a-louer/hab-5472-1ere-avenue-882773</t>
         </is>
       </c>
-      <c r="O35" s="5" t="inlineStr">
+      <c r="O35" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="P35" s="6" t="inlineStr">
+      <c r="P35" s="3" t="inlineStr">
         <is>
           <t>Chauffage au plancher radiant, climatisation, cour privée avec remise, près Promenade Masson et parc Pélican, non-fumeurs</t>
         </is>
       </c>
-      <c r="Q35" s="5" t="inlineStr">
+      <c r="Q35" s="2" t="inlineStr">
         <is>
           <t>https://photos.duproprio.com/photos/public/for_rent/201911/882773/5-1-2-plateau-mont-royal-1600-10690669.jpg</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>4216 avenue de Lorimier, app. 204, Montréal</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>2150</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I36" s="5" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J36" s="5" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Mont-Royal ou Papineau (à vérifier)</t>
         </is>
       </c>
-      <c r="K36" s="5" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L36" s="5" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>12 (estimé)</t>
         </is>
       </c>
-      <c r="M36" s="5" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>DuProprio</t>
         </is>
       </c>
-      <c r="N36" s="7" t="inlineStr">
+      <c r="N36" s="4" t="inlineStr">
         <is>
           <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
         </is>
       </c>
-      <c r="O36" s="5" t="inlineStr">
+      <c r="O36" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="P36" s="6" t="inlineStr">
+      <c r="P36" s="3" t="inlineStr">
         <is>
           <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
         </is>
       </c>
-      <c r="Q36" s="5" t="inlineStr">
+      <c r="Q36" s="2" t="inlineStr">
         <is>
           <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>62 rue Rachel Est, Montréal</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>2195</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I37" s="5" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J37" s="5" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
         </is>
       </c>
-      <c r="K37" s="5" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L37" s="5" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>8 (estimé)</t>
         </is>
       </c>
-      <c r="M37" s="5" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>DuProprio</t>
         </is>
       </c>
-      <c r="N37" s="7" t="inlineStr">
+      <c r="N37" s="4" t="inlineStr">
         <is>
           <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
         </is>
       </c>
-      <c r="O37" s="5" t="inlineStr">
+      <c r="O37" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="P37" s="6" t="inlineStr">
+      <c r="P37" s="3" t="inlineStr">
         <is>
           <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
         </is>
       </c>
-      <c r="Q37" s="5" t="inlineStr">
+      <c r="Q37" s="2" t="inlineStr">
         <is>
           <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>4275 Rue de Bordeaux, Montréal</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>2095</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I38" s="5" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J38" s="5" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Mont-Royal</t>
         </is>
       </c>
-      <c r="K38" s="5" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L38" s="5" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>10 (estimé)</t>
         </is>
       </c>
-      <c r="M38" s="5" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>DuProprio</t>
         </is>
       </c>
-      <c r="N38" s="7" t="inlineStr">
+      <c r="N38" s="4" t="inlineStr">
         <is>
           <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
         </is>
       </c>
-      <c r="O38" s="5" t="inlineStr">
+      <c r="O38" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="P38" s="6" t="inlineStr">
+      <c r="P38" s="3" t="inlineStr">
         <is>
           <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
         </is>
       </c>
-      <c r="Q38" s="5" t="inlineStr">
+      <c r="Q38" s="2" t="inlineStr">
         <is>
           <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>vu</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>1889 Rue des Carrières, Montréal</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>2375</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="K39" s="5" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="L39" s="5" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="M39" s="5" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>Centris</t>
         </is>
       </c>
-      <c r="N39" s="7" t="inlineStr">
+      <c r="N39" s="4" t="inlineStr">
         <is>
           <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
         </is>
       </c>
-      <c r="O39" s="5" t="inlineStr">
+      <c r="O39" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="P39" s="6" t="inlineStr">
+      <c r="P39" s="3" t="inlineStr">
         <is>
           <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
         </is>
       </c>
-      <c r="Q39" s="5" t="inlineStr">
+      <c r="Q39" s="2" t="inlineStr">
         <is>
           <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE603764DDDDDDDDDDD&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>

</xml_diff>

<commit_message>
Nettoyage automatique des annonces expirées (check_links.py) avec garde-fou
</commit_message>
<xml_diff>
--- a/annonces.xlsx
+++ b/annonces.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Annonces" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1001,7 +1001,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -1011,27 +1011,27 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Condo 3 chambres, 1100 pi², 2 balcons – Centre-Sud, près métro Frontenac</t>
+          <t>6 et demi avec cour arrière privative - Villeray - 1er juillet!</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Centre-Sud</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>2553 Avenue Gascon, Montréal, QC H2K 2W5</t>
+          <t>8413 rue Saint-Hubert, Montréal, QC H2P 1Z6</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>2090</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1046,17 +1046,17 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Frontenac</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
@@ -1066,22 +1066,22 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-1100pc-3ch-pres-metro-et-plateau/1740479448</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/6-et-demi-avec-cour-arriere-privative-villeray-1er-juillet/1734943312</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>3 chambres fermées + bureau, 2 balcons, planchers bois franc, grande fenestration, animaux acceptés, dispo 1er août 2026, bail 1 an, secteur vivant à la frontière Plateau/Hochelaga (rue Ontario), aucun stationnement inclus</t>
+          <t>Dispo 1er juillet 2026, prix promo 12 mois (régulier 2050$), RDC + sous-sol aménagé, cour arrière privée, lave-vaisselle inclus, option 4 électros +100$/mois, 1 chat ou petit chien accepté</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/6c/6c93d656-ed7d-413a-ac8b-986e4f7f2eda?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8a/8a62cfb1-09e6-4e8b-bc96-fe68a77e35b2?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1098,32 +1098,32 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>6 et demi avec cour arrière privative - Villeray - 1er juillet!</t>
+          <t>Beau 6 1/2 ensoleillé - proche metro - Hochelaga</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>8413 rue Saint-Hubert, Montréal, QC H2P 1Z6</t>
+          <t>Montréal, QC H1W 1M3</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1133,17 +1133,17 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/6-et-demi-avec-cour-arriere-privative-villeray-1er-juillet/1734943312</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/beau-6-1-2-ensoleille-proche-metro-hochelaga/1738000997</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
@@ -1163,12 +1163,12 @@
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er juillet 2026, prix promo 12 mois (régulier 2050$), RDC + sous-sol aménagé, cour arrière privée, lave-vaisselle inclus, option 4 électros +100$/mois, 1 chat ou petit chien accepté</t>
+          <t>Dispo 1er juin 2026, eau incluse, 4 électros inclus (frigo cuisinière laveuse sécheuse), 2e étage, plafonds hauts, animaux limités, près Promenade Ontario</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8a/8a62cfb1-09e6-4e8b-bc96-fe68a77e35b2?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/77/77a71464-4b91-4435-bf29-e86a1a84a6a8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1185,32 +1185,32 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Beau 6 1/2 ensoleillé - proche metro - Hochelaga</t>
+          <t>Grand 6 1/2 Villeray, metro Jarry</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H1W 1M3</t>
+          <t>Montréal, QC H2R 2E8</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1250</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -1220,17 +1220,17 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/beau-6-1-2-ensoleille-proche-metro-hochelaga/1738000997</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-6-1-2-villeray-metro-jarry/1740222569</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
@@ -1250,19 +1250,19 @@
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er juin 2026, eau incluse, 4 électros inclus (frigo cuisinière laveuse sécheuse), 2e étage, plafonds hauts, animaux limités, près Promenade Ontario</t>
+          <t>Dispo 1er août 2026 (ou 1er juillet), 2 balcons (avant + grand arrière), 3 chambres fermées, électros non inclus mais négociable, pas d'animaux, non-fumeur, chauffage/électricité aux frais du locataire</t>
         </is>
       </c>
       <c r="Q9" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/77/77a71464-4b91-4435-bf29-e86a1a84a6a8?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/41/41b6a01a-67b3-4d74-8966-ac23a1a991aa?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1272,32 +1272,32 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Grand 6 1/2 Villeray, metro Jarry</t>
+          <t>Condo 5½ meublé, balcon vue sur parc – Angus/Rosemont, près métro Joliette</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H2R 2E8</t>
+          <t>3439 Rue William-Tremblay, Montréal</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>1250</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1307,44 +1307,40 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-6-1-2-villeray-metro-jarry/1740222569</t>
+          <t>https://www.logisquebec.com/condo-a-louer-rosemont_la-petite-patrie-l353563</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er août 2026 (ou 1er juillet), 2 balcons (avant + grand arrière), 3 chambres fermées, électros non inclus mais négociable, pas d'animaux, non-fumeur, chauffage/électricité aux frais du locataire</t>
-        </is>
-      </c>
-      <c r="Q10" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/41/41b6a01a-67b3-4d74-8966-ac23a1a991aa?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>Unité de coin entièrement meublée (TV, lit, sofa, climatiseur portatif, électros inclus), vue sur parc, arrêt de bus à 1 min vers le métro, électricité et internet en sus (~70$/mois chacun), dispo 1er août ou 1er sept 2026, secteur Angus vivant (écoles, parcs, commerces à pied)</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1359,27 +1355,27 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Grand 4 1/2 avec balcon, wifi et électros neufs inclus – Hochelaga</t>
+          <t>Condo 4½ neuf sur 2 étages, semi-meublé, balcon – Plateau/Centre-Sud, près métro Préfontaine</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H1W 3N5</t>
+          <t>2484 Rue Marie-Anne Est, Montréal</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>2075</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1394,7 +1390,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Joliette ou Pie-IX</t>
+          <t>Préfontaine</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -1404,17 +1400,17 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>quelques min (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-4-1-2-avec-balcon-wifi-electros-inclus/1740319117</t>
+          <t>https://www.logisquebec.com/condo-a-louer-le-plateau-mont-royal-l353552</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
@@ -1424,19 +1420,15 @@
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>2 chambres fermées + den, grand balcon arrière vue jardin, wifi et électroménagers neufs inclus (laveuse-sécheuse, lave-vaisselle, thermopompe/climatisation), salle de bain rénovée 2025, non-fumeur, pas d'animaux, dispo 1er août 2026 (possibilité plus tôt), bail 1 an</t>
-        </is>
-      </c>
-      <c r="Q11" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/20/2040a77c-67f8-4d3c-8b23-22071ed8ca1b?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>Condo construit en 2019, climatisation centrale, système d'alarme, entrées laveuse-sécheuse, dispo 1er sept 2026, station Frontenac aussi accessible à 12 min</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1446,27 +1438,27 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Condo 5½ meublé, balcon vue sur parc – Angus/Rosemont, près métro Joliette</t>
+          <t>4 1/2 rénové, grand balcon, près métro Joliette/Pie-IX</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>3439 Rue William-Tremblay, Montréal</t>
+          <t>1695 Avenue Bourbonnière, Montréal</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1481,7 +1473,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Joliette/Pie-IX</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1491,17 +1483,17 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/condo-a-louer-rosemont_la-petite-patrie-l353563</t>
+          <t>https://duproprio.com/fr/location/montreal/mercier-hochelaga-maisonneuve/4-1-2-a-louer/hab-1695-avenue-bourbonniere-1135855</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -1511,15 +1503,19 @@
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>Unité de coin entièrement meublée (TV, lit, sofa, climatiseur portatif, électros inclus), vue sur parc, arrêt de bus à 1 min vers le métro, électricité et internet en sus (~70$/mois chacun), dispo 1er août ou 1er sept 2026, secteur Angus vivant (écoles, parcs, commerces à pied)</t>
-        </is>
-      </c>
-      <c r="Q12" s="5" t="inlineStr"/>
+          <t>2 ch fermées (1 grande chambre double) + salle d'eau, grand balcon arrière sur jardin paisible, dispo 1er août 2026 (ou 18 juillet), à 1 min du Metro épicerie, 3 min boulangerie Arhoma, Promenade Ontario et Place Simon-Valois à pied</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135855/mercier-hochelaga-maisonneuve-600-15749477.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1529,32 +1525,32 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Condo 4½ neuf sur 2 étages, semi-meublé, balcon – Plateau/Centre-Sud, près métro Préfontaine</t>
+          <t>5 1/2 balcon, 1200 pi² – Rosemont</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>2484 Rue Marie-Anne Est, Montréal</t>
+          <t>6885 43e Avenue, Montréal, QC H1T 2R9</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>2075</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1564,27 +1560,27 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Préfontaine</t>
+          <t>Mary Two-Axe Earley (à vérifier)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/condo-a-louer-le-plateau-mont-royal-l353552</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-bedroom-apartment-for-rent-in-rosemont/1739297378</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -1594,10 +1590,14 @@
       </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>Condo construit en 2019, climatisation centrale, système d'alarme, entrées laveuse-sécheuse, dispo 1er sept 2026, station Frontenac aussi accessible à 12 min</t>
-        </is>
-      </c>
-      <c r="Q13" s="5" t="inlineStr"/>
+          <t>Animaux permis, eau chaude incluse, électricité et internet à la charge du locataire, libre 16 juin 2026, nom de station à vérifier</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2efd08ab-2014-42f0-bde7-3afc97ccb893?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1612,32 +1612,32 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 rénové, grand balcon, près métro Joliette/Pie-IX</t>
+          <t>5 1/2 style condo, 2 balcons – Rosemont (Promenade Masson)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>1695 Avenue Bourbonnière, Montréal</t>
+          <t>n/d (Montréal, QC H1Y 1Y3, secteur Promenade Masson)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1925</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -1647,27 +1647,27 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Joliette/Pie-IX</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>n/d (bus ~20 min)</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/mercier-hochelaga-maisonneuve/4-1-2-a-louer/hab-1695-avenue-bourbonniere-1135855</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cessation-de-bail-5-style-condo-promenade-masson-rosemont/1739478440</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -1677,12 +1677,12 @@
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>2 ch fermées (1 grande chambre double) + salle d'eau, grand balcon arrière sur jardin paisible, dispo 1er août 2026 (ou 18 juillet), à 1 min du Metro épicerie, 3 min boulangerie Arhoma, Promenade Ontario et Place Simon-Valois à pied</t>
+          <t>Chiens et chats acceptés, chauffage non inclus, Walk Score 99, très proche des commerces de la Promenade Masson</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135855/mercier-hochelaga-maisonneuve-600-15749477.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/21/219d597c-7a1f-471a-9c6c-a7768c42324c?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1699,22 +1699,22 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 balcon, 1200 pi² – Rosemont</t>
+          <t>Appartement 3 chambres, jardin, parking, Hochelaga</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>6885 43e Avenue, Montréal, QC H1T 2R9</t>
+          <t>Montréal, QC H1W 3A8</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>2135</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1729,22 +1729,22 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Mary Two-Axe Earley (à vérifier)</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-bedroom-apartment-for-rent-in-rosemont/1739297378</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-3-chambres-jardin-parking-hochelaga/1739953364</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>Animaux permis, eau chaude incluse, électricité et internet à la charge du locataire, libre 16 juin 2026, nom de station à vérifier</t>
+          <t>Cession de bail jusqu'au 1er juillet 2027, dispo 1er sept 2026, cour privée, stationnement, rangement au sous-sol, lave-vaisselle inclus, animaux limités, enquête de crédit</t>
         </is>
       </c>
       <c r="Q15" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2efd08ab-2014-42f0-bde7-3afc97ccb893?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/43/4348c9c2-4f70-41ce-a65d-9ed5490935cd?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1786,32 +1786,32 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 style condo, 2 balcons – Rosemont (Promenade Masson)</t>
+          <t>5½ meublé tout inclus à 3 min du métro Joliette</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1Y 1Y3, secteur Promenade Masson)</t>
+          <t>3602 rue de Rouen, Montréal</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>1925</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1821,27 +1821,27 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Laurier</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>n/d (bus ~20 min)</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cessation-de-bail-5-style-condo-promenade-masson-rosemont/1739478440</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-mercier_hochelaga-maisonneuve-l353091</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -1851,14 +1851,10 @@
       </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>Chiens et chats acceptés, chauffage non inclus, Walk Score 99, très proche des commerces de la Promenade Masson</t>
-        </is>
-      </c>
-      <c r="Q16" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/21/219d597c-7a1f-471a-9c6c-a7768c42324c?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>5½ 900 pi² meublé, chauffé, wifi et tout inclus, grande terrasse arrière 100 pi², métro Joliette à 287 m, disponible 11 octobre 2026, bail min 3 mois, pas d'animaux</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1873,27 +1869,27 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 1000 pi², balcon – Rosemont/Beaubien</t>
+          <t>5 1/2 + annexe rénové près du métro Beaubien</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>La Petite-Patrie</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Rue de Normanville, Montréal, QC H2S 2B5</t>
+          <t>secteur métro Beaubien, H2S 2J5</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1064</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1908,7 +1904,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Rosemont/Beaubien</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -1918,7 +1914,7 @@
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M17" s="5" t="inlineStr">
@@ -1928,7 +1924,7 @@
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appart-5-1-2-a-louer-3-bed-apartment-for-rent-la-petite-patrie/1740477077</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-annexe-renove-pres-du-metro-beaubien/1735720589</t>
         </is>
       </c>
       <c r="O17" s="5" t="inlineStr">
@@ -1938,10 +1934,14 @@
       </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>1 mois gratuit 1ère année (régulier 2160$), animaux non acceptés, près du parc Père-Marquette, libre 12 juillet 2026</t>
-        </is>
-      </c>
-      <c r="Q17" s="5" t="inlineStr"/>
+          <t>3 ch fermées + annexe (ancien solarium), rénové récemment, 2 grands balcons, entrées laveuse-sécheuse et lave-vaisselle, climatisation, dispo 1er sept 2026, rue Beaubien et commerces à pied, non-fumeur, pas d'animaux</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ca/ca9a1937-a625-413b-ba4b-233b3a0e900b?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1956,27 +1956,27 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Appartement 3 chambres, jardin, parking, Hochelaga</t>
+          <t>Magnifique 5 1/2 sur le plateau mont-royal</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H1W 3A8</t>
+          <t>rue Marie-Anne, H2H 1M9</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>2135</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -1986,22 +1986,22 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Mont-Royal</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-3-chambres-jardin-parking-hochelaga/1739953364</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/magnifique-5-1-2-sur-le-plateau-mont-royal/1734803750</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -2021,12 +2021,12 @@
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail jusqu'au 1er juillet 2027, dispo 1er sept 2026, cour privée, stationnement, rangement au sous-sol, lave-vaisselle inclus, animaux limités, enquête de crédit</t>
+          <t>3 ch fermées, cuisine rénovée comptoirs quartz, planchers bois franc d'origine, laveuse-sécheuse dans l'unité, balcon privé, animaux acceptés, bail au mois, avenue Mont-Royal et ses commerces à pied, chauffage/électricité en sus</t>
         </is>
       </c>
       <c r="Q18" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/43/4348c9c2-4f70-41ce-a65d-9ed5490935cd?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/38/389e0d3d-7bcf-42a9-8fe4-8a27fa531359?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>5½ meublé tout inclus à 3 min du métro Joliette</t>
+          <t>Unité neuve 3 chambres 1120 pi2 projet boutique</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -2053,32 +2053,32 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>3602 rue de Rouen, Montréal</t>
+          <t>2017, avenue Letourneux, app. 101, Montréal</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1120</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Pie-IX</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -2088,17 +2088,17 @@
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-mercier_hochelaga-maisonneuve-l353091</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/27359064</t>
         </is>
       </c>
       <c r="O19" s="5" t="inlineStr">
@@ -2108,10 +2108,14 @@
       </c>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>5½ 900 pi² meublé, chauffé, wifi et tout inclus, grande terrasse arrière 100 pi², métro Joliette à 287 m, disponible 11 octobre 2026, bail min 3 mois, pas d'animaux</t>
-        </is>
-      </c>
-      <c r="Q19" s="5" t="inlineStr"/>
+          <t>Construction neuve 2026, 6 pièces, 3 chambres en demi-sous-sol, terrasse commune sur le toit, semi-meublé, internet inclus, 1 mois gratuit bail 24 mois, dispo 1er juillet 2026</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15A15CDDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -2126,27 +2130,27 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 + annexe rénové près du métro Beaubien</t>
+          <t>Plateau - Superbe 5 1/2 de 3 Chambres - Disponible le 1er Juillet</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>secteur métro Beaubien, H2S 2J5</t>
+          <t>3477 rue Saint-Dominique, H2X 2X5</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>1064</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -2161,7 +2165,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Sherbrooke</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2171,7 +2175,7 @@
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
@@ -2181,7 +2185,7 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-annexe-renove-pres-du-metro-beaubien/1735720589</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/plateau-superbe-5-1-2-de-3-chambres-disponible-le-1er-juillet/1740256791</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr">
@@ -2191,19 +2195,19 @@
       </c>
       <c r="P20" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées + annexe (ancien solarium), rénové récemment, 2 grands balcons, entrées laveuse-sécheuse et lave-vaisselle, climatisation, dispo 1er sept 2026, rue Beaubien et commerces à pied, non-fumeur, pas d'animaux</t>
+          <t>3 ch fermées, 2e étage, laveuse-sécheuse dans l'unité, climatisation, balcon arrière, boul. Saint-Laurent et ses commerces à 1 rue, secteur sud du Plateau (limite Milton-Parc), métro Sherbrooke ou Saint-Laurent à pied, dispo 1er juillet 2026, animaux limités, prix à la limite haute du budget</t>
         </is>
       </c>
       <c r="Q20" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ca/ca9a1937-a625-413b-ba4b-233b3a0e900b?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8d/8d95567f-3a46-42b2-bcd6-c8ea29c0a1ff?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -2213,32 +2217,32 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Magnifique 5 1/2 sur le plateau mont-royal</t>
+          <t>4 1/2 (2 chambres), 900 pi², balcon, tout inclus – Rosemont (rue Dandurand)</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>rue Marie-Anne, H2H 1M9</t>
+          <t>3320 Rue Dandurand, Montréal, QC H1X 1M6</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>1999</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -2248,17 +2252,17 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Iberville</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5 (estimé)</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
@@ -2268,29 +2272,29 @@
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/magnifique-5-1-2-sur-le-plateau-mont-royal/1734803750</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-a-louer-2-chambres-rosemont-petite-patrie-tout-inclus/1739170766</t>
         </is>
       </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées, cuisine rénovée comptoirs quartz, planchers bois franc d'origine, laveuse-sécheuse dans l'unité, balcon privé, animaux acceptés, bail au mois, avenue Mont-Royal et ses commerces à pied, chauffage/électricité en sus</t>
+          <t>Construit 2012, tout inclus (chauffage, hydro, eau, wifi, climatisation), semi-meublé (électros + meubles salon/cuisine, matelas non inclus), animaux limités, dispo 1er juillet 2026, à 5-10 min à pied des commerces/restos de la rue Masson</t>
         </is>
       </c>
       <c r="Q21" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/38/389e0d3d-7bcf-42a9-8fe4-8a27fa531359?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ba/bacee7d5-1abf-4a36-80b6-12877aa40971?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -2300,77 +2304,77 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Unité neuve 3 chambres 1120 pi2 projet boutique</t>
+          <t>Appartement 2 chambres fermées, 974 pi², balcon – Plateau (Gilford/Chambord)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>2017, avenue Letourneux, app. 101, Montréal</t>
+          <t>n/d (Montréal, QC H2J 3L2, coin Gilford/Chambord)</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>1120</t>
+          <t>974</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Pie-IX</t>
+          <t>Mont-Royal ou Laurier</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N22" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/27359064</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-2-chambre-plateau-mont-royal/1739725006</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P22" s="6" t="inlineStr">
         <is>
-          <t>Construction neuve 2026, 6 pièces, 3 chambres en demi-sous-sol, terrasse commune sur le toit, semi-meublé, internet inclus, 1 mois gratuit bail 24 mois, dispo 1er juillet 2026</t>
+          <t>Rez-de-jardin lumineux, sdb rénovée 2021, cuisine rénovée 2019, tous électros inclus + laveuse-sécheuse, à 2 min de l'avenue Mont-Royal, près parcs Lafontaine et Laurier, animaux limités, dispo 1er juillet ou août 2026</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15A15CDDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/83/83da6eb9-3422-4702-b436-ed820032998c?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2387,32 +2391,32 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Plateau - Superbe 5 1/2 de 3 Chambres - Disponible le 1er Juillet</t>
+          <t>5 1/2 lumineux, 2 chambres fermées, 2 balcons – Rosemont, près Cinéma Beaubien</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>3477 rue Saint-Dominique, H2X 2X5</t>
+          <t>n/d (Montréal, QC H2G 2S1)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>946</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -2422,7 +2426,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Sherbrooke</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -2432,39 +2436,39 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
+          <t>8 (estimé)</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Kijiji</t>
+        </is>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-lumineux-2-ch-fermees-renove-rosemont-petite-patrie/1739560132</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N23" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/plateau-superbe-5-1-2-de-3-chambres-disponible-le-1er-juillet/1740256791</t>
-        </is>
-      </c>
-      <c r="O23" s="5" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
       <c r="P23" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées, 2e étage, laveuse-sécheuse dans l'unité, climatisation, balcon arrière, boul. Saint-Laurent et ses commerces à 1 rue, secteur sud du Plateau (limite Milton-Parc), métro Sherbrooke ou Saint-Laurent à pied, dispo 1er juillet 2026, animaux limités, prix à la limite haute du budget</t>
+          <t>Animaux limités, 3e étage, buanderie et lave-vaisselle inclus, à deux pas du Cinéma Beaubien, libre 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q23" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8d/8d95567f-3a46-42b2-bcd6-c8ea29c0a1ff?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c1/c15d7c88-4278-46b2-b504-86cd39d6404b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2474,27 +2478,27 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 (2 chambres), 900 pi², balcon, tout inclus – Rosemont (rue Dandurand)</t>
+          <t>Appartement lumineux sur la plaza</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>La Petite-Patrie</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>3320 Rue Dandurand, Montréal, QC H1X 1M6</t>
+          <t>rue Saint-Hubert, H2S 2L9</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -2509,17 +2513,17 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Iberville</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>5 (estimé)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
@@ -2529,7 +2533,7 @@
       </c>
       <c r="N24" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-a-louer-2-chambres-rosemont-petite-patrie-tout-inclus/1739170766</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-lumineux-sur-la-plaza/1739853332</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -2539,19 +2543,19 @@
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>Construit 2012, tout inclus (chauffage, hydro, eau, wifi, climatisation), semi-meublé (électros + meubles salon/cuisine, matelas non inclus), animaux limités, dispo 1er juillet 2026, à 5-10 min à pied des commerces/restos de la rue Masson</t>
+          <t>2 ch fermées + boudoir avec grand placard, Plaza St-Hubert au pied de l'immeuble (quartier très vivant), laveuse-sécheuse dans l'unité, clim, 1 stationnement, grand balcon, métro Beaubien à 2 min selon l'annonce, dispo 15 juillet 2026, animaux limités</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ba/bacee7d5-1abf-4a36-80b6-12877aa40971?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/29/29f42067-d07c-42c9-9127-b218f6f690f8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -2561,27 +2565,27 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Appartement 2 chambres fermées, 974 pi², balcon – Plateau (Gilford/Chambord)</t>
+          <t>Condo 4½ rénové avec stationnement</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont/La Petite-Patrie</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2J 3L2, coin Gilford/Chambord)</t>
+          <t>6855, rue d'Iberville, Montréal</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>974</t>
+          <t>1010</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -2596,27 +2600,27 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal ou Laurier</t>
+          <t>D'Iberville</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-2-chambre-plateau-mont-royal/1739725006</t>
+          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/4-1-2-a-louer/hab-6855-diberville-1136946</t>
         </is>
       </c>
       <c r="O25" s="5" t="inlineStr">
@@ -2626,12 +2630,12 @@
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>Rez-de-jardin lumineux, sdb rénovée 2021, cuisine rénovée 2019, tous électros inclus + laveuse-sécheuse, à 2 min de l'avenue Mont-Royal, près parcs Lafontaine et Laurier, animaux limités, dispo 1er juillet ou août 2026</t>
+          <t>2 chambres fermées, cuisine et sdb modernes, climatisé, stationnement, rangement ext., animaux acceptés, dispo 16 juillet 2026</t>
         </is>
       </c>
       <c r="Q25" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/83/83da6eb9-3422-4702-b436-ed820032998c?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202607/1136946/4-1-2-rosemont-petite-patrie-600-15776920.jpg</t>
         </is>
       </c>
     </row>
@@ -2648,32 +2652,32 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 lumineux, 2 chambres fermées, 2 balcons – Rosemont, près Cinéma Beaubien</t>
+          <t>6 1/2, balcon et terrasse, animaux acceptés – Hochelaga</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2G 2S1)</t>
+          <t>1841 Rue Saint-Germain, Montréal</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>946</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -2683,27 +2687,27 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Préfontaine</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-lumineux-2-ch-fermees-renove-rosemont-petite-patrie/1739560132</t>
+          <t>https://centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/25697495</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
@@ -2713,12 +2717,12 @@
       </c>
       <c r="P26" s="6" t="inlineStr">
         <is>
-          <t>Animaux limités, 3e étage, buanderie et lave-vaisselle inclus, à deux pas du Cinéma Beaubien, libre 1er juillet 2026</t>
+          <t>Semi-meublé, animaux acceptés sous conditions (chiens ok), 1 stationnement, libre 7 jours après acceptation du bail, vérification de crédit requise</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c1/c15d7c88-4278-46b2-b504-86cd39d6404b?rule=kijijica-960-jpg</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA16F1EEDDDDDDDDDD4&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -2735,32 +2739,32 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Appartement lumineux sur la plaza</t>
+          <t>Cession de bail – Grand 5 1/2 lumineux, balcon et terrasse – Hochelaga/Préfontaine</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>rue Saint-Hubert, H2S 2L9</t>
+          <t>n/d (Montréal, QC H1V 2X2, secteur Préfontaine)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -2770,17 +2774,17 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Préfontaine</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -2790,7 +2794,7 @@
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-lumineux-sur-la-plaza/1739853332</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cession-de-bail-grand-5-1-2-lumineux-hochelaga-prefontaine/1739376269</t>
         </is>
       </c>
       <c r="O27" s="5" t="inlineStr">
@@ -2800,12 +2804,12 @@
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>2 ch fermées + boudoir avec grand placard, Plaza St-Hubert au pied de l'immeuble (quartier très vivant), laveuse-sécheuse dans l'unité, clim, 1 stationnement, grand balcon, métro Beaubien à 2 min selon l'annonce, dispo 15 juillet 2026, animaux limités</t>
+          <t>1er mois gratuit, animaux acceptés (même chiens), hydro et stationnement inclus, buanderie, bail jusqu'en juin 2027</t>
         </is>
       </c>
       <c r="Q27" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/29/29f42067-d07c-42c9-9127-b218f6f690f8?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/9b/9b7ac581-3ab1-482b-9f87-d703dcb6bcc3?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2822,27 +2826,27 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Condo 4½ rénové avec stationnement</t>
+          <t>4 1/2 Villeray . Christophe-Colomb.</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Rosemont/La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>6855, rue d'Iberville, Montréal</t>
+          <t>Jarry/Christophe-Colomb, Montréal, QC H2P 0C3</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2305</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>1010</t>
+          <t>1054</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2857,27 +2861,27 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>D'Iberville</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/4-1-2-a-louer/hab-6855-diberville-1136946</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -2887,19 +2891,19 @@
       </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>2 chambres fermées, cuisine et sdb modernes, climatisé, stationnement, rangement ext., animaux acceptés, dispo 16 juillet 2026</t>
+          <t>Dispo 1er sept 2026, internet et clim inclus, tous électros inclus (four frigo lave-vaisselle laveuse-sécheuse), animaux acceptés, immeuble béton insonorisé avec gym/ascenseur/concierge, grand balcon-terrasse privé</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202607/1136946/4-1-2-rosemont-petite-patrie-600-15776920.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -2909,22 +2913,22 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>6 1/2, balcon et terrasse, animaux acceptés – Hochelaga</t>
+          <t>4 1/2 sur 2 étages, condo neuf « Joseph », balcon, près métro Joliette</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>1841 Rue Saint-Germain, Montréal</t>
+          <t>3420 boul. Saint-Joseph Est, Montréal, QC H1X 0A6</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -2934,7 +2938,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2944,7 +2948,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Préfontaine</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -2954,32 +2958,32 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>https://centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/25697495</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-sur-2-etages-condo-appartement-a-louer-rosemont-joseph/1727979165</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, animaux acceptés sous conditions (chiens ok), 1 stationnement, libre 7 jours après acceptation du bail, vérification de crédit requise</t>
+          <t>Condo neuf « Joseph » sur 2 étages, face au parc Lafond, eau chaude et climatisation incluses, électros neufs (laveuse-sécheuse inclus), piscine extérieure/gym/stationnement intérieur payant, animaux acceptés, superficie non précisée, près Stade olympique et Jardin botanique</t>
         </is>
       </c>
       <c r="Q29" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA16F1EEDDDDDDDDDD4&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/2a/2a378c4c-30df-42fd-8c0d-515e4ee71bc4?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2996,7 +3000,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail – Grand 5 1/2 lumineux, balcon et terrasse – Hochelaga/Préfontaine</t>
+          <t>5 1/2 RDC rénové avec cour – Hochelaga, près Pie-IX</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -3006,32 +3010,32 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1V 2X2, secteur Préfontaine)</t>
+          <t>1711 Avenue d'Orléans, Montréal, QC H1W 3R4</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>Préfontaine</t>
+          <t>Pie-IX</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -3041,7 +3045,7 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
@@ -3051,22 +3055,22 @@
       </c>
       <c r="N30" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cession-de-bail-grand-5-1-2-lumineux-hochelaga-prefontaine/1739376269</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/hochelaga-superbe-5-1-2-renove-au-rez-de-chaussee-avec-cour/1740256793</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>1er mois gratuit, animaux acceptés (même chiens), hydro et stationnement inclus, buanderie, bail jusqu'en juin 2027</t>
+          <t>Animaux limités, stationnement inclus, cour arrière privée, climatisation, libre 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/9b/9b7ac581-3ab1-482b-9f87-d703dcb6bcc3?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/d0/d0d75179-15a9-4d6e-a66c-024195759d32?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3083,27 +3087,27 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 Villeray . Christophe-Colomb.</t>
+          <t>5 1/2 avec garage, grande cour – Hochelaga (Place Valois)</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Jarry/Christophe-Colomb, Montréal, QC H2P 0C3</t>
+          <t>n/d (Montréal, QC H1W 3N6, angle Bourbonnière/Ontario)</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>2305</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>1054</t>
+          <t>950</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -3113,22 +3117,22 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>n/d (grande cour arrière privée)</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9 (estimé)</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
@@ -3138,29 +3142,29 @@
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-avec-garage-a-louer-dans-hochelaga-mainsonneuve/1739944242</t>
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P31" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er sept 2026, internet et clim inclus, tous électros inclus (four frigo lave-vaisselle laveuse-sécheuse), animaux acceptés, immeuble béton insonorisé avec gym/ascenseur/concierge, grand balcon-terrasse privé</t>
+          <t>Chauffage et climatisation centrale inclus, chats seulement (pas de chiens), 2 places de stationnement + 1 garage, libre 1er août 2026, près Place Valois</t>
         </is>
       </c>
       <c r="Q31" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/3e/3efd086c-a651-43a1-8291-a49f0c1d38d5?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -3170,27 +3174,27 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 sur 2 étages, condo neuf « Joseph », balcon, près métro Joliette</t>
+          <t>Grand 5 1/2 lumineux, à 200m du métro Laurier – Plateau</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>3420 boul. Saint-Joseph Est, Montréal, QC H1X 0A6</t>
+          <t>n/d (Montréal, QC H2J 2Y3)</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -3200,22 +3204,22 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>oui (petit balcon cuisine)</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
@@ -3225,7 +3229,7 @@
       </c>
       <c r="N32" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-sur-2-etages-condo-appartement-a-louer-rosemont-joseph/1727979165</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-51-2-lumineux-sur-plateau-mont-royal/1738318103</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr">
@@ -3235,12 +3239,12 @@
       </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>Condo neuf « Joseph » sur 2 étages, face au parc Lafond, eau chaude et climatisation incluses, électros neufs (laveuse-sécheuse inclus), piscine extérieure/gym/stationnement intérieur payant, animaux acceptés, superficie non précisée, près Stade olympique et Jardin botanique</t>
+          <t>Chauffage inclus, animaux limités, walk-in dans chambre principale, libre 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/2a/2a378c4c-30df-42fd-8c0d-515e4ee71bc4?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/d0/d0ca9a85-dbf8-4673-a89d-264708952626?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3257,62 +3261,62 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 RDC rénové avec cour – Hochelaga, près Pie-IX</t>
+          <t>Grand 5½ meublé et entièrement rénové</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>1711 Avenue d'Orléans, Montréal, QC H1W 3R4</t>
+          <t>13e Avenue, Montréal (près métro Saint-Michel)</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2265</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Pie-IX</t>
+          <t>Saint-Michel</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/hochelaga-superbe-5-1-2-renove-au-rez-de-chaussee-avec-cour/1740256793</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353226</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr">
@@ -3322,14 +3326,10 @@
       </c>
       <c r="P33" s="6" t="inlineStr">
         <is>
-          <t>Animaux limités, stationnement inclus, cour arrière privée, climatisation, libre 1er juillet 2026</t>
-        </is>
-      </c>
-      <c r="Q33" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/d0/d0d75179-15a9-4d6e-a66c-024195759d32?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>5½ 3 chambres, meublé, laveuse-sécheuse, comptoirs quartz, balcon + terrasse, métro Saint-Michel à 394 m, cession de bail jusqu'au 30 juin 2027, pas d'animaux, limite est de Villeray</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -3344,62 +3344,62 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 avec garage, grande cour – Hochelaga (Place Valois)</t>
+          <t>5½ 2e étage Jarry Est rénové</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1W 3N6, angle Bourbonnière/Ontario)</t>
+          <t>582 rue Jarry Est, Montréal</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Jarry</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>n/d (grande cour arrière privée)</t>
-        </is>
-      </c>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>Joliette</t>
-        </is>
-      </c>
-      <c r="K34" s="5" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
-      <c r="L34" s="5" t="inlineStr">
-        <is>
-          <t>9 (estimé)</t>
-        </is>
-      </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-avec-garage-a-louer-dans-hochelaga-mainsonneuve/1739944242</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353442</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
@@ -3409,14 +3409,10 @@
       </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>Chauffage et climatisation centrale inclus, chats seulement (pas de chiens), 2 places de stationnement + 1 garage, libre 1er août 2026, près Place Valois</t>
-        </is>
-      </c>
-      <c r="Q34" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/3e/3efd086c-a651-43a1-8291-a49f0c1d38d5?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>5½ 3 chambres fermées, rénové, climatisation murale, balcons avant et arrière, métro Jarry à 103 m, disponible immédiatement, enquête de crédit exigée</t>
+        </is>
+      </c>
+      <c r="Q34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -3431,7 +3427,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Grand 5 1/2 lumineux, à 200m du métro Laurier – Plateau</t>
+          <t>5 1/2 rénové, stationnement, patio – Plateau</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -3441,12 +3437,12 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2J 2Y3)</t>
+          <t>2181A Rue Marie-Anne, Montréal, QC H2H 1M9</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -3461,22 +3457,22 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>oui (petit balcon cuisine)</t>
+          <t>oui (patio arrière)</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>Laurier</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
@@ -3486,22 +3482,22 @@
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-51-2-lumineux-sur-plateau-mont-royal/1738318103</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-avec-stationnement-2-chambres-renove/1739130207</t>
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P35" s="6" t="inlineStr">
         <is>
-          <t>Chauffage inclus, animaux limités, walk-in dans chambre principale, libre 1er juillet 2026</t>
+          <t>Non chauffé, animaux limités, stationnement privé inclus, planchers bois franc, libre 15 juillet 2026</t>
         </is>
       </c>
       <c r="Q35" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/d0/d0ca9a85-dbf8-4673-a89d-264708952626?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2e8a22d5-2d29-437c-bd2c-a9be0878ff77?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3514,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Grand 5½ meublé et entièrement rénové</t>
+          <t>5 1/2 Villeray - 2 chambres - près du métro Jarry - 2050$</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -3528,37 +3524,37 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>13e Avenue, Montréal (près métro Saint-Michel)</t>
+          <t>Montréal, QC H2R</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>2265</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>Saint-Michel</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
@@ -3568,25 +3564,29 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N36" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353226</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-villeray-2-chambres-pres-du-metro-jarry-2050/1738384606</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P36" s="6" t="inlineStr">
         <is>
-          <t>5½ 3 chambres, meublé, laveuse-sécheuse, comptoirs quartz, balcon + terrasse, métro Saint-Michel à 394 m, cession de bail jusqu'au 30 juin 2027, pas d'animaux, limite est de Villeray</t>
-        </is>
-      </c>
-      <c r="Q36" s="5" t="inlineStr"/>
+          <t>Dispo 1er juin 2026, rénové, 2 chambres + bureau, thermopompe (chauffage/clim), 5 électros inclus, cour-patio arrière, planchers bois franc refaits, pas d'animaux</t>
+        </is>
+      </c>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cf44ffec-5a1f-4ffd-81e0-2eb0cfc316d8?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -3601,80 +3601,84 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>5½ 2e étage Jarry Est rénové</t>
+          <t>5 1/2 rénové, 995 pi², près Promenade Masson – Rosemont</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>582 rue Jarry Est, Montréal</t>
+          <t>5472 1ere Avenue, Montréal</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
+          <t>995</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353442</t>
+          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/5-1-2-a-louer/hab-5472-1ere-avenue-882773</t>
         </is>
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P37" s="6" t="inlineStr">
         <is>
-          <t>5½ 3 chambres fermées, rénové, climatisation murale, balcons avant et arrière, métro Jarry à 103 m, disponible immédiatement, enquête de crédit exigée</t>
-        </is>
-      </c>
-      <c r="Q37" s="5" t="inlineStr"/>
+          <t>Chauffage au plancher radiant, climatisation, cour privée avec remise, près Promenade Masson et parc Pélican, non-fumeurs</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/201911/882773/5-1-2-plateau-mont-royal-1600-10690669.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -3684,7 +3688,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 rénové, stationnement, patio – Plateau</t>
+          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -3694,67 +3698,67 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>2181A Rue Marie-Anne, Montréal, QC H2H 1M9</t>
+          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>oui (patio arrière)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Mont-Royal ou Papineau (à vérifier)</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>12 (estimé)</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-avec-stationnement-2-chambres-renove/1739130207</t>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
-          <t>Non chauffé, animaux limités, stationnement privé inclus, planchers bois franc, libre 15 juillet 2026</t>
+          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
         </is>
       </c>
       <c r="Q38" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2e8a22d5-2d29-437c-bd2c-a9be0878ff77?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
         </is>
       </c>
     </row>
@@ -3771,42 +3775,42 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 Villeray - 2 chambres - près du métro Jarry - 2050$</t>
+          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H2R</t>
+          <t>62 rue Rachel Est, Montréal</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
@@ -3816,32 +3820,32 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-villeray-2-chambres-pres-du-metro-jarry-2050/1738384606</t>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
         </is>
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P39" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er juin 2026, rénové, 2 chambres + bureau, thermopompe (chauffage/clim), 5 électros inclus, cour-patio arrière, planchers bois franc refaits, pas d'animaux</t>
+          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
         </is>
       </c>
       <c r="Q39" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cf44ffec-5a1f-4ffd-81e0-2eb0cfc316d8?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
         </is>
       </c>
     </row>
@@ -3858,27 +3862,27 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 rénové, 995 pi², près Promenade Masson – Rosemont</t>
+          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>5472 1ere Avenue, Montréal</t>
+          <t>4275 Rue de Bordeaux, Montréal</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2095</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
@@ -3893,17 +3897,17 @@
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Mont-Royal</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M40" s="5" t="inlineStr">
@@ -3913,29 +3917,29 @@
       </c>
       <c r="N40" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/5-1-2-a-louer/hab-5472-1ere-avenue-882773</t>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
         </is>
       </c>
       <c r="O40" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>Chauffage au plancher radiant, climatisation, cour privée avec remise, près Promenade Masson et parc Pélican, non-fumeurs</t>
+          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
         </is>
       </c>
       <c r="Q40" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/201911/882773/5-1-2-plateau-mont-royal-1600-10690669.jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -3945,22 +3949,22 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
+          <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
+          <t>1889 Rue des Carrières, Montréal</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2375</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -3980,308 +3984,47 @@
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal ou Papineau (à vérifier)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>12 (estimé)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
+          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
         </is>
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="P41" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
+          <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
         </is>
       </c>
       <c r="Q41" s="5" t="inlineStr">
-        <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>vu</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Le Plateau-Mont-Royal</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>62 rue Rachel Est, Montréal</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>2195</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J42" s="5" t="inlineStr">
-        <is>
-          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
-        </is>
-      </c>
-      <c r="K42" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L42" s="5" t="inlineStr">
-        <is>
-          <t>8 (estimé)</t>
-        </is>
-      </c>
-      <c r="M42" s="5" t="inlineStr">
-        <is>
-          <t>DuProprio</t>
-        </is>
-      </c>
-      <c r="N42" s="7" t="inlineStr">
-        <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
-        </is>
-      </c>
-      <c r="O42" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="P42" s="6" t="inlineStr">
-        <is>
-          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
-        </is>
-      </c>
-      <c r="Q42" s="5" t="inlineStr">
-        <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>vu</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Le Plateau-Mont-Royal</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>4275 Rue de Bordeaux, Montréal</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>2095</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I43" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J43" s="5" t="inlineStr">
-        <is>
-          <t>Mont-Royal</t>
-        </is>
-      </c>
-      <c r="K43" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L43" s="5" t="inlineStr">
-        <is>
-          <t>10 (estimé)</t>
-        </is>
-      </c>
-      <c r="M43" s="5" t="inlineStr">
-        <is>
-          <t>DuProprio</t>
-        </is>
-      </c>
-      <c r="N43" s="7" t="inlineStr">
-        <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
-        </is>
-      </c>
-      <c r="O43" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="P43" s="6" t="inlineStr">
-        <is>
-          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
-        </is>
-      </c>
-      <c r="Q43" s="5" t="inlineStr">
-        <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>vu</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Rosemont-La Petite-Patrie</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>1889 Rue des Carrières, Montréal</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>2375</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J44" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="K44" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M44" s="5" t="inlineStr">
-        <is>
-          <t>Centris</t>
-        </is>
-      </c>
-      <c r="N44" s="7" t="inlineStr">
-        <is>
-          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
-        </is>
-      </c>
-      <c r="O44" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P44" s="6" t="inlineStr">
-        <is>
-          <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
-        </is>
-      </c>
-      <c r="Q44" s="5" t="inlineStr">
         <is>
           <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE603764DDDDDDDDDDD&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q44"/>
+  <autoFilter ref="A1:Q41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -4323,9 +4066,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour des annonces — 2026-07-15 10:12
</commit_message>
<xml_diff>
--- a/annonces.xlsx
+++ b/annonces.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Annonces" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -576,54 +576,54 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>5 1/2 balcon, 3 chambres – Rosemont (14e Avenue / Masson)</t>
+          <t>Grand 6 1/2 rénové, terrasse privée – Villeray, près métro Crémazie</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1X 2W2, secteur 14e Avenue/Masson)</t>
+          <t>n/d (Montréal, QC H2P 2G9, secteur parc Jarry)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2035</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1250</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Crémazie</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Beaubien</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Kijiji</t>
@@ -631,7 +631,7 @@
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-beds-2-baths-apartment/1740599440</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/a-louer:-appartement-6-1-2-dans-villeray/1738327789</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -641,12 +641,12 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Unité au rez-de-chaussée d'un duplex/triplex, salon-solarium lumineux, cour arrière privée, garage intérieur + stationnement extérieur, climatisation, pas d'animaux, dispo 1er août 2026</t>
+          <t>Grande terrasse privée arrière + balcons avant/arrière, cuisine et salle de bain rénovées (douche romaine, puits de lumière), 4 électros + lave-vaisselle inclus, chauffage et eau chaude inclus (160$/mois fixe), piste cyclable devant, dispo 1er juillet 2026, bail 1 an</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/69/69d4ef7d-f6c5-401d-a2f8-9ca904eb6639?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c3/c339486c-6795-4d47-bcc5-625d60d299a0?rule=kpetroleumica-640-webp</t>
         </is>
       </c>
     </row>
@@ -663,32 +663,32 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>5 1/2 Rosemont rénové avec cour privée</t>
+          <t>4 1/2 avec grand balcon, électros et clim inclus – Hochelaga</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>9e Avenue, Montréal, QC H1Y 2J9</t>
+          <t>n/d (Montréal, QC H1W 3N5)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2215</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -698,17 +698,17 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Rosemont</t>
+          <t>Joliette ou Pie-IX</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-rosemont-renove-avec-cour-privee/1739626532</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-4-1-2-avec-balcon-electros-ac-inclus/1740573339</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -728,12 +728,12 @@
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Cour privée avec cabanon, climatisation incluse, animaux acceptés, non meublé, dispo 1er août 2026, bail 1 an, Vieux Rosemont, walk score 10/10</t>
+          <t>2 chambres fermées + boudoir, grand balcon arrière donnant sur jardin tranquille, électros neufs inclus (laveuse-sécheuse, lave-vaisselle, thermopompe), cuisine rénovée comptoir marbre, sdb rénovée 2025, internet haute vitesse inclus, sécurité 24h, non-fumeur, pas d'animaux, enquête de crédit, dispo 1er août 2026</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/0d/0d2593ae-6698-452f-a94e-40f11723e9a8?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/4c/4cb38191-e06a-433d-ad8f-fce80a96fe75?rule=kijijica-640-webp</t>
         </is>
       </c>
     </row>
@@ -750,52 +750,52 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Grand 5 1/2 rénové au RDC, près métro Pie-IX – Rosemont</t>
+          <t>Superbe 4 1/2, près métro Jarry – Villeray</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>4419 Avenue Charlemagne, Montréal, QC H1X 2H2</t>
+          <t>Avenue des Belges, Montréal, QC H2P 2B1</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Pie-IX</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-5-1-2-renove-a-louer-au-rdc-a-rosemont/1740506864</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/superbe-4-1-2-disponible-des-le-1er-septembre/1739673965</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -815,12 +815,12 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Climatisation incluse, fumage autorisé, pas d'animaux, aucun stationnement inclus, dispo 1er juillet 2026, proche Jardin botanique/Biodôme/Promenade Masson</t>
+          <t>Cour arrière privée, tous électros inclus (cuisinière, frigo, lave-vaisselle, laveuse-sécheuse), climatisation, stationnement dans la rue, proche épiceries/pharmacie/restos/parcs, dispo 1er sept 2026, prix à la limite haute du budget</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/1d/1d7cfe92-1f54-4f36-9a36-2e82fab03b52?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/a6/a6a41b4d-bb53-4c62-a720-a074f2806f46?rule=kijijica-640-webp</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Condo 4½ meublé avec stationnement, près métro Jarry/Crémazie – Villeray</t>
+          <t>5 1/2 lumineux, 2 balcons – Villeray (rue de Castelnau Est)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -847,154 +847,154 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>8478 Rue Saint-Dominique, Montréal</t>
+          <t>361 Rue de Castelnau Est, Montréal, QC H2R</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2290</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Jean-Talon</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>orange/bleue</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Jarry ou Crémazie</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>5 (estimé)</t>
-        </is>
-      </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/villeray-st-michel-parc-extension/4-1-2-a-louer/hab-8478-saint-dominique-1134387</t>
+          <t>https://www.facebook.com/marketplace/item/4364819800401491</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Meublé (TV 65po, mobilier complet), stationnement intérieur inclus, thermopompe, animaux négociables, bail min 12 mois, dispo 1er juillet 2026, hydro ~75$/mois + assurance 25$/mois en sus</t>
+          <t>3 chambres fermées, 2 salles de bain, 2 balcons, tous électros inclus + climatiseur, 1 animal accepté, à quelques pas de cafés/restos/commerces/parcs/épiceries, dispo 15 sept 2026, bail 1 an — lien Marketplace exige une connexion Facebook</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1134387/4-1-2-villeray-st-michel-parc-extension-600-15713346.jpg</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/738175791_122163358448956236_8893879274479902982_n.jpg?stp=c181.0.1086.1086a_dst-jpg_tt6&amp;cstp=mx1086x1086&amp;ctp=s565x565&amp;_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=rpx2E0vyW3kQ7kNvwGfclmJ&amp;_nc_oc=AdpALm3YusJq0Maav6el9qX4etr-2lUMEAPvYv1MfGvC3tr715UbWgD4CmQchGPjt44&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=EBKM-YBwAXSEbwqv2KAm-A&amp;_nc_ss=7f2a8&amp;oh=00_AQALNx8M-H3ukcmH2qnLjQMRNiPmxzCkC373khtB7tqWEQ&amp;oe=6A5D6801</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>NOUVEAU</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>4½ rénové, 1000 pi², près métro Laurier – Plateau (Parc-Lafontaine)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Le Plateau-Mont-Royal</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>4225 Rue de Lanaudière, Montréal, QC H2J 3N8</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>1900</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Laurier</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>5 1/2 balcon, 3 chambres – Rosemont (14e Avenue / Masson)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Rosemont-La Petite-Patrie</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>n/d (Montréal, QC H1X 2W2, secteur 14e Avenue/Masson)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>2250</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Beaubien</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>orange</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>10 (estimé)</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/tres-beau-4-recemment-renove-au-coeur-du-plateau-mont-royal/1739158104</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
-        <is>
-          <t>2e étage, laveuse-sécheuse-poêle-frigo inclus, non-fumeur, pas d'animaux, aucun stationnement, dispo 1er juillet 2026, près parc La Fontaine, walk score 10/10</t>
-        </is>
-      </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/15/15437f31-23a1-4bd9-9a52-5d9b817ca005?rule=kijijica-960-jpg</t>
+      <c r="N6" s="7" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-beds-2-baths-apartment/1740599440</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="inlineStr">
+        <is>
+          <t>Unité au rez-de-chaussée d'un duplex/triplex, salon-solarium lumineux, cour arrière privée, garage intérieur + stationnement extérieur, climatisation, pas d'animaux, dispo 1er août 2026</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/69/69d4ef7d-f6c5-401d-a2f8-9ca904eb6639?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Condo 5½ meublé, balcon vue sur parc – Angus/Rosemont, près métro Joliette</t>
+          <t>5 1/2 Rosemont rénové avec cour privée</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1282,12 +1282,12 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>3439 Rue William-Tremblay, Montréal</t>
+          <t>9e Avenue, Montréal, QC H1Y 2J9</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2215</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1307,27 +1307,27 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Rosemont</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/condo-a-louer-rosemont_la-petite-patrie-l353563</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-rosemont-renove-avec-cour-privee/1739626532</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1337,15 +1337,19 @@
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>Unité de coin entièrement meublée (TV, lit, sofa, climatiseur portatif, électros inclus), vue sur parc, arrêt de bus à 1 min vers le métro, électricité et internet en sus (~70$/mois chacun), dispo 1er août ou 1er sept 2026, secteur Angus vivant (écoles, parcs, commerces à pied)</t>
-        </is>
-      </c>
-      <c r="Q10" s="5" t="inlineStr"/>
+          <t>Cour privée avec cabanon, climatisation incluse, animaux acceptés, non meublé, dispo 1er août 2026, bail 1 an, Vieux Rosemont, walk score 10/10</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/0d/0d2593ae-6698-452f-a94e-40f11723e9a8?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1355,42 +1359,42 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Condo 4½ neuf sur 2 étages, semi-meublé, balcon – Plateau/Centre-Sud, près métro Préfontaine</t>
+          <t>Grand 5 1/2 rénové au RDC, près métro Pie-IX – Rosemont</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>2484 Rue Marie-Anne Est, Montréal</t>
+          <t>4419 Avenue Charlemagne, Montréal, QC H1X 2H2</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>2075</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Préfontaine</t>
+          <t>Pie-IX</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -1400,17 +1404,17 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/condo-a-louer-le-plateau-mont-royal-l353552</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-5-1-2-renove-a-louer-au-rdc-a-rosemont/1740506864</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
@@ -1420,15 +1424,19 @@
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>Condo construit en 2019, climatisation centrale, système d'alarme, entrées laveuse-sécheuse, dispo 1er sept 2026, station Frontenac aussi accessible à 12 min</t>
-        </is>
-      </c>
-      <c r="Q11" s="5" t="inlineStr"/>
+          <t>Climatisation incluse, fumage autorisé, pas d'animaux, aucun stationnement inclus, dispo 1er juillet 2026, proche Jardin botanique/Biodôme/Promenade Masson</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/1d/1d7cfe92-1f54-4f36-9a36-2e82fab03b52?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1438,27 +1446,27 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 rénové, grand balcon, près métro Joliette/Pie-IX</t>
+          <t>Condo 5½ meublé, balcon vue sur parc – Angus/Rosemont, près métro Joliette</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>1695 Avenue Bourbonnière, Montréal</t>
+          <t>3439 Rue William-Tremblay, Montréal</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1473,7 +1481,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Joliette/Pie-IX</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1483,17 +1491,17 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/mercier-hochelaga-maisonneuve/4-1-2-a-louer/hab-1695-avenue-bourbonniere-1135855</t>
+          <t>https://www.logisquebec.com/condo-a-louer-rosemont_la-petite-patrie-l353563</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -1503,19 +1511,15 @@
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>2 ch fermées (1 grande chambre double) + salle d'eau, grand balcon arrière sur jardin paisible, dispo 1er août 2026 (ou 18 juillet), à 1 min du Metro épicerie, 3 min boulangerie Arhoma, Promenade Ontario et Place Simon-Valois à pied</t>
-        </is>
-      </c>
-      <c r="Q12" s="5" t="inlineStr">
-        <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135855/mercier-hochelaga-maisonneuve-600-15749477.jpg</t>
-        </is>
-      </c>
+          <t>Unité de coin entièrement meublée (TV, lit, sofa, climatiseur portatif, électros inclus), vue sur parc, arrêt de bus à 1 min vers le métro, électricité et internet en sus (~70$/mois chacun), dispo 1er août ou 1er sept 2026, secteur Angus vivant (écoles, parcs, commerces à pied)</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1525,32 +1529,32 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 balcon, 1200 pi² – Rosemont</t>
+          <t>Condo 4½ neuf sur 2 étages, semi-meublé, balcon – Plateau/Centre-Sud, près métro Préfontaine</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>6885 43e Avenue, Montréal, QC H1T 2R9</t>
+          <t>2484 Rue Marie-Anne Est, Montréal</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>2075</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1560,27 +1564,27 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Mary Two-Axe Earley (à vérifier)</t>
+          <t>Préfontaine</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-bedroom-apartment-for-rent-in-rosemont/1739297378</t>
+          <t>https://www.logisquebec.com/condo-a-louer-le-plateau-mont-royal-l353552</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -1590,14 +1594,10 @@
       </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>Animaux permis, eau chaude incluse, électricité et internet à la charge du locataire, libre 16 juin 2026, nom de station à vérifier</t>
-        </is>
-      </c>
-      <c r="Q13" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2efd08ab-2014-42f0-bde7-3afc97ccb893?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>Condo construit en 2019, climatisation centrale, système d'alarme, entrées laveuse-sécheuse, dispo 1er sept 2026, station Frontenac aussi accessible à 12 min</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1612,32 +1612,32 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 style condo, 2 balcons – Rosemont (Promenade Masson)</t>
+          <t>4 1/2 rénové, grand balcon, près métro Joliette/Pie-IX</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1Y 1Y3, secteur Promenade Masson)</t>
+          <t>1695 Avenue Bourbonnière, Montréal</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>1925</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -1647,27 +1647,27 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Laurier</t>
+          <t>Joliette/Pie-IX</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>n/d (bus ~20 min)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cessation-de-bail-5-style-condo-promenade-masson-rosemont/1739478440</t>
+          <t>https://duproprio.com/fr/location/montreal/mercier-hochelaga-maisonneuve/4-1-2-a-louer/hab-1695-avenue-bourbonniere-1135855</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -1677,12 +1677,12 @@
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>Chiens et chats acceptés, chauffage non inclus, Walk Score 99, très proche des commerces de la Promenade Masson</t>
+          <t>2 ch fermées (1 grande chambre double) + salle d'eau, grand balcon arrière sur jardin paisible, dispo 1er août 2026 (ou 18 juillet), à 1 min du Metro épicerie, 3 min boulangerie Arhoma, Promenade Ontario et Place Simon-Valois à pied</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/21/219d597c-7a1f-471a-9c6c-a7768c42324c?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135855/mercier-hochelaga-maisonneuve-600-15749477.jpg</t>
         </is>
       </c>
     </row>
@@ -1699,22 +1699,22 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Appartement 3 chambres, jardin, parking, Hochelaga</t>
+          <t>5 1/2 balcon, 1200 pi² – Rosemont</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H1W 3A8</t>
+          <t>6885 43e Avenue, Montréal, QC H1T 2R9</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>2135</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1729,22 +1729,22 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Mary Two-Axe Earley (à vérifier)</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Joliette</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-3-chambres-jardin-parking-hochelaga/1739953364</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-bedroom-apartment-for-rent-in-rosemont/1739297378</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail jusqu'au 1er juillet 2027, dispo 1er sept 2026, cour privée, stationnement, rangement au sous-sol, lave-vaisselle inclus, animaux limités, enquête de crédit</t>
+          <t>Animaux permis, eau chaude incluse, électricité et internet à la charge du locataire, libre 16 juin 2026, nom de station à vérifier</t>
         </is>
       </c>
       <c r="Q15" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/43/4348c9c2-4f70-41ce-a65d-9ed5490935cd?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2efd08ab-2014-42f0-bde7-3afc97ccb893?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1786,32 +1786,32 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>5½ meublé tout inclus à 3 min du métro Joliette</t>
+          <t>5 1/2 style condo, 2 balcons – Rosemont (Promenade Masson)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>3602 rue de Rouen, Montréal</t>
+          <t>n/d (Montréal, QC H1Y 1Y3, secteur Promenade Masson)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>1925</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1821,27 +1821,27 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>n/d (bus ~20 min)</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-mercier_hochelaga-maisonneuve-l353091</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cessation-de-bail-5-style-condo-promenade-masson-rosemont/1739478440</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -1851,10 +1851,14 @@
       </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>5½ 900 pi² meublé, chauffé, wifi et tout inclus, grande terrasse arrière 100 pi², métro Joliette à 287 m, disponible 11 octobre 2026, bail min 3 mois, pas d'animaux</t>
-        </is>
-      </c>
-      <c r="Q16" s="5" t="inlineStr"/>
+          <t>Chiens et chats acceptés, chauffage non inclus, Walk Score 99, très proche des commerces de la Promenade Masson</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/21/219d597c-7a1f-471a-9c6c-a7768c42324c?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1869,27 +1873,27 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 + annexe rénové près du métro Beaubien</t>
+          <t>Appartement 3 chambres, jardin, parking, Hochelaga</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>secteur métro Beaubien, H2S 2J5</t>
+          <t>Montréal, QC H1W 3A8</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2135</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>1064</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1899,22 +1903,22 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M17" s="5" t="inlineStr">
@@ -1924,7 +1928,7 @@
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-annexe-renove-pres-du-metro-beaubien/1735720589</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-3-chambres-jardin-parking-hochelaga/1739953364</t>
         </is>
       </c>
       <c r="O17" s="5" t="inlineStr">
@@ -1934,12 +1938,12 @@
       </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées + annexe (ancien solarium), rénové récemment, 2 grands balcons, entrées laveuse-sécheuse et lave-vaisselle, climatisation, dispo 1er sept 2026, rue Beaubien et commerces à pied, non-fumeur, pas d'animaux</t>
+          <t>Cession de bail jusqu'au 1er juillet 2027, dispo 1er sept 2026, cour privée, stationnement, rangement au sous-sol, lave-vaisselle inclus, animaux limités, enquête de crédit</t>
         </is>
       </c>
       <c r="Q17" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ca/ca9a1937-a625-413b-ba4b-233b3a0e900b?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/43/4348c9c2-4f70-41ce-a65d-9ed5490935cd?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -1956,32 +1960,32 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Magnifique 5 1/2 sur le plateau mont-royal</t>
+          <t>5½ meublé tout inclus à 3 min du métro Joliette</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>rue Marie-Anne, H2H 1M9</t>
+          <t>3602 rue de Rouen, Montréal</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1991,27 +1995,27 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/magnifique-5-1-2-sur-le-plateau-mont-royal/1734803750</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-mercier_hochelaga-maisonneuve-l353091</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -2021,14 +2025,10 @@
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées, cuisine rénovée comptoirs quartz, planchers bois franc d'origine, laveuse-sécheuse dans l'unité, balcon privé, animaux acceptés, bail au mois, avenue Mont-Royal et ses commerces à pied, chauffage/électricité en sus</t>
-        </is>
-      </c>
-      <c r="Q18" s="5" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/38/389e0d3d-7bcf-42a9-8fe4-8a27fa531359?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
+          <t>5½ 900 pi² meublé, chauffé, wifi et tout inclus, grande terrasse arrière 100 pi², métro Joliette à 287 m, disponible 11 octobre 2026, bail min 3 mois, pas d'animaux</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2043,27 +2043,27 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Unité neuve 3 chambres 1120 pi2 projet boutique</t>
+          <t>5 1/2 + annexe rénové près du métro Beaubien</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>La Petite-Patrie</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>2017, avenue Letourneux, app. 101, Montréal</t>
+          <t>secteur métro Beaubien, H2S 2J5</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>1120</t>
+          <t>1064</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -2073,32 +2073,32 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Pie-IX</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/27359064</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-annexe-renove-pres-du-metro-beaubien/1735720589</t>
         </is>
       </c>
       <c r="O19" s="5" t="inlineStr">
@@ -2108,12 +2108,12 @@
       </c>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>Construction neuve 2026, 6 pièces, 3 chambres en demi-sous-sol, terrasse commune sur le toit, semi-meublé, internet inclus, 1 mois gratuit bail 24 mois, dispo 1er juillet 2026</t>
+          <t>3 ch fermées + annexe (ancien solarium), rénové récemment, 2 grands balcons, entrées laveuse-sécheuse et lave-vaisselle, climatisation, dispo 1er sept 2026, rue Beaubien et commerces à pied, non-fumeur, pas d'animaux</t>
         </is>
       </c>
       <c r="Q19" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15A15CDDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ca/ca9a1937-a625-413b-ba4b-233b3a0e900b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Plateau - Superbe 5 1/2 de 3 Chambres - Disponible le 1er Juillet</t>
+          <t>Magnifique 5 1/2 sur le plateau mont-royal</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -2140,12 +2140,12 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>3477 rue Saint-Dominique, H2X 2X5</t>
+          <t>rue Marie-Anne, H2H 1M9</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Sherbrooke</t>
+          <t>Mont-Royal</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/plateau-superbe-5-1-2-de-3-chambres-disponible-le-1er-juillet/1740256791</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/magnifique-5-1-2-sur-le-plateau-mont-royal/1734803750</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="P20" s="6" t="inlineStr">
         <is>
-          <t>3 ch fermées, 2e étage, laveuse-sécheuse dans l'unité, climatisation, balcon arrière, boul. Saint-Laurent et ses commerces à 1 rue, secteur sud du Plateau (limite Milton-Parc), métro Sherbrooke ou Saint-Laurent à pied, dispo 1er juillet 2026, animaux limités, prix à la limite haute du budget</t>
+          <t>3 ch fermées, cuisine rénovée comptoirs quartz, planchers bois franc d'origine, laveuse-sécheuse dans l'unité, balcon privé, animaux acceptés, bail au mois, avenue Mont-Royal et ses commerces à pied, chauffage/électricité en sus</t>
         </is>
       </c>
       <c r="Q20" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8d/8d95567f-3a46-42b2-bcd6-c8ea29c0a1ff?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/38/389e0d3d-7bcf-42a9-8fe4-8a27fa531359?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -2217,84 +2217,84 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 (2 chambres), 900 pi², balcon, tout inclus – Rosemont (rue Dandurand)</t>
+          <t>Unité neuve 3 chambres 1120 pi2 projet boutique</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>3320 Rue Dandurand, Montréal, QC H1X 1M6</t>
+          <t>2017, avenue Letourneux, app. 101, Montréal</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1120</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Iberville</t>
+          <t>Pie-IX</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>5 (estimé)</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-a-louer-2-chambres-rosemont-petite-patrie-tout-inclus/1739170766</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/27359064</t>
         </is>
       </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>Construit 2012, tout inclus (chauffage, hydro, eau, wifi, climatisation), semi-meublé (électros + meubles salon/cuisine, matelas non inclus), animaux limités, dispo 1er juillet 2026, à 5-10 min à pied des commerces/restos de la rue Masson</t>
+          <t>Construction neuve 2026, 6 pièces, 3 chambres en demi-sous-sol, terrasse commune sur le toit, semi-meublé, internet inclus, 1 mois gratuit bail 24 mois, dispo 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q21" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ba/bacee7d5-1abf-4a36-80b6-12877aa40971?rule=kijijica-960-jpg</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15A15CDDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Appartement 2 chambres fermées, 974 pi², balcon – Plateau (Gilford/Chambord)</t>
+          <t>Plateau - Superbe 5 1/2 de 3 Chambres - Disponible le 1er Juillet</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -2314,22 +2314,22 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2J 3L2, coin Gilford/Chambord)</t>
+          <t>3477 rue Saint-Dominique, H2X 2X5</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>974</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal ou Laurier</t>
+          <t>Sherbrooke</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
@@ -2359,29 +2359,29 @@
       </c>
       <c r="N22" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-2-chambre-plateau-mont-royal/1739725006</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/plateau-superbe-5-1-2-de-3-chambres-disponible-le-1er-juillet/1740256791</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P22" s="6" t="inlineStr">
         <is>
-          <t>Rez-de-jardin lumineux, sdb rénovée 2021, cuisine rénovée 2019, tous électros inclus + laveuse-sécheuse, à 2 min de l'avenue Mont-Royal, près parcs Lafontaine et Laurier, animaux limités, dispo 1er juillet ou août 2026</t>
+          <t>3 ch fermées, 2e étage, laveuse-sécheuse dans l'unité, climatisation, balcon arrière, boul. Saint-Laurent et ses commerces à 1 rue, secteur sud du Plateau (limite Milton-Parc), métro Sherbrooke ou Saint-Laurent à pied, dispo 1er juillet 2026, animaux limités, prix à la limite haute du budget</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/83/83da6eb9-3422-4702-b436-ed820032998c?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/8d/8d95567f-3a46-42b2-bcd6-c8ea29c0a1ff?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -2391,27 +2391,27 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 lumineux, 2 chambres fermées, 2 balcons – Rosemont, près Cinéma Beaubien</t>
+          <t>Condo 4½ meublé avec stationnement, près métro Jarry/Crémazie – Villeray</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2G 2S1)</t>
+          <t>8478 Rue Saint-Dominique, Montréal</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2290</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>946</t>
+          <t>930</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Jarry ou Crémazie</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -2436,17 +2436,17 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>5 (estimé)</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-lumineux-2-ch-fermees-renove-rosemont-petite-patrie/1739560132</t>
+          <t>https://duproprio.com/fr/location/montreal/villeray-st-michel-parc-extension/4-1-2-a-louer/hab-8478-saint-dominique-1134387</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">
@@ -2456,19 +2456,19 @@
       </c>
       <c r="P23" s="6" t="inlineStr">
         <is>
-          <t>Animaux limités, 3e étage, buanderie et lave-vaisselle inclus, à deux pas du Cinéma Beaubien, libre 1er juillet 2026</t>
+          <t>Meublé (TV 65po, mobilier complet), stationnement intérieur inclus, thermopompe, animaux négociables, bail min 12 mois, dispo 1er juillet 2026, hydro ~75$/mois + assurance 25$/mois en sus</t>
         </is>
       </c>
       <c r="Q23" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c1/c15d7c88-4278-46b2-b504-86cd39d6404b?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1134387/4-1-2-villeray-st-michel-parc-extension-600-15713346.jpg</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2478,27 +2478,27 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Appartement lumineux sur la plaza</t>
+          <t>4 1/2 (2 chambres), 900 pi², balcon, tout inclus – Rosemont (rue Dandurand)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>La Petite-Patrie</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>rue Saint-Hubert, H2S 2L9</t>
+          <t>3320 Rue Dandurand, Montréal, QC H1X 1M6</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>1999</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -2513,17 +2513,17 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Iberville</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5 (estimé)</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="N24" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-lumineux-sur-la-plaza/1739853332</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/condo-a-louer-2-chambres-rosemont-petite-patrie-tout-inclus/1739170766</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -2543,19 +2543,19 @@
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>2 ch fermées + boudoir avec grand placard, Plaza St-Hubert au pied de l'immeuble (quartier très vivant), laveuse-sécheuse dans l'unité, clim, 1 stationnement, grand balcon, métro Beaubien à 2 min selon l'annonce, dispo 15 juillet 2026, animaux limités</t>
+          <t>Construit 2012, tout inclus (chauffage, hydro, eau, wifi, climatisation), semi-meublé (électros + meubles salon/cuisine, matelas non inclus), animaux limités, dispo 1er juillet 2026, à 5-10 min à pied des commerces/restos de la rue Masson</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/29/29f42067-d07c-42c9-9127-b218f6f690f8?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/ba/bacee7d5-1abf-4a36-80b6-12877aa40971?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -2565,27 +2565,27 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Condo 4½ rénové avec stationnement</t>
+          <t>Appartement 2 chambres fermées, 974 pi², balcon – Plateau (Gilford/Chambord)</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Rosemont/La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>6855, rue d'Iberville, Montréal</t>
+          <t>n/d (Montréal, QC H2J 3L2, coin Gilford/Chambord)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>1010</t>
+          <t>974</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -2600,27 +2600,27 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>D'Iberville</t>
+          <t>Mont-Royal ou Laurier</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/4-1-2-a-louer/hab-6855-diberville-1136946</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-2-chambre-plateau-mont-royal/1739725006</t>
         </is>
       </c>
       <c r="O25" s="5" t="inlineStr">
@@ -2630,12 +2630,12 @@
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>2 chambres fermées, cuisine et sdb modernes, climatisé, stationnement, rangement ext., animaux acceptés, dispo 16 juillet 2026</t>
+          <t>Rez-de-jardin lumineux, sdb rénovée 2021, cuisine rénovée 2019, tous électros inclus + laveuse-sécheuse, à 2 min de l'avenue Mont-Royal, près parcs Lafontaine et Laurier, animaux limités, dispo 1er juillet ou août 2026</t>
         </is>
       </c>
       <c r="Q25" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202607/1136946/4-1-2-rosemont-petite-patrie-600-15776920.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/83/83da6eb9-3422-4702-b436-ed820032998c?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2652,32 +2652,32 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>6 1/2, balcon et terrasse, animaux acceptés – Hochelaga</t>
+          <t>5 1/2 lumineux, 2 chambres fermées, 2 balcons – Rosemont, près Cinéma Beaubien</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>1841 Rue Saint-Germain, Montréal</t>
+          <t>n/d (Montréal, QC H2G 2S1)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>946</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -2687,27 +2687,27 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Préfontaine</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr">
         <is>
-          <t>https://centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/25697495</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-lumineux-2-ch-fermees-renove-rosemont-petite-patrie/1739560132</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
@@ -2717,12 +2717,12 @@
       </c>
       <c r="P26" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, animaux acceptés sous conditions (chiens ok), 1 stationnement, libre 7 jours après acceptation du bail, vérification de crédit requise</t>
+          <t>Animaux limités, 3e étage, buanderie et lave-vaisselle inclus, à deux pas du Cinéma Beaubien, libre 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA16F1EEDDDDDDDDDD4&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c1/c15d7c88-4278-46b2-b504-86cd39d6404b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2739,32 +2739,32 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail – Grand 5 1/2 lumineux, balcon et terrasse – Hochelaga/Préfontaine</t>
+          <t>Appartement lumineux sur la plaza</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>La Petite-Patrie</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1V 2X2, secteur Préfontaine)</t>
+          <t>rue Saint-Hubert, H2S 2L9</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -2774,17 +2774,17 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Préfontaine</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cession-de-bail-grand-5-1-2-lumineux-hochelaga-prefontaine/1739376269</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/appartement-lumineux-sur-la-plaza/1739853332</t>
         </is>
       </c>
       <c r="O27" s="5" t="inlineStr">
@@ -2804,12 +2804,12 @@
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>1er mois gratuit, animaux acceptés (même chiens), hydro et stationnement inclus, buanderie, bail jusqu'en juin 2027</t>
+          <t>2 ch fermées + boudoir avec grand placard, Plaza St-Hubert au pied de l'immeuble (quartier très vivant), laveuse-sécheuse dans l'unité, clim, 1 stationnement, grand balcon, métro Beaubien à 2 min selon l'annonce, dispo 15 juillet 2026, animaux limités</t>
         </is>
       </c>
       <c r="Q27" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/9b/9b7ac581-3ab1-482b-9f87-d703dcb6bcc3?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/29/29f42067-d07c-42c9-9127-b218f6f690f8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -2826,27 +2826,27 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 Villeray . Christophe-Colomb.</t>
+          <t>Condo 4½ rénové avec stationnement</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Rosemont/La Petite-Patrie</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Jarry/Christophe-Colomb, Montréal, QC H2P 0C3</t>
+          <t>6855, rue d'Iberville, Montréal</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>2305</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>1054</t>
+          <t>1010</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2861,27 +2861,27 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>D'Iberville</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
+          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/4-1-2-a-louer/hab-6855-diberville-1136946</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -2891,19 +2891,19 @@
       </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er sept 2026, internet et clim inclus, tous électros inclus (four frigo lave-vaisselle laveuse-sécheuse), animaux acceptés, immeuble béton insonorisé avec gym/ascenseur/concierge, grand balcon-terrasse privé</t>
+          <t>2 chambres fermées, cuisine et sdb modernes, climatisé, stationnement, rangement ext., animaux acceptés, dispo 16 juillet 2026</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202607/1136946/4-1-2-rosemont-petite-patrie-600-15776920.jpg</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -2913,22 +2913,22 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>4 1/2 sur 2 étages, condo neuf « Joseph », balcon, près métro Joliette</t>
+          <t>6 1/2, balcon et terrasse, animaux acceptés – Hochelaga</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>3420 boul. Saint-Joseph Est, Montréal, QC H1X 0A6</t>
+          <t>1841 Rue Saint-Germain, Montréal</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Préfontaine</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -2958,32 +2958,32 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-sur-2-etages-condo-appartement-a-louer-rosemont-joseph/1727979165</t>
+          <t>https://centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/25697495</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>Condo neuf « Joseph » sur 2 étages, face au parc Lafond, eau chaude et climatisation incluses, électros neufs (laveuse-sécheuse inclus), piscine extérieure/gym/stationnement intérieur payant, animaux acceptés, superficie non précisée, près Stade olympique et Jardin botanique</t>
+          <t>Semi-meublé, animaux acceptés sous conditions (chiens ok), 1 stationnement, libre 7 jours après acceptation du bail, vérification de crédit requise</t>
         </is>
       </c>
       <c r="Q29" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/2a/2a378c4c-30df-42fd-8c0d-515e4ee71bc4?rule=kijijica-960-jpg</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA16F1EEDDDDDDDDDD4&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 RDC rénové avec cour – Hochelaga, près Pie-IX</t>
+          <t>Cession de bail – Grand 5 1/2 lumineux, balcon et terrasse – Hochelaga/Préfontaine</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -3010,32 +3010,32 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>1711 Avenue d'Orléans, Montréal, QC H1W 3R4</t>
+          <t>n/d (Montréal, QC H1V 2X2, secteur Préfontaine)</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>Pie-IX</t>
+          <t>Préfontaine</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
@@ -3055,22 +3055,22 @@
       </c>
       <c r="N30" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/hochelaga-superbe-5-1-2-renove-au-rez-de-chaussee-avec-cour/1740256793</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/cession-de-bail-grand-5-1-2-lumineux-hochelaga-prefontaine/1739376269</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>Animaux limités, stationnement inclus, cour arrière privée, climatisation, libre 1er juillet 2026</t>
+          <t>1er mois gratuit, animaux acceptés (même chiens), hydro et stationnement inclus, buanderie, bail jusqu'en juin 2027</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/d0/d0d75179-15a9-4d6e-a66c-024195759d32?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/9b/9b7ac581-3ab1-482b-9f87-d703dcb6bcc3?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3087,27 +3087,27 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 avec garage, grande cour – Hochelaga (Place Valois)</t>
+          <t>4 1/2 Villeray . Christophe-Colomb.</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1W 3N6, angle Bourbonnière/Ontario)</t>
+          <t>Jarry/Christophe-Colomb, Montréal, QC H2P 0C3</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2305</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>1054</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -3117,22 +3117,22 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>n/d (grande cour arrière privée)</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>9 (estimé)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
@@ -3142,29 +3142,29 @@
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-avec-garage-a-louer-dans-hochelaga-mainsonneuve/1739944242</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P31" s="6" t="inlineStr">
         <is>
-          <t>Chauffage et climatisation centrale inclus, chats seulement (pas de chiens), 2 places de stationnement + 1 garage, libre 1er août 2026, près Place Valois</t>
+          <t>Dispo 1er sept 2026, internet et clim inclus, tous électros inclus (four frigo lave-vaisselle laveuse-sécheuse), animaux acceptés, immeuble béton insonorisé avec gym/ascenseur/concierge, grand balcon-terrasse privé</t>
         </is>
       </c>
       <c r="Q31" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/3e/3efd086c-a651-43a1-8291-a49f0c1d38d5?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Grand 5 1/2 lumineux, à 200m du métro Laurier – Plateau</t>
+          <t>4½ rénové, 1000 pi², près métro Laurier – Plateau (Parc-Lafontaine)</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -3184,17 +3184,17 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2J 2Y3)</t>
+          <t>4225 Rue de Lanaudière, Montréal, QC H2J 3N8</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>oui (petit balcon cuisine)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="N32" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-51-2-lumineux-sur-plateau-mont-royal/1738318103</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/tres-beau-4-recemment-renove-au-coeur-du-plateau-mont-royal/1739158104</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr">
@@ -3239,19 +3239,19 @@
       </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>Chauffage inclus, animaux limités, walk-in dans chambre principale, libre 1er juillet 2026</t>
+          <t>2e étage, laveuse-sécheuse-poêle-frigo inclus, non-fumeur, pas d'animaux, aucun stationnement, dispo 1er juillet 2026, près parc La Fontaine, walk score 10/10</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/d0/d0ca9a85-dbf8-4673-a89d-264708952626?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/15/15437f31-23a1-4bd9-9a52-5d9b817ca005?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -3261,22 +3261,22 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Grand 5½ meublé et entièrement rénové</t>
+          <t>4 1/2 sur 2 étages, condo neuf « Joseph », balcon, près métro Joliette</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>13e Avenue, Montréal (près métro Saint-Michel)</t>
+          <t>3420 boul. Saint-Joseph Est, Montréal, QC H1X 0A6</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>2265</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -3296,27 +3296,27 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Saint-Michel</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353226</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-sur-2-etages-condo-appartement-a-louer-rosemont-joseph/1727979165</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr">
@@ -3326,10 +3326,14 @@
       </c>
       <c r="P33" s="6" t="inlineStr">
         <is>
-          <t>5½ 3 chambres, meublé, laveuse-sécheuse, comptoirs quartz, balcon + terrasse, métro Saint-Michel à 394 m, cession de bail jusqu'au 30 juin 2027, pas d'animaux, limite est de Villeray</t>
-        </is>
-      </c>
-      <c r="Q33" s="5" t="inlineStr"/>
+          <t>Condo neuf « Joseph » sur 2 étages, face au parc Lafond, eau chaude et climatisation incluses, électros neufs (laveuse-sécheuse inclus), piscine extérieure/gym/stationnement intérieur payant, animaux acceptés, superficie non précisée, près Stade olympique et Jardin botanique</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/2a/2a378c4c-30df-42fd-8c0d-515e4ee71bc4?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -3344,62 +3348,62 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>5½ 2e étage Jarry Est rénové</t>
+          <t>5 1/2 RDC rénové avec cour – Hochelaga, près Pie-IX</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>582 rue Jarry Est, Montréal</t>
+          <t>1711 Avenue d'Orléans, Montréal, QC H1W 3R4</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Pie-IX</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>LogisQuébec</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr">
         <is>
-          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353442</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/hochelaga-superbe-5-1-2-renove-au-rez-de-chaussee-avec-cour/1740256793</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
@@ -3409,10 +3413,14 @@
       </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>5½ 3 chambres fermées, rénové, climatisation murale, balcons avant et arrière, métro Jarry à 103 m, disponible immédiatement, enquête de crédit exigée</t>
-        </is>
-      </c>
-      <c r="Q34" s="5" t="inlineStr"/>
+          <t>Animaux limités, stationnement inclus, cour arrière privée, climatisation, libre 1er juillet 2026</t>
+        </is>
+      </c>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/d0/d0d75179-15a9-4d6e-a66c-024195759d32?rule=kijijica-960-jpg</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -3427,27 +3435,27 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 rénové, stationnement, patio – Plateau</t>
+          <t>5 1/2 avec garage, grande cour – Hochelaga (Place Valois)</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>2181A Rue Marie-Anne, Montréal, QC H2H 1M9</t>
+          <t>n/d (Montréal, QC H1W 3N6, angle Bourbonnière/Ontario)</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>950</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -3457,22 +3465,22 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>oui (patio arrière)</t>
+          <t>n/d (grande cour arrière privée)</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>9 (estimé)</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
@@ -3482,22 +3490,22 @@
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-avec-stationnement-2-chambres-renove/1739130207</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-avec-garage-a-louer-dans-hochelaga-mainsonneuve/1739944242</t>
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P35" s="6" t="inlineStr">
         <is>
-          <t>Non chauffé, animaux limités, stationnement privé inclus, planchers bois franc, libre 15 juillet 2026</t>
+          <t>Chauffage et climatisation centrale inclus, chats seulement (pas de chiens), 2 places de stationnement + 1 garage, libre 1er août 2026, près Place Valois</t>
         </is>
       </c>
       <c r="Q35" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2e8a22d5-2d29-437c-bd2c-a9be0878ff77?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/3e/3efd086c-a651-43a1-8291-a49f0c1d38d5?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3514,27 +3522,27 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 Villeray - 2 chambres - près du métro Jarry - 2050$</t>
+          <t>Grand 5 1/2 lumineux, à 200m du métro Laurier – Plateau</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Montréal, QC H2R</t>
+          <t>n/d (Montréal, QC H2J 2Y3)</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
@@ -3544,12 +3552,12 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui (petit balcon cuisine)</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -3559,7 +3567,7 @@
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr">
@@ -3569,22 +3577,22 @@
       </c>
       <c r="N36" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-villeray-2-chambres-pres-du-metro-jarry-2050/1738384606</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-51-2-lumineux-sur-plateau-mont-royal/1738318103</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P36" s="6" t="inlineStr">
         <is>
-          <t>Dispo 1er juin 2026, rénové, 2 chambres + bureau, thermopompe (chauffage/clim), 5 électros inclus, cour-patio arrière, planchers bois franc refaits, pas d'animaux</t>
+          <t>Chauffage inclus, animaux limités, walk-in dans chambre principale, libre 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q36" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cf44ffec-5a1f-4ffd-81e0-2eb0cfc316d8?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/d0/d0ca9a85-dbf8-4673-a89d-264708952626?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3601,27 +3609,27 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 rénové, 995 pi², près Promenade Masson – Rosemont</t>
+          <t>Grand 5½ meublé et entièrement rénové</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>5472 1ere Avenue, Montréal</t>
+          <t>13e Avenue, Montréal (près métro Saint-Michel)</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2265</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -3631,54 +3639,50 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Saint-Michel</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/5-1-2-a-louer/hab-5472-1ere-avenue-882773</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353226</t>
         </is>
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P37" s="6" t="inlineStr">
         <is>
-          <t>Chauffage au plancher radiant, climatisation, cour privée avec remise, près Promenade Masson et parc Pélican, non-fumeurs</t>
-        </is>
-      </c>
-      <c r="Q37" s="5" t="inlineStr">
-        <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/201911/882773/5-1-2-plateau-mont-royal-1600-10690669.jpg</t>
-        </is>
-      </c>
+          <t>5½ 3 chambres, meublé, laveuse-sécheuse, comptoirs quartz, balcon + terrasse, métro Saint-Michel à 394 m, cession de bail jusqu'au 30 juin 2027, pas d'animaux, limite est de Villeray</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -3688,22 +3692,22 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
+          <t>5½ 2e étage Jarry Est rénové</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
+          <t>582 rue Jarry Est, Montréal</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -3718,12 +3722,12 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal ou Papineau (à vérifier)</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -3733,34 +3737,30 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>12 (estimé)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>LogisQuébec</t>
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
+          <t>https://www.logisquebec.com/appartement-a-louer-villeray_saint-michel_parc-extension-l353442</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
-        </is>
-      </c>
-      <c r="Q38" s="5" t="inlineStr">
-        <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
-        </is>
-      </c>
+          <t>5½ 3 chambres fermées, rénové, climatisation murale, balcons avant et arrière, métro Jarry à 103 m, disponible immédiatement, enquête de crédit exigée</t>
+        </is>
+      </c>
+      <c r="Q38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
+          <t>5 1/2 rénové, stationnement, patio – Plateau</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -3785,67 +3785,67 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>62 rue Rachel Est, Montréal</t>
+          <t>2181A Rue Marie-Anne, Montréal, QC H2H 1M9</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>oui (patio arrière)</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="K39" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
-        </is>
-      </c>
-      <c r="K39" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-avec-stationnement-2-chambres-renove/1739130207</t>
         </is>
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P39" s="6" t="inlineStr">
         <is>
-          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
+          <t>Non chauffé, animaux limités, stationnement privé inclus, planchers bois franc, libre 15 juillet 2026</t>
         </is>
       </c>
       <c r="Q39" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/2e/2e8a22d5-2d29-437c-bd2c-a9be0878ff77?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3862,42 +3862,42 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
+          <t>5 1/2 Villeray - 2 chambres - près du métro Jarry - 2050$</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>4275 Rue de Bordeaux, Montréal</t>
+          <t>Montréal, QC H2R</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>2095</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -3907,32 +3907,32 @@
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-villeray-2-chambres-pres-du-metro-jarry-2050/1738384606</t>
         </is>
       </c>
       <c r="O40" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
+          <t>Dispo 1er juin 2026, rénové, 2 chambres + bureau, thermopompe (chauffage/clim), 5 électros inclus, cour-patio arrière, planchers bois franc refaits, pas d'animaux</t>
         </is>
       </c>
       <c r="Q40" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cf44ffec-5a1f-4ffd-81e0-2eb0cfc316d8?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -3949,82 +3949,430 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
+          <t>5 1/2 rénové, 995 pi², près Promenade Masson – Rosemont</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Rosemont-La Petite-Patrie</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>5472 1ere Avenue, Montréal</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>995</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N41" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/rosemont-la-petite-patrie/5-1-2-a-louer/hab-5472-1ere-avenue-882773</t>
+        </is>
+      </c>
+      <c r="O41" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="P41" s="6" t="inlineStr">
+        <is>
+          <t>Chauffage au plancher radiant, climatisation, cour privée avec remise, près Promenade Masson et parc Pélican, non-fumeurs</t>
+        </is>
+      </c>
+      <c r="Q41" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/201911/882773/5-1-2-plateau-mont-royal-1600-10690669.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>2150</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>Mont-Royal ou Papineau (à vérifier)</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>12 (estimé)</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N42" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
+        </is>
+      </c>
+      <c r="O42" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P42" s="6" t="inlineStr">
+        <is>
+          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
+        </is>
+      </c>
+      <c r="Q42" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>62 rue Rachel Est, Montréal</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>2195</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>8 (estimé)</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
+        </is>
+      </c>
+      <c r="O43" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P43" s="6" t="inlineStr">
+        <is>
+          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
+        </is>
+      </c>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Le Plateau-Mont-Royal</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>4275 Rue de Bordeaux, Montréal</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>2095</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>Mont-Royal</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>10 (estimé)</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N44" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
+        </is>
+      </c>
+      <c r="O44" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P44" s="6" t="inlineStr">
+        <is>
+          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
+        </is>
+      </c>
+      <c r="Q44" s="5" t="inlineStr">
+        <is>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
           <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>1889 Rue des Carrières, Montréal</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t>2375</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I41" s="5" t="inlineStr">
+      <c r="I45" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="J41" s="5" t="inlineStr">
+      <c r="J45" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="K41" s="5" t="inlineStr">
+      <c r="K45" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="L41" s="5" t="inlineStr">
+      <c r="L45" s="5" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="M41" s="5" t="inlineStr">
+      <c r="M45" s="5" t="inlineStr">
         <is>
           <t>Centris</t>
         </is>
       </c>
-      <c r="N41" s="7" t="inlineStr">
+      <c r="N45" s="7" t="inlineStr">
         <is>
           <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
         </is>
       </c>
-      <c r="O41" s="5" t="inlineStr">
+      <c r="O45" s="5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="P41" s="6" t="inlineStr">
+      <c r="P45" s="6" t="inlineStr">
         <is>
           <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
         </is>
       </c>
-      <c r="Q41" s="5" t="inlineStr">
+      <c r="Q45" s="5" t="inlineStr">
         <is>
           <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE603764DDDDDDDDDDD&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q41"/>
+  <autoFilter ref="A1:Q45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -4066,6 +4414,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour des annonces — 2026-07-27 17:19
</commit_message>
<xml_diff>
--- a/annonces.xlsx
+++ b/annonces.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Annonces" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$173</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$172</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q173"/>
+  <dimension ref="A1:Q172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -576,7 +576,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Grand logement 5½ sur deux niveaux, 3 chambres (2 au sous-sol), terrasse privée, +1300 pi² - rue Villeray</t>
+          <t>Grand 6½ rénové, 3 chambres fermées, 2 balcons, 1250 pi² - Villeray (à 3 min du métro Jarry)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -586,17 +586,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1180, Rue Villeray, Montréal, QC</t>
+          <t>n/d (Montréal, QC H2R 2E8)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1300</t>
+          <t>1250</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Jarry (estimé)</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -621,17 +621,17 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>n/d (estimé, non précisé par l'annonce)</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/28201368</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-6-1-2-villeray-metro-jarry/1741040354</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -641,12 +641,12 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Sur deux niveaux, 2 chambres au sous-sol, 2 salles de bain, terrasse privée accessible depuis le salon, climatisation, chats acceptés (chiens refusés), disponible 1er juillet 2026, vérification de crédit exigée. Walk Score 97. Distance exacte au métro non précisée par l'annonce.</t>
+          <t>2 balcons (avant et grand balcon arriere), tres proche du metro Jarry, bon rapport superficie/prix. Date de disponibilite et politique animaux non precisees par l'annonce.</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA12F7C2DDDDDDDDDDB&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/46/46b63ae7-8eba-4e92-8ed2-6e9e7bc83ccc?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>4½ meublé tout inclus, 2 chambres fermées, 2 balcons, 1062 pi² - coin Marie-Anne / De La Roche (Plateau, 10 min métro Mont-Royal)</t>
+          <t>4½ rénové, 2 chambres fermées, balcon, 950 pi² - Mile-End (Plateau), à ~10 min du métro Outremont</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Coin Marie-Anne / De La Roche, Montréal, QC</t>
+          <t>5970, Avenue du Parc, app. 7, Montréal</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>1062</t>
+          <t>950</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -698,42 +698,42 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Outremont</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10 (estime, non precise par l'annonce)</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-renove-meuble-tout-inclus-a-louer-au-plateau-mont-royal/1741126451</t>
+          <t>https://duproprio.com/en/rental/montreal/le-plateau-mont-royal/4-1-2-for-rent/hab-7-5970-ave-du-parc-1138366</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Meublé et tout inclus (chauffage, hydro, eau), climatisation, laveuse-sécheuse, duplex rénové, bail d'un an, disponible 1er octobre 2026. Animaux non acceptés. Près du parc La Fontaine.</t>
+          <t>Dernier etage (3e), semi-meuble, stationnement exterieur inclus, disponible 1er septembre 2026. Secteur Mile-End (bordure Plateau/Outremont), distance au metro estimee.</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/64/648b2cd8-c897-4566-a61f-606084978ae2?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202607/1138366/4-1-2-plateau-mont-royal-1600-15812906.jpg</t>
         </is>
       </c>
     </row>
@@ -750,171 +750,171 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>4½ rénové, 2 chambres fermées, balcon, 1060 pi² - Plateau-Mont-Royal (proche métro Mont-Royal et Laurier)</t>
+          <t>Grand condo 4 chambres fermées - rue Jean-Talon Ouest (Villeray), à ~5 min du métro Acadie</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2T 1R2)</t>
+          <t>816, Rue Jean-Talon Ouest, Montréal</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1060</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Acadie</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>bleue</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>5-6 (estime)</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Centris</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/25680514</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>7 pieces / 4 chambres fermees, 2 salles de bain, animaux acceptes sous conditions, disponible 1er juillet 2026, visite virtuelle 3D. Superficie non precisee par la fiche ; balcon non mentionne.</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD978B3DDDDDDDDDD1&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>vu</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Joli 7½ (3 chambres), terrasse et cour - à 5 min du métro Joliette (Hochelaga)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Hochelaga-Maisonneuve</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>n/d (Montréal, QC H1W 3C5)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Mont-Royal / Laurier</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Joliette</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>verte</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>n/d (à proximité, non précisé)</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Kijiji</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-a-louer-for-rent-a-montreal/1740574295</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>Cuisine et salle de bain rénovées, laveuse-sécheuse et lave-vaisselle inclus, disponible 14 juillet 2026, animaux non acceptés. Proche marché Jean-Talon et rues commerçantes. Distance exacte au métro non précisée dans l'annonce.</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/81/81465b98-f467-42c0-b787-6b73694a8b76?rule=kijijica-960-jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>NOUVEAU</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>4½ meublé tout inclus, 2 chambres + bureau, balcon et patio, 1000 pi² - rue St-Denis (5 min métro Crémazie)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Villeray</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>n/d (Rue St-Denis, Montréal, QC H2M)</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>2100</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Crémazie</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Kijiji</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-4-renove-patio-stationnement-ve-internet-cremazie/1740602257</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
-        <is>
-          <t>Meublé et tout inclus, internet haute vitesse, recharge VE niveau 2, climatisation, disponible 1er septembre 2026, bail d'un an, sous-location et Airbnb interdits, animaux limités. À la limite Villeray/Ahuntsic près du métro Crémazie (ligne orange, pas ligne verte).</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cfa981e7-1243-46fe-b5b8-1cbe5357eb8b?rule=kijijica-960-jpg</t>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/joli-7-lumineux-avec-terrasse-et-cour-a-5-min-metro-joliette/1740607211</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>Rez-de-chaussée avec étage, balcon + grande terrasse arrière et cabanon, 1 stationnement inclus, lave-vaisselle et laveuse-sécheuse inclus, meubles disponibles au besoin, animaux acceptés sous conditions, bail au mois possible, dispo 1er août 2026</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/51/51601618-bdf1-4776-88b2-c87738ad33ef?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Joli 7½ (3 chambres), terrasse et cour - à 5 min du métro Joliette (Hochelaga)</t>
+          <t>5 1/2 rénové 3 chambres près métro Joliette (cession de bail)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1W 3C5)</t>
+          <t>Près du parc Lalancette (adresse exacte n/d)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2245</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/joli-7-lumineux-avec-terrasse-et-cour-a-5-min-metro-joliette/1740607211</t>
+          <t>https://www.facebook.com/marketplace/item/1611452633675447</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>Rez-de-chaussée avec étage, balcon + grande terrasse arrière et cabanon, 1 stationnement inclus, lave-vaisselle et laveuse-sécheuse inclus, meubles disponibles au besoin, animaux acceptés sous conditions, bail au mois possible, dispo 1er août 2026</t>
+          <t>Cession de bail. 1100 pi2 rénové, 3 grandes chambres fermées avec garde-robe dont une avec balcon, second balcon sur cour, locker au sous-sol, chauffage/eau chaude/wifi inclus. 5 min à pied du métro Joliette selon la fiche, dispo 1er août. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/51/51601618-bdf1-4776-88b2-c87738ad33ef?rule=kijijica-960-jpg</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/744782828_2425425677956674_6748123711102009567_n.jpg?stp=c0.123.1290.1290a_dst-jpg_tt6&amp;cstp=mx1290x1290&amp;ctp=s565x565&amp;_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=QyFHGQtYXmAQ7kNvwGAvYTo&amp;_nc_oc=Adq0n0QGekjLictcQqyNCD5OWzTZP-ByT68TnmMdUFrBRe8Gta7m-AQEhavEJDocpUc&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=yYLPvMa76LbSuFVLINSV0A&amp;_nc_ss=7f2a8&amp;oh=00_AQDVDHWYGsY5IWfgFMiwv6A_Kyu3om9l3ovYSoj1ta0YRw&amp;oe=6A5D72BA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -1011,27 +1011,27 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 rénové 3 chambres près métro Joliette (cession de bail)</t>
+          <t>Grand logement 5½ sur deux niveaux, 3 chambres (2 au sous-sol), terrasse privée, +1300 pi² - rue Villeray</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Près du parc Lalancette (adresse exacte n/d)</t>
+          <t>1180, Rue Villeray, Montréal, QC</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>2245</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1300</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1046,42 +1046,42 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Jarry (estimé)</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>n/d (estimé, non précisé par l'annonce)</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1611452633675447</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/28201368</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail. 1100 pi2 rénové, 3 grandes chambres fermées avec garde-robe dont une avec balcon, second balcon sur cour, locker au sous-sol, chauffage/eau chaude/wifi inclus. 5 min à pied du métro Joliette selon la fiche, dispo 1er août. Lien Facebook (connexion requise)</t>
+          <t>Sur deux niveaux, 2 chambres au sous-sol, 2 salles de bain, terrasse privée accessible depuis le salon, climatisation, chats acceptés (chiens refusés), disponible 1er juillet 2026, vérification de crédit exigée. Walk Score 97. Distance exacte au métro non précisée par l'annonce.</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/744782828_2425425677956674_6748123711102009567_n.jpg?stp=c0.123.1290.1290a_dst-jpg_tt6&amp;cstp=mx1290x1290&amp;ctp=s565x565&amp;_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=QyFHGQtYXmAQ7kNvwGAvYTo&amp;_nc_oc=Adq0n0QGekjLictcQqyNCD5OWzTZP-ByT68TnmMdUFrBRe8Gta7m-AQEhavEJDocpUc&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=yYLPvMa76LbSuFVLINSV0A&amp;_nc_ss=7f2a8&amp;oh=00_AQDVDHWYGsY5IWfgFMiwv6A_Kyu3om9l3ovYSoj1ta0YRw&amp;oe=6A5D72BA</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA12F7C2DDDDDDDDDDB&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -2490,32 +2490,32 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Grand 6 1/2 rénové, terrasse privée – Villeray, près métro Crémazie</t>
+          <t>5 1/2 balcon, 3 chambres – Rosemont (14e Avenue / Masson)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2P 2G9, secteur parc Jarry)</t>
+          <t>n/d (Montréal, QC H1X 2W2, secteur 14e Avenue/Masson)</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>2035</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>1250</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Crémazie</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="N24" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/a-louer:-appartement-6-1-2-dans-villeray/1738327789</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-beds-2-baths-apartment/1740599440</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -2555,19 +2555,19 @@
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>Grande terrasse privée arrière + balcons avant/arrière, cuisine et salle de bain rénovées (douche romaine, puits de lumière), 4 électros + lave-vaisselle inclus, chauffage et eau chaude inclus (160$/mois fixe), piste cyclable devant, dispo 1er juillet 2026, bail 1 an</t>
+          <t>Unité au rez-de-chaussée d'un duplex/triplex, salon-solarium lumineux, cour arrière privée, garage intérieur + stationnement extérieur, climatisation, pas d'animaux, dispo 1er août 2026</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/c3/c339486c-6795-4d47-bcc5-625d60d299a0?rule=kpetroleumica-640-webp</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/69/69d4ef7d-f6c5-401d-a2f8-9ca904eb6639?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -2577,32 +2577,32 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 balcon, 3 chambres – Rosemont (14e Avenue / Masson)</t>
+          <t>4½ rénové, 2 chambres fermées, balcon, 1060 pi² - Plateau-Mont-Royal (proche métro Mont-Royal et Laurier)</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H1X 2W2, secteur 14e Avenue/Masson)</t>
+          <t>n/d (Montréal, QC H2T 1R2)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1060</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2612,17 +2612,17 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Mont-Royal / Laurier</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>n/d (à proximité, non précisé)</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
@@ -2632,22 +2632,22 @@
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/3-beds-2-baths-apartment/1740599440</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-5-a-louer-for-rent-a-montreal/1740574295</t>
         </is>
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>Unité au rez-de-chaussée d'un duplex/triplex, salon-solarium lumineux, cour arrière privée, garage intérieur + stationnement extérieur, climatisation, pas d'animaux, dispo 1er août 2026</t>
+          <t>Cuisine et salle de bain rénovées, laveuse-sécheuse et lave-vaisselle inclus, disponible 14 juillet 2026, animaux non acceptés. Proche marché Jean-Talon et rues commerçantes. Distance exacte au métro non précisée dans l'annonce.</t>
         </is>
       </c>
       <c r="Q25" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-dealer-ads/images/69/69d4ef7d-f6c5-401d-a2f8-9ca904eb6639?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/81/81465b98-f467-42c0-b787-6b73694a8b76?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -5509,7 +5509,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -5519,7 +5519,7 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>4½ spacieux, 2 chambres, grand balcon-terrasse privé, 1054 pi² - avenue Christophe-Colomb (Villeray, près rue Jarry)</t>
+          <t>4½ meublé tout inclus, 2 chambres + bureau, balcon et patio, 1000 pi² - rue St-Denis (5 min métro Crémazie)</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -5529,17 +5529,17 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Avenue Christophe-Colomb (près rue Jarry), Montréal, QC H2P 0C3</t>
+          <t>n/d (Rue St-Denis, Montréal, QC H2M)</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>2305</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>1054</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Crémazie</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="L59" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M59" s="5" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="N59" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/grand-4-renove-patio-stationnement-ve-internet-cremazie/1740602257</t>
         </is>
       </c>
       <c r="O59" s="5" t="inlineStr">
@@ -5584,12 +5584,12 @@
       </c>
       <c r="P59" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail (locataires actuels achètent un condo), disponible 1er septembre 2026. 2 chambres (12x13 et 12x14 pi), électroménagers inclus (four, frigo, lave-vaisselle, laveuse-sécheuse), climatisation, internet inclus, salle d'entraînement dans l'immeuble. Près de la rue Jarry (IGA, café, pharmacie). Enquête de crédit requise. Adresse précise non indiquée par l'annonce (seulement code postal H2P 0C3) — distance exacte au métro Jarry estimée.</t>
+          <t>Meublé et tout inclus, internet haute vitesse, recharge VE niveau 2, climatisation, disponible 1er septembre 2026, bail d'un an, sous-location et Airbnb interdits, animaux limités. À la limite Villeray/Ahuntsic près du métro Crémazie (ligne orange, pas ligne verte).</t>
         </is>
       </c>
       <c r="Q59" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/cf/cfa981e7-1243-46fe-b5b8-1cbe5357eb8b?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -5606,32 +5606,32 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Grand logement de 4 chambres fermées, terrasse ~1100 pi² - rue Ontario Est (Hochelaga-Maisonneuve, entre métro Pie-IX et Joliette)</t>
+          <t>4½ spacieux, 2 chambres, grand balcon-terrasse privé, 1054 pi² - avenue Christophe-Colomb (Villeray, près rue Jarry)</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>3889, rue Ontario Est, Montréal</t>
+          <t>Avenue Christophe-Colomb (près rue Jarry), Montréal, QC H2P 0C3</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2305</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>1054</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
@@ -5641,27 +5641,27 @@
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M60" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N60" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/3191099554424215</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-1-2-villeray-christophe-colomb/1739980393</t>
         </is>
       </c>
       <c r="O60" s="5" t="inlineStr">
@@ -5671,12 +5671,12 @@
       </c>
       <c r="P60" s="6" t="inlineStr">
         <is>
-          <t>4 chambres fermées, situé au 2e étage, aucun locataire en dessous, grande terrasse ~1100 pi² (superficie intérieure non précisée), dispo 1er juillet 2026. Walk Score 98/Transit 72. Lien Facebook (connexion requise).</t>
+          <t>Cession de bail (locataires actuels achètent un condo), disponible 1er septembre 2026. 2 chambres (12x13 et 12x14 pi), électroménagers inclus (four, frigo, lave-vaisselle, laveuse-sécheuse), climatisation, internet inclus, salle d'entraînement dans l'immeuble. Près de la rue Jarry (IGA, café, pharmacie). Enquête de crédit requise. Adresse précise non indiquée par l'annonce (seulement code postal H2P 0C3) — distance exacte au métro Jarry estimée.</t>
         </is>
       </c>
       <c r="Q60" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/734367592_37516698021250688_9048995181085965231_n.jpg?stp=c0.273.1206.1206a_dst-jpg_tt6&amp;cstp=mx1206x1206&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=nR4bexDdA7kQ7kNvwETwXRu&amp;_nc_oc=Adr8b_ZPIzcfgyLtbIjdkZ5tD3NsD-JGZbJKl6RPXDVY72qwup6OtDttajaoVBxtwXs&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=DKAPrnNgmI9udtZ3TamYHQ&amp;_nc_ss=7f2a8&amp;oh=00_AQB-a9NpI4qTkrXbihGbIld6aXJDIH_w-iC6HuVrESJzYg&amp;oe=6A6BCFE1</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/5d/5d7a6647-dba7-4661-87c0-6b86eeb875b6?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -5693,32 +5693,32 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>4½ rénové, 950 pi², balcon avant + terrasse arrière privée - rue St-Joseph Est (Plateau, près parc Laurier)</t>
+          <t>Grand logement de 4 chambres fermées, terrasse ~1100 pi² - rue Ontario Est (Hochelaga-Maisonneuve, entre métro Pie-IX et Joliette)</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>1570, rue St-Joseph Est, Montréal</t>
+          <t>3889, rue Ontario Est, Montréal</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
@@ -5728,27 +5728,27 @@
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>Laurier</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>12 (estimé, incertain)</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N61" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/4-1-2-a-louer/hab-1570-stjoseph-est-1119590</t>
+          <t>https://www.facebook.com/marketplace/item/3191099554424215</t>
         </is>
       </c>
       <c r="O61" s="5" t="inlineStr">
@@ -5758,19 +5758,19 @@
       </c>
       <c r="P61" s="6" t="inlineStr">
         <is>
-          <t>Planchers de bois franc, comptoirs de granit, cuisine à îlot, disponible maintenant. Distance réelle au métro Laurier non confirmée par l'annonce, possiblement proche de la limite de 12 min - à vérifier avant de contacter.</t>
+          <t>4 chambres fermées, situé au 2e étage, aucun locataire en dessous, grande terrasse ~1100 pi² (superficie intérieure non précisée), dispo 1er juillet 2026. Walk Score 98/Transit 72. Lien Facebook (connexion requise).</t>
         </is>
       </c>
       <c r="Q61" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202512/1119590/plateau-mont-royal-600-15379636.jpg</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/734367592_37516698021250688_9048995181085965231_n.jpg?stp=c0.273.1206.1206a_dst-jpg_tt6&amp;cstp=mx1206x1206&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=nR4bexDdA7kQ7kNvwETwXRu&amp;_nc_oc=Adr8b_ZPIzcfgyLtbIjdkZ5tD3NsD-JGZbJKl6RPXDVY72qwup6OtDttajaoVBxtwXs&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=DKAPrnNgmI9udtZ3TamYHQ&amp;_nc_ss=7f2a8&amp;oh=00_AQB-a9NpI4qTkrXbihGbIld6aXJDIH_w-iC6HuVrESJzYg&amp;oe=6A6BCFE1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
@@ -5780,7 +5780,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>4½ construction récente (2021), terrasse privée, animaux acceptés, 900 pi² - Plateau, 10 min du métro Mont-Royal/Laurier</t>
+          <t>4½ rénové, 950 pi², balcon avant + terrasse arrière privée - rue St-Joseph Est (Plateau, près parc Laurier)</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -5790,17 +5790,17 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>4609, Rue de la Roche, Montréal, QC H2J 3J5</t>
+          <t>1570, rue St-Joseph Est, Montréal</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>2265</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>950</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
@@ -5815,7 +5815,7 @@
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
@@ -5825,17 +5825,17 @@
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12 (estimé, incertain)</t>
         </is>
       </c>
       <c r="M62" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N62" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-sur-le-plateau-mont-royal-animaux-acceptes/1740915606</t>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/4-1-2-a-louer/hab-1570-stjoseph-est-1119590</t>
         </is>
       </c>
       <c r="O62" s="5" t="inlineStr">
@@ -5845,12 +5845,12 @@
       </c>
       <c r="P62" s="6" t="inlineStr">
         <is>
-          <t>Construction récente en béton (2021), tous électroménagers inclus (laveuse-sécheuse, lave-vaisselle, climatisation), grande terrasse privée avec accès cour, immeuble calme, gestion professionnelle, disponible 2026-08-01 (flexible)</t>
+          <t>Planchers de bois franc, comptoirs de granit, cuisine à îlot, disponible maintenant. Distance réelle au métro Laurier non confirmée par l'annonce, possiblement proche de la limite de 12 min - à vérifier avant de contacter.</t>
         </is>
       </c>
       <c r="Q62" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/6a/6a80881b-c819-4bdb-8f24-fa8f01cd5d3e?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202512/1119590/plateau-mont-royal-600-15379636.jpg</t>
         </is>
       </c>
     </row>
@@ -5867,7 +5867,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>5½ de 998 pi², 2 chambres + bureau, balcon et accès cour - Plateau (rue St-André, entre Roy et Cherrier), 5 min du métro Sherbrooke</t>
+          <t>4½ construction récente (2021), terrasse privée, animaux acceptés, 900 pi² - Plateau, 10 min du métro Mont-Royal/Laurier</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
@@ -5877,17 +5877,17 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Rue St-André (entre Roy et Cherrier), Montréal, QC H2L 3V7</t>
+          <t>4609, Rue de la Roche, Montréal, QC H2J 3J5</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2265</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>998</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>Sherbrooke</t>
+          <t>Mont-Royal</t>
         </is>
       </c>
       <c r="K63" s="5" t="inlineStr">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="L63" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="M63" s="5" t="inlineStr">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="N63" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-2-ch-bureau-balcon-acces-cour/1740581764</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/4-sur-le-plateau-mont-royal-animaux-acceptes/1740915606</t>
         </is>
       </c>
       <c r="O63" s="5" t="inlineStr">
@@ -5932,19 +5932,19 @@
       </c>
       <c r="P63" s="6" t="inlineStr">
         <is>
-          <t>3e étage, 2 chambres fermées + bureau fermé avec accès balcon, cour partagée, chauffage non inclus, animaux limités (pas de chien), près du parc La Fontaine, disponible 1er août</t>
+          <t>Construction récente en béton (2021), tous électroménagers inclus (laveuse-sécheuse, lave-vaisselle, climatisation), grande terrasse privée avec accès cour, immeuble calme, gestion professionnelle, disponible 2026-08-01 (flexible)</t>
         </is>
       </c>
       <c r="Q63" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/71/7166db6f-14eb-4ab6-ae28-b5af701014be?rule=kijijica-960-jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/6a/6a80881b-c819-4bdb-8f24-fa8f01cd5d3e?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
@@ -5954,27 +5954,27 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>2 chambres avec balcon, immeuble rénové - rue Iberville (Villeray/Parc-Ex), à 1 min du métro d'Iberville</t>
+          <t>5½ de 998 pi², 2 chambres + bureau, balcon et accès cour - Plateau (rue St-André, entre Roy et Cherrier), 5 min du métro Sherbrooke</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>7186, Rue Iberville, Montréal</t>
+          <t>Rue St-André (entre Roy et Cherrier), Montréal, QC H2L 3V7</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>998</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
@@ -5989,27 +5989,27 @@
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>D'Iberville</t>
+          <t>Sherbrooke</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M64" s="5" t="inlineStr">
         <is>
-          <t>DuProprio</t>
+          <t>Kijiji</t>
         </is>
       </c>
       <c r="N64" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/villeray-st-michel-parc-extension/5-1-2-a-louer/hab-7186-iberville-1132385</t>
+          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-1-2-plateau-2-ch-bureau-balcon-acces-cour/1740581764</t>
         </is>
       </c>
       <c r="O64" s="5" t="inlineStr">
@@ -6019,12 +6019,12 @@
       </c>
       <c r="P64" s="6" t="inlineStr">
         <is>
-          <t>Entièrement rénové (2024), plancher chauffant salle de bain, grand balcon arrière couvert, aucun animal, Walk Score 94, disponible 1er juillet 2026</t>
+          <t>3e étage, 2 chambres fermées + bureau fermé avec accès balcon, cour partagée, chauffage non inclus, animaux limités (pas de chien), près du parc La Fontaine, disponible 1er août</t>
         </is>
       </c>
       <c r="Q64" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132385/villeray-st-michel-parc-extension-600-15662542.jpg</t>
+          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/71/7166db6f-14eb-4ab6-ae28-b5af701014be?rule=kijijica-960-jpg</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6041,7 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 haut de gamme rénové, 2 chambres - à 1 min du métro Iberville (Villeray)</t>
+          <t>2 chambres avec balcon, immeuble rénové - rue Iberville (Villeray/Parc-Ex), à 1 min du métro d'Iberville</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
@@ -6051,17 +6051,17 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Secteur métro Iberville (H1X), Montréal</t>
+          <t>7186, Rue Iberville, Montréal</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>900</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
@@ -6081,7 +6081,7 @@
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L65" s="5" t="inlineStr">
@@ -6091,12 +6091,12 @@
       </c>
       <c r="M65" s="5" t="inlineStr">
         <is>
-          <t>Kijiji</t>
+          <t>DuProprio</t>
         </is>
       </c>
       <c r="N65" s="7" t="inlineStr">
         <is>
-          <t>https://www.kijiji.ca/v-apartments-condos/ville-de-montreal/5-haut-de-gamme-renove-a-2-pas-du-metro-iberville/1740921727</t>
+          <t>https://duproprio.com/fr/location/montreal/villeray-st-michel-parc-extension/5-1-2-a-louer/hab-7186-iberville-1132385</t>
         </is>
       </c>
       <c r="O65" s="5" t="inlineStr">
@@ -6106,12 +6106,12 @@
       </c>
       <c r="P65" s="6" t="inlineStr">
         <is>
-          <t>Entièrement rénové (printemps 2024), plancher chauffant salle de bain, grand balcon arrière couvert, aucun animal, disponible 1er juillet 2026</t>
+          <t>Entièrement rénové (2024), plancher chauffant salle de bain, grand balcon arrière couvert, aucun animal, Walk Score 94, disponible 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q65" s="5" t="inlineStr">
         <is>
-          <t>https://media.kijiji.ca/api/v1/ca-prod-fsbo-ads/images/b5/b541622f-9bb2-429e-b0b4-54478821573a?rule=kijijica-960-jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132385/villeray-st-michel-parc-extension-600-15662542.jpg</t>
         </is>
       </c>
     </row>
@@ -12902,22 +12902,22 @@
       </c>
       <c r="C144" s="6" t="inlineStr">
         <is>
-          <t>Condo 2 chambres, finitions haut de gamme - rue Durocher (Plateau), à 9 min du métro Place-des-Arts</t>
+          <t>3 chambres + bureau avec cour privée - rue Drolet (Villeray, près Jean-Talon/De Castelnau)</t>
         </is>
       </c>
       <c r="D144" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>3518, Rue Durocher, app. 303, Montréal</t>
+          <t>7372, Rue Drolet, Montréal</t>
         </is>
       </c>
       <c r="F144" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2350</t>
         </is>
       </c>
       <c r="G144" s="5" t="inlineStr">
@@ -12927,27 +12927,27 @@
       </c>
       <c r="H144" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I144" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J144" s="5" t="inlineStr">
         <is>
-          <t>Place-des-Arts</t>
+          <t>De Castelnau</t>
         </is>
       </c>
       <c r="K144" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L144" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M144" s="5" t="inlineStr">
@@ -12957,7 +12957,7 @@
       </c>
       <c r="N144" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/28667761</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/23857701</t>
         </is>
       </c>
       <c r="O144" s="5" t="inlineStr">
@@ -12967,19 +12967,19 @@
       </c>
       <c r="P144" s="6" t="inlineStr">
         <is>
-          <t>Finitions italiennes haut de gamme, entrée privée, vue sur parc, immeuble sécurisé (interphone/caméras), Walk Score 99, disponible 1 jour après acceptation, secteur Milton-Parc/McGill</t>
+          <t>Rez-de-chaussée avec cour privée (pas de balcon), immeuble de 1923, proche Marché Jean-Talon et Petite Italie, Walk Score 98, non-fumeur, animaux non acceptés, disponible 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q144" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE68A282DDDDDDDDDDA&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD115E0DDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
@@ -12989,22 +12989,22 @@
       </c>
       <c r="C145" s="6" t="inlineStr">
         <is>
-          <t>3 chambres + bureau avec cour privée - rue Drolet (Villeray, près Jean-Talon/De Castelnau)</t>
+          <t>2 chambres meublé, secteur Place Valois (Hochelaga), près métro Joliette</t>
         </is>
       </c>
       <c r="D145" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t>7372, Rue Drolet, Montréal</t>
+          <t>2117A, Rue Nicolet, Montréal</t>
         </is>
       </c>
       <c r="F145" s="5" t="inlineStr">
         <is>
-          <t>2350</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G145" s="5" t="inlineStr">
@@ -13014,27 +13014,27 @@
       </c>
       <c r="H145" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I145" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J145" s="5" t="inlineStr">
         <is>
-          <t>De Castelnau</t>
+          <t>Joliette</t>
         </is>
       </c>
       <c r="K145" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L145" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M145" s="5" t="inlineStr">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="N145" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/23857701</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/21083818</t>
         </is>
       </c>
       <c r="O145" s="5" t="inlineStr">
@@ -13054,12 +13054,12 @@
       </c>
       <c r="P145" s="6" t="inlineStr">
         <is>
-          <t>Rez-de-chaussée avec cour privée (pas de balcon), immeuble de 1923, proche Marché Jean-Talon et Petite Italie, Walk Score 98, non-fumeur, animaux non acceptés, disponible 1er juillet 2026</t>
+          <t>Meublé et équipé (laveuse-sécheuse, frigo, cuisinière, lave-vaisselle inclus), internet inclus, secteur Place Valois, Walk Score 97, disponible 7 jours après acceptation, superficie et balcon non précisés</t>
         </is>
       </c>
       <c r="Q145" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD115E0DDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15AD50DDDDDDDDDDE&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -13076,17 +13076,17 @@
       </c>
       <c r="C146" s="6" t="inlineStr">
         <is>
-          <t>2 chambres meublé, secteur Place Valois (Hochelaga), près métro Joliette</t>
+          <t>6½ (3 chambres), rez-de-chaussée avec cour et stationnement - 27e Avenue (Rosemont, près métro D'Iberville)</t>
         </is>
       </c>
       <c r="D146" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t>2117A, Rue Nicolet, Montréal</t>
+          <t>6749, 27e Avenue, Montréal</t>
         </is>
       </c>
       <c r="F146" s="5" t="inlineStr">
@@ -13101,7 +13101,7 @@
       </c>
       <c r="H146" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I146" s="5" t="inlineStr">
@@ -13111,17 +13111,17 @@
       </c>
       <c r="J146" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>D'Iberville</t>
         </is>
       </c>
       <c r="K146" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L146" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M146" s="5" t="inlineStr">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="N146" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/21083818</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/20987825</t>
         </is>
       </c>
       <c r="O146" s="5" t="inlineStr">
@@ -13141,12 +13141,12 @@
       </c>
       <c r="P146" s="6" t="inlineStr">
         <is>
-          <t>Meublé et équipé (laveuse-sécheuse, frigo, cuisinière, lave-vaisselle inclus), internet inclus, secteur Place Valois, Walk Score 97, disponible 7 jours après acceptation, superficie et balcon non précisés</t>
+          <t>7 pièces, rez-de-chaussée de triplex avec sous-sol, cour et stationnement inclus, animaux permis sur analyse, disponible 1er juillet 2026, métro Fabre aussi accessible (~5 min)</t>
         </is>
       </c>
       <c r="Q146" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15AD50DDDDDDDDDDE&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE6C9AB9DDDDDDDDDDC&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -13163,22 +13163,22 @@
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>6½ (3 chambres), rez-de-chaussée avec cour et stationnement - 27e Avenue (Rosemont, près métro D'Iberville)</t>
+          <t>5½ semi-meublé, 3 grandes chambres - rue Saint-Hubert (Villeray, près métro Jarry)</t>
         </is>
       </c>
       <c r="D147" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t>6749, 27e Avenue, Montréal</t>
+          <t>7635, Rue Saint-Hubert, Montréal</t>
         </is>
       </c>
       <c r="F147" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="G147" s="5" t="inlineStr">
@@ -13198,17 +13198,17 @@
       </c>
       <c r="J147" s="5" t="inlineStr">
         <is>
-          <t>D'Iberville</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K147" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L147" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M147" s="5" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="N147" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/20987825</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/25817021</t>
         </is>
       </c>
       <c r="O147" s="5" t="inlineStr">
@@ -13228,19 +13228,19 @@
       </c>
       <c r="P147" s="6" t="inlineStr">
         <is>
-          <t>7 pièces, rez-de-chaussée de triplex avec sous-sol, cour et stationnement inclus, animaux permis sur analyse, disponible 1er juillet 2026, métro Fabre aussi accessible (~5 min)</t>
+          <t>Semi-meublé, animaux acceptés sous conditions, disponible 1er juillet 2026, à ~11 min du métro Jarry (proche de la limite de 12 min) ; à ne pas confondre avec le 7639 rue Saint-Hubert déjà répertorié (adresse voisine, annonce distincte)</t>
         </is>
       </c>
       <c r="Q147" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE6C9AB9DDDDDDDDDDC&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD627F1DDDDDDDDDD2&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B148" s="5" t="inlineStr">
@@ -13250,22 +13250,22 @@
       </c>
       <c r="C148" s="6" t="inlineStr">
         <is>
-          <t>5½ semi-meublé, 3 grandes chambres - rue Saint-Hubert (Villeray, près métro Jarry)</t>
+          <t>4 chambres meublé, Plateau-Mont-Royal (Marketplace)</t>
         </is>
       </c>
       <c r="D148" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>7635, Rue Saint-Hubert, Montréal</t>
+          <t>3681, avenue Coloniale, Montréal (H2X 2Y7)</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G148" s="5" t="inlineStr">
@@ -13275,7 +13275,7 @@
       </c>
       <c r="H148" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I148" s="5" t="inlineStr">
@@ -13285,7 +13285,7 @@
       </c>
       <c r="J148" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Mont-Royal ou Sherbrooke (à vérifier)</t>
         </is>
       </c>
       <c r="K148" s="5" t="inlineStr">
@@ -13295,17 +13295,17 @@
       </c>
       <c r="L148" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M148" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N148" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/25817021</t>
+          <t>https://www.facebook.com/marketplace/item/1578661203923320</t>
         </is>
       </c>
       <c r="O148" s="5" t="inlineStr">
@@ -13315,19 +13315,19 @@
       </c>
       <c r="P148" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, animaux acceptés sous conditions, disponible 1er juillet 2026, à ~11 min du métro Jarry (proche de la limite de 12 min) ; à ne pas confondre avec le 7639 rue Saint-Hubert déjà répertorié (adresse voisine, annonce distincte)</t>
+          <t>Meublé, orienté étudiants, bail 1 an, dispo maintenant. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q148" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD627F1DDDDDDDDDD2&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/746058480_2385279625296639_1965210297754561149_n.jpg?stp=c93.0.895.895a_dst-jpg_tt6&amp;cstp=mx895x895&amp;ctp=s565x565&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=ngElLDKbnLQQ7kNvwHndFuc&amp;_nc_oc=AdpOYEcvWwImdnqaiYyy1pwfVcV2sab1mFRQ5KYGa5FE_CkYORsBa8yvv6PCL2lbQ7E&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=EorVHkPe0HNRZxtO75C5fg&amp;_nc_ss=7f2a8&amp;oh=00_AQBlE2b8WT_3jlX6ddiFysYujtaCjsMiZRfF96JJT7pp3g&amp;oe=6A60805A</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B149" s="5" t="inlineStr">
@@ -13337,17 +13337,17 @@
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>4 chambres meublé, Plateau-Mont-Royal (Marketplace)</t>
+          <t>4½ moderne, thermopompe - avenue Papineau (Centre-Sud)</t>
         </is>
       </c>
       <c r="D149" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Ville-Marie (Centre-Sud)</t>
         </is>
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t>3681, avenue Coloniale, Montréal (H2X 2Y7)</t>
+          <t>2121 Avenue Papineau, app. 106, Montréal</t>
         </is>
       </c>
       <c r="F149" s="5" t="inlineStr">
@@ -13362,52 +13362,52 @@
       </c>
       <c r="H149" s="5" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I149" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J149" s="5" t="inlineStr">
+        <is>
+          <t>Papineau</t>
+        </is>
+      </c>
+      <c r="K149" s="5" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L149" s="5" t="inlineStr">
+        <is>
+          <t>11 (estimé)</t>
+        </is>
+      </c>
+      <c r="M149" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="N149" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1345509854217640</t>
+        </is>
+      </c>
+      <c r="O149" s="5" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I149" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J149" s="5" t="inlineStr">
-        <is>
-          <t>Mont-Royal ou Sherbrooke (à vérifier)</t>
-        </is>
-      </c>
-      <c r="K149" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L149" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M149" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N149" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1578661203923320</t>
-        </is>
-      </c>
-      <c r="O149" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="P149" s="6" t="inlineStr">
         <is>
-          <t>Meublé, orienté étudiants, bail 1 an, dispo maintenant. Lien Facebook (connexion requise)</t>
+          <t>Thermopompe (chauffage/climatisation), 5 électros inclus, stationnement intérieur +200$/mois, dispo 1er sept 2026. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q149" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/746058480_2385279625296639_1965210297754561149_n.jpg?stp=c93.0.895.895a_dst-jpg_tt6&amp;cstp=mx895x895&amp;ctp=s565x565&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=ngElLDKbnLQQ7kNvwHndFuc&amp;_nc_oc=AdpOYEcvWwImdnqaiYyy1pwfVcV2sab1mFRQ5KYGa5FE_CkYORsBa8yvv6PCL2lbQ7E&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=EorVHkPe0HNRZxtO75C5fg&amp;_nc_ss=7f2a8&amp;oh=00_AQBlE2b8WT_3jlX6ddiFysYujtaCjsMiZRfF96JJT7pp3g&amp;oe=6A60805A</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/740967146_10163353758868282_6445879430357129287_n.jpg?stp=c267.0.1067.1067a_dst-jpg_tt6&amp;cstp=mx1067x1067&amp;ctp=s565x565&amp;_nc_cat=105&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=NBpCPM0lMZ0Q7kNvwEgcjRv&amp;_nc_oc=AdpKpJOW9gIXzADTI6MMd8QgF1AIUSvmXyA1OhFaypIfCHhp5Q_WLet_FlJK9JeWopU&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=po_Fub79cNJDfbGc2ZS1tQ&amp;_nc_ss=7f2a8&amp;oh=00_AQAYyDy-ZzVKaSsRH6KHfK-C3t6CRRIgCb8d-ae59ygZwA&amp;oe=6A5E8565</t>
         </is>
       </c>
     </row>
@@ -13424,22 +13424,22 @@
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>4½ moderne, thermopompe - avenue Papineau (Centre-Sud)</t>
+          <t>6 pièces, 3 chambres - rue Fabre (Rosemont)</t>
         </is>
       </c>
       <c r="D150" s="5" t="inlineStr">
         <is>
-          <t>Ville-Marie (Centre-Sud)</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>2121 Avenue Papineau, app. 106, Montréal</t>
+          <t>6525 Rue Fabre, app. 2, Montréal</t>
         </is>
       </c>
       <c r="F150" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="G150" s="5" t="inlineStr">
@@ -13449,7 +13449,7 @@
       </c>
       <c r="H150" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I150" s="5" t="inlineStr">
@@ -13459,27 +13459,27 @@
       </c>
       <c r="J150" s="5" t="inlineStr">
         <is>
-          <t>Papineau</t>
+          <t>Beaubien (à vérifier)</t>
         </is>
       </c>
       <c r="K150" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L150" s="5" t="inlineStr">
         <is>
-          <t>11 (estimé)</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M150" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N150" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1345509854217640</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/28139377</t>
         </is>
       </c>
       <c r="O150" s="5" t="inlineStr">
@@ -13489,19 +13489,19 @@
       </c>
       <c r="P150" s="6" t="inlineStr">
         <is>
-          <t>Thermopompe (chauffage/climatisation), 5 électros inclus, stationnement intérieur +200$/mois, dispo 1er sept 2026. Lien Facebook (connexion requise)</t>
+          <t>Semi-meublé, 1 stationnement (allée), Walk Score 95, dispo 7 jours après acceptation, station de métro non précisée par l'annonce</t>
         </is>
       </c>
       <c r="Q150" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/740967146_10163353758868282_6445879430357129287_n.jpg?stp=c267.0.1067.1067a_dst-jpg_tt6&amp;cstp=mx1067x1067&amp;ctp=s565x565&amp;_nc_cat=105&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=NBpCPM0lMZ0Q7kNvwEgcjRv&amp;_nc_oc=AdpKpJOW9gIXzADTI6MMd8QgF1AIUSvmXyA1OhFaypIfCHhp5Q_WLet_FlJK9JeWopU&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=po_Fub79cNJDfbGc2ZS1tQ&amp;_nc_ss=7f2a8&amp;oh=00_AQAYyDy-ZzVKaSsRH6KHfK-C3t6CRRIgCb8d-ae59ygZwA&amp;oe=6A5E8565</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA149845DDDDDDDDDDD&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B151" s="5" t="inlineStr">
@@ -13511,22 +13511,22 @@
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>6 pièces, 3 chambres - rue Fabre (Rosemont)</t>
+          <t>Grand 4 chambres + bureau – St-André bas Plateau</t>
         </is>
       </c>
       <c r="D151" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t>6525 Rue Fabre, app. 2, Montréal</t>
+          <t>3855 rue St-André (H2L 3V9)</t>
         </is>
       </c>
       <c r="F151" s="5" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="G151" s="5" t="inlineStr">
@@ -13536,7 +13536,7 @@
       </c>
       <c r="H151" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I151" s="5" t="inlineStr">
@@ -13546,7 +13546,7 @@
       </c>
       <c r="J151" s="5" t="inlineStr">
         <is>
-          <t>Beaubien (à vérifier)</t>
+          <t>Sherbrooke</t>
         </is>
       </c>
       <c r="K151" s="5" t="inlineStr">
@@ -13556,17 +13556,17 @@
       </c>
       <c r="L151" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M151" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N151" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/28139377</t>
+          <t>https://www.facebook.com/marketplace/item/1550150270173512</t>
         </is>
       </c>
       <c r="O151" s="5" t="inlineStr">
@@ -13576,19 +13576,19 @@
       </c>
       <c r="P151" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, 1 stationnement (allée), Walk Score 95, dispo 7 jours après acceptation, station de métro non précisée par l'annonce</t>
+          <t>4 chambres (dont 1 sans fenêtre) + bureau fermé, électros inclus, dispo 1er juillet. ~7 min à pied du métro Sherbrooke (estimé depuis l'adresse). Superficie non indiquée. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q151" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA149845DDDDDDDDDDD&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/728474326_10231683771185831_6727292866936668830_n.jpg?stp=c256.0.1537.1537a_dst-jpg_tt6&amp;cstp=mx1537x1537&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=943KDXUX1RQQ7kNvwFf3aXH&amp;_nc_oc=AdqiIy58nJFG1aGG5u9HQW6_QOL-2IMomb6kZpX5RbtE63MiJU-sRJMxj6FOz1Mq-C8&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=fqv6VHej6TNF8DZvOf_nSw&amp;_nc_ss=7f2a8&amp;oh=00_AQDIA5orKA1mjUQENX8o5T3X6Cteocg2jKTYaTNLxvUcJw&amp;oe=6A5D72DF</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B152" s="5" t="inlineStr">
@@ -13598,7 +13598,7 @@
       </c>
       <c r="C152" s="6" t="inlineStr">
         <is>
-          <t>Grand 4 chambres + bureau – St-André bas Plateau</t>
+          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
         </is>
       </c>
       <c r="D152" s="5" t="inlineStr">
@@ -13608,12 +13608,12 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t>3855 rue St-André (H2L 3V9)</t>
+          <t>4275 Rue de Bordeaux, Montréal</t>
         </is>
       </c>
       <c r="F152" s="5" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>2095</t>
         </is>
       </c>
       <c r="G152" s="5" t="inlineStr">
@@ -13623,59 +13623,59 @@
       </c>
       <c r="H152" s="5" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I152" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J152" s="5" t="inlineStr">
+        <is>
+          <t>Mont-Royal</t>
+        </is>
+      </c>
+      <c r="K152" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L152" s="5" t="inlineStr">
+        <is>
+          <t>10 (estimé)</t>
+        </is>
+      </c>
+      <c r="M152" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N152" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
+        </is>
+      </c>
+      <c r="O152" s="5" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I152" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J152" s="5" t="inlineStr">
-        <is>
-          <t>Sherbrooke</t>
-        </is>
-      </c>
-      <c r="K152" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L152" s="5" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="M152" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N152" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1550150270173512</t>
-        </is>
-      </c>
-      <c r="O152" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="P152" s="6" t="inlineStr">
         <is>
-          <t>4 chambres (dont 1 sans fenêtre) + bureau fermé, électros inclus, dispo 1er juillet. ~7 min à pied du métro Sherbrooke (estimé depuis l'adresse). Superficie non indiquée. Lien Facebook (connexion requise)</t>
+          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
         </is>
       </c>
       <c r="Q152" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/728474326_10231683771185831_6727292866936668830_n.jpg?stp=c256.0.1537.1537a_dst-jpg_tt6&amp;cstp=mx1537x1537&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=943KDXUX1RQQ7kNvwFf3aXH&amp;_nc_oc=AdqiIy58nJFG1aGG5u9HQW6_QOL-2IMomb6kZpX5RbtE63MiJU-sRJMxj6FOz1Mq-C8&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=fqv6VHej6TNF8DZvOf_nSw&amp;_nc_ss=7f2a8&amp;oh=00_AQDIA5orKA1mjUQENX8o5T3X6Cteocg2jKTYaTNLxvUcJw&amp;oe=6A5D72DF</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
+          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
         </is>
       </c>
       <c r="D153" s="5" t="inlineStr">
@@ -13695,12 +13695,12 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t>4275 Rue de Bordeaux, Montréal</t>
+          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
         </is>
       </c>
       <c r="F153" s="5" t="inlineStr">
         <is>
-          <t>2095</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G153" s="5" t="inlineStr">
@@ -13720,7 +13720,7 @@
       </c>
       <c r="J153" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Mont-Royal ou Papineau (à vérifier)</t>
         </is>
       </c>
       <c r="K153" s="5" t="inlineStr">
@@ -13730,7 +13730,7 @@
       </c>
       <c r="L153" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>12 (estimé)</t>
         </is>
       </c>
       <c r="M153" s="5" t="inlineStr">
@@ -13740,7 +13740,7 @@
       </c>
       <c r="N153" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
         </is>
       </c>
       <c r="O153" s="5" t="inlineStr">
@@ -13750,19 +13750,19 @@
       </c>
       <c r="P153" s="6" t="inlineStr">
         <is>
-          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
+          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
         </is>
       </c>
       <c r="Q153" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B154" s="5" t="inlineStr">
@@ -13772,7 +13772,7 @@
       </c>
       <c r="C154" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
+          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
         </is>
       </c>
       <c r="D154" s="5" t="inlineStr">
@@ -13782,12 +13782,12 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
+          <t>62 rue Rachel Est, Montréal</t>
         </is>
       </c>
       <c r="F154" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G154" s="5" t="inlineStr">
@@ -13807,7 +13807,7 @@
       </c>
       <c r="J154" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal ou Papineau (à vérifier)</t>
+          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
         </is>
       </c>
       <c r="K154" s="5" t="inlineStr">
@@ -13817,7 +13817,7 @@
       </c>
       <c r="L154" s="5" t="inlineStr">
         <is>
-          <t>12 (estimé)</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M154" s="5" t="inlineStr">
@@ -13827,7 +13827,7 @@
       </c>
       <c r="N154" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
         </is>
       </c>
       <c r="O154" s="5" t="inlineStr">
@@ -13837,19 +13837,19 @@
       </c>
       <c r="P154" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
+          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
         </is>
       </c>
       <c r="Q154" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B155" s="5" t="inlineStr">
@@ -13859,22 +13859,22 @@
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
+          <t>2 chambres - rue De Lanaudière (Rosemont), à 6 min du métro Jean-Talon</t>
         </is>
       </c>
       <c r="D155" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>62 rue Rachel Est, Montréal</t>
+          <t>6583, Rue De Lanaudière, Montréal</t>
         </is>
       </c>
       <c r="F155" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="G155" s="5" t="inlineStr">
@@ -13884,52 +13884,52 @@
       </c>
       <c r="H155" s="5" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I155" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J155" s="5" t="inlineStr">
+        <is>
+          <t>Jean-Talon</t>
+        </is>
+      </c>
+      <c r="K155" s="5" t="inlineStr">
+        <is>
+          <t>orange/bleue</t>
+        </is>
+      </c>
+      <c r="L155" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M155" s="5" t="inlineStr">
+        <is>
+          <t>Centris</t>
+        </is>
+      </c>
+      <c r="N155" s="7" t="inlineStr">
+        <is>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/20257676</t>
+        </is>
+      </c>
+      <c r="O155" s="5" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I155" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J155" s="5" t="inlineStr">
-        <is>
-          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
-        </is>
-      </c>
-      <c r="K155" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L155" s="5" t="inlineStr">
-        <is>
-          <t>8 (estimé)</t>
-        </is>
-      </c>
-      <c r="M155" s="5" t="inlineStr">
-        <is>
-          <t>DuProprio</t>
-        </is>
-      </c>
-      <c r="N155" s="7" t="inlineStr">
-        <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
-        </is>
-      </c>
-      <c r="O155" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="P155" s="6" t="inlineStr">
         <is>
-          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
+          <t>Chauffage central inclus + 5 électroménagers, quintuplex de 1932, disponible 1er sept. 2026, Walk Score 94</t>
         </is>
       </c>
       <c r="Q155" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15EA61DDDDDDDDDDE&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -13946,22 +13946,22 @@
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>2 chambres - rue De Lanaudière (Rosemont), à 6 min du métro Jean-Talon</t>
+          <t>2 chambres avec cour privée - rue Demers (Plateau), près du métro Laurier</t>
         </is>
       </c>
       <c r="D156" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E156" s="5" t="inlineStr">
         <is>
-          <t>6583, Rue De Lanaudière, Montréal</t>
+          <t>170, Rue Demers, Montréal</t>
         </is>
       </c>
       <c r="F156" s="5" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>2350</t>
         </is>
       </c>
       <c r="G156" s="5" t="inlineStr">
@@ -13976,22 +13976,22 @@
       </c>
       <c r="I156" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J156" s="5" t="inlineStr">
         <is>
-          <t>Jean-Talon</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K156" s="5" t="inlineStr">
         <is>
-          <t>orange/bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L156" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8-10 (estimé)</t>
         </is>
       </c>
       <c r="M156" s="5" t="inlineStr">
@@ -14001,7 +14001,7 @@
       </c>
       <c r="N156" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/20257676</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/15892581</t>
         </is>
       </c>
       <c r="O156" s="5" t="inlineStr">
@@ -14011,19 +14011,19 @@
       </c>
       <c r="P156" s="6" t="inlineStr">
         <is>
-          <t>Chauffage central inclus + 5 électroménagers, quintuplex de 1932, disponible 1er sept. 2026, Walk Score 94</t>
+          <t>Thermopompe murale incluse, meublé, cour privée (pas de balcon), animaux non acceptés, secteur Mile End, Walk Score 99</t>
         </is>
       </c>
       <c r="Q156" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15EA61DDDDDDDDDDE&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADFCE64DDDDDDDDDD1&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
@@ -14033,7 +14033,7 @@
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>2 chambres avec cour privée - rue Demers (Plateau), près du métro Laurier</t>
+          <t>Spacieux 4½ rénové, 2 chambres - avenue Henri-Julien (Plateau), à 2 min du métro Laurier</t>
         </is>
       </c>
       <c r="D157" s="5" t="inlineStr">
@@ -14043,12 +14043,12 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>170, Rue Demers, Montréal</t>
+          <t>5010, Avenue Henri-Julien, Montréal</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
         <is>
-          <t>2350</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G157" s="5" t="inlineStr">
@@ -14063,7 +14063,7 @@
       </c>
       <c r="I157" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J157" s="5" t="inlineStr">
@@ -14078,7 +14078,7 @@
       </c>
       <c r="L157" s="5" t="inlineStr">
         <is>
-          <t>8-10 (estimé)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M157" s="5" t="inlineStr">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="N157" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/15892581</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/13104221</t>
         </is>
       </c>
       <c r="O157" s="5" t="inlineStr">
@@ -14098,12 +14098,12 @@
       </c>
       <c r="P157" s="6" t="inlineStr">
         <is>
-          <t>Thermopompe murale incluse, meublé, cour privée (pas de balcon), animaux non acceptés, secteur Mile End, Walk Score 99</t>
+          <t>Cuisine et salle de bain rénovées, hauts plafonds, immeuble de 1910, chats acceptés, disponible 7 jours après acceptation, Walk Score 99</t>
         </is>
       </c>
       <c r="Q157" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADFCE64DDDDDDDDDD1&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA41C20BDDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -14120,7 +14120,7 @@
       </c>
       <c r="C158" s="6" t="inlineStr">
         <is>
-          <t>Spacieux 4½ rénové, 2 chambres - avenue Henri-Julien (Plateau), à 2 min du métro Laurier</t>
+          <t>4½ avec cour arrière privée - rue Rivard (Plateau), à quelques pas du métro Mont-Royal</t>
         </is>
       </c>
       <c r="D158" s="5" t="inlineStr">
@@ -14130,7 +14130,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t>5010, Avenue Henri-Julien, Montréal</t>
+          <t>4452, Rue Rivard, Montréal</t>
         </is>
       </c>
       <c r="F158" s="5" t="inlineStr">
@@ -14150,12 +14150,12 @@
       </c>
       <c r="I158" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J158" s="5" t="inlineStr">
         <is>
-          <t>Laurier</t>
+          <t>Mont-Royal</t>
         </is>
       </c>
       <c r="K158" s="5" t="inlineStr">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="L158" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3 (estimé)</t>
         </is>
       </c>
       <c r="M158" s="5" t="inlineStr">
@@ -14175,7 +14175,7 @@
       </c>
       <c r="N158" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/13104221</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/14560801</t>
         </is>
       </c>
       <c r="O158" s="5" t="inlineStr">
@@ -14185,12 +14185,12 @@
       </c>
       <c r="P158" s="6" t="inlineStr">
         <is>
-          <t>Cuisine et salle de bain rénovées, hauts plafonds, immeuble de 1910, chats acceptés, disponible 7 jours après acceptation, Walk Score 99</t>
+          <t>Cour arrière privée, lumineux et bien entretenu, Walk Score 100, animaux acceptés sous conditions, disponible 1er août 2026</t>
         </is>
       </c>
       <c r="Q158" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA41C20BDDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA44883FDDDDDDDDDDA&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -14207,22 +14207,22 @@
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>4½ avec cour arrière privée - rue Rivard (Plateau), à quelques pas du métro Mont-Royal</t>
+          <t>2 chambres, 6 pièces au total - rue De Normanville (Rosemont, secteur Beaubien)</t>
         </is>
       </c>
       <c r="D159" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
-          <t>4452, Rue Rivard, Montréal</t>
+          <t>6540, Rue De Normanville, Montréal</t>
         </is>
       </c>
       <c r="F159" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G159" s="5" t="inlineStr">
@@ -14237,12 +14237,12 @@
       </c>
       <c r="I159" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J159" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K159" s="5" t="inlineStr">
@@ -14252,7 +14252,7 @@
       </c>
       <c r="L159" s="5" t="inlineStr">
         <is>
-          <t>3 (estimé)</t>
+          <t>9 (estimé)</t>
         </is>
       </c>
       <c r="M159" s="5" t="inlineStr">
@@ -14262,7 +14262,7 @@
       </c>
       <c r="N159" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/14560801</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/15865457</t>
         </is>
       </c>
       <c r="O159" s="5" t="inlineStr">
@@ -14272,19 +14272,19 @@
       </c>
       <c r="P159" s="6" t="inlineStr">
         <is>
-          <t>Cour arrière privée, lumineux et bien entretenu, Walk Score 100, animaux acceptés sous conditions, disponible 1er août 2026</t>
+          <t>Entièrement meublé, rez-de-chaussée d'un immeuble de 1923, 6 pièces au total pour 2 chambres (suggère un espace généreux malgré l'absence de superficie précisée), animaux non acceptés, stationnement arrière en supplément, Walk Score 92, disponible 24 février 2026</t>
         </is>
       </c>
       <c r="Q159" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA44883FDDDDDDDDDDA&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE5DEDACDDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B160" s="5" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="C160" s="6" t="inlineStr">
         <is>
-          <t>2 chambres, 6 pièces au total - rue De Normanville (Rosemont, secteur Beaubien)</t>
+          <t>Grand 6 1/2, 2 chambres - rue Jean-Talon Est (Rosemont, près marché Jean-Talon)</t>
         </is>
       </c>
       <c r="D160" s="5" t="inlineStr">
@@ -14304,12 +14304,12 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t>6540, Rue De Normanville, Montréal</t>
+          <t>274, Rue Jean-Talon Est, app. 302, Montréal</t>
         </is>
       </c>
       <c r="F160" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G160" s="5" t="inlineStr">
@@ -14329,17 +14329,17 @@
       </c>
       <c r="J160" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Jean-Talon</t>
         </is>
       </c>
       <c r="K160" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>orange/bleue</t>
         </is>
       </c>
       <c r="L160" s="5" t="inlineStr">
         <is>
-          <t>9 (estimé)</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M160" s="5" t="inlineStr">
@@ -14349,7 +14349,7 @@
       </c>
       <c r="N160" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/15865457</t>
+          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/14545078</t>
         </is>
       </c>
       <c r="O160" s="5" t="inlineStr">
@@ -14359,19 +14359,19 @@
       </c>
       <c r="P160" s="6" t="inlineStr">
         <is>
-          <t>Entièrement meublé, rez-de-chaussée d'un immeuble de 1923, 6 pièces au total pour 2 chambres (suggère un espace généreux malgré l'absence de superficie précisée), animaux non acceptés, stationnement arrière en supplément, Walk Score 92, disponible 24 février 2026</t>
+          <t>6 pièces au total, concept ouvert, comptoirs de quartz, walk score 100, dispo 1er juillet 2026, près du marché Jean-Talon, superficie non précisée</t>
         </is>
       </c>
       <c r="Q160" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE5DEDACDDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADE4013DDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
@@ -14381,7 +14381,7 @@
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>Grand 6 1/2, 2 chambres - rue Jean-Talon Est (Rosemont, près marché Jean-Talon)</t>
+          <t>Cession de bail 7½, Rosemont-La Petite-Patrie (Marketplace)</t>
         </is>
       </c>
       <c r="D161" s="5" t="inlineStr">
@@ -14391,12 +14391,12 @@
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
-          <t>274, Rue Jean-Talon Est, app. 302, Montréal</t>
+          <t>n/d (Montréal, QC H2G 1T5)</t>
         </is>
       </c>
       <c r="F161" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2060</t>
         </is>
       </c>
       <c r="G161" s="5" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H161" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I161" s="5" t="inlineStr">
@@ -14416,27 +14416,27 @@
       </c>
       <c r="J161" s="5" t="inlineStr">
         <is>
-          <t>Jean-Talon</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K161" s="5" t="inlineStr">
         <is>
-          <t>orange/bleue</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L161" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M161" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N161" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/14545078</t>
+          <t>https://www.facebook.com/marketplace/item/1375157431101110</t>
         </is>
       </c>
       <c r="O161" s="5" t="inlineStr">
@@ -14446,12 +14446,12 @@
       </c>
       <c r="P161" s="6" t="inlineStr">
         <is>
-          <t>6 pièces au total, concept ouvert, comptoirs de quartz, walk score 100, dispo 1er juillet 2026, près du marché Jean-Talon, superficie non précisée</t>
+          <t>Cession de bail. Peu de détails disponibles dans l'annonce (pas d'adresse exacte ni de superficie). Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q161" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADE4013DDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/702670571_1710902896599779_1133264177050399379_n.jpg?stp=c0.86.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=110&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=akFqSvK3rfAQ7kNvwG-Cqey&amp;_nc_oc=Adrp5N9Rg13Pf-obfNZqB1ZqwyOcgjJji8vk0ggvRJiA9uCo-xDJXuQAit6O7YIGPW0&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=8ft2OWSslHjx1ccZ2nFb1w&amp;_nc_ss=7f2a8&amp;oh=00_AQBG56r36JKH2gkm4Baddcm0ylaFria-4p9Il0vYABnyMg&amp;oe=6A607060</t>
         </is>
       </c>
     </row>
@@ -14468,22 +14468,22 @@
       </c>
       <c r="C162" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail 7½, Rosemont-La Petite-Patrie (Marketplace)</t>
+          <t>Condo 2 chambres semi-meublé, stationnement intérieur - rue Villeray, à 9 min du métro Fabre</t>
         </is>
       </c>
       <c r="D162" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E162" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2G 1T5)</t>
+          <t>1414 Rue Villeray, app. 105, Montréal</t>
         </is>
       </c>
       <c r="F162" s="5" t="inlineStr">
         <is>
-          <t>2060</t>
+          <t>2350</t>
         </is>
       </c>
       <c r="G162" s="5" t="inlineStr">
@@ -14493,59 +14493,59 @@
       </c>
       <c r="H162" s="5" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I162" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J162" s="5" t="inlineStr">
+        <is>
+          <t>Fabre</t>
+        </is>
+      </c>
+      <c r="K162" s="5" t="inlineStr">
+        <is>
+          <t>bleue</t>
+        </is>
+      </c>
+      <c r="L162" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="M162" s="5" t="inlineStr">
+        <is>
+          <t>Centris</t>
+        </is>
+      </c>
+      <c r="N162" s="7" t="inlineStr">
+        <is>
+          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-villeray-saint-michel-parc-extension/25583093</t>
+        </is>
+      </c>
+      <c r="O162" s="5" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I162" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J162" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="K162" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="L162" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M162" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N162" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1375157431101110</t>
-        </is>
-      </c>
-      <c r="O162" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="P162" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail. Peu de détails disponibles dans l'annonce (pas d'adresse exacte ni de superficie). Lien Facebook (connexion requise)</t>
+          <t>Immeuble de 2011 (30 unités), RDC, plancher chauffant salle de bain, stationnement intérieur avec borne de recharge, casier de rangement, buanderie commune, terrasse sur le toit, Walk Score 94, dispo 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q162" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/702670571_1710902896599779_1133264177050399379_n.jpg?stp=c0.86.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=110&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=akFqSvK3rfAQ7kNvwG-Cqey&amp;_nc_oc=Adrp5N9Rg13Pf-obfNZqB1ZqwyOcgjJji8vk0ggvRJiA9uCo-xDJXuQAit6O7YIGPW0&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=8ft2OWSslHjx1ccZ2nFb1w&amp;_nc_ss=7f2a8&amp;oh=00_AQBG56r36JKH2gkm4Baddcm0ylaFria-4p9Il0vYABnyMg&amp;oe=6A607060</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD77D67DDDDDDDDDDB&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
@@ -14555,22 +14555,22 @@
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>Condo 2 chambres semi-meublé, stationnement intérieur - rue Villeray, à 9 min du métro Fabre</t>
+          <t>4½ rénové, 2 chambres, à 3-4 min du métro Sherbrooke</t>
         </is>
       </c>
       <c r="D163" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>1414 Rue Villeray, app. 105, Montréal</t>
+          <t>3711 Rue Saint-Urbain, app. A, Montréal</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
         <is>
-          <t>2350</t>
+          <t>2292</t>
         </is>
       </c>
       <c r="G163" s="5" t="inlineStr">
@@ -14590,17 +14590,17 @@
       </c>
       <c r="J163" s="5" t="inlineStr">
         <is>
-          <t>Fabre</t>
+          <t>Sherbrooke</t>
         </is>
       </c>
       <c r="K163" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L163" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M163" s="5" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
       <c r="N163" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-villeray-saint-michel-parc-extension/25583093</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/9588101</t>
         </is>
       </c>
       <c r="O163" s="5" t="inlineStr">
@@ -14620,12 +14620,12 @@
       </c>
       <c r="P163" s="6" t="inlineStr">
         <is>
-          <t>Immeuble de 2011 (30 unités), RDC, plancher chauffant salle de bain, stationnement intérieur avec borne de recharge, casier de rangement, buanderie commune, terrasse sur le toit, Walk Score 94, dispo 1er juillet 2026</t>
+          <t>Cuisine et salle de bain rénovées, plafonds hauts, tous électros inclus, Walk Score 100, dispo 5 jours après acceptation, à 5 min de McGill</t>
         </is>
       </c>
       <c r="Q163" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD77D67DDDDDDDDDDB&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE6F28A2DDDDDDDDDDB&amp;t=pi&amp;w=1024&amp;h=640&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -14642,22 +14642,22 @@
       </c>
       <c r="C164" s="6" t="inlineStr">
         <is>
-          <t>4½ rénové, 2 chambres, à 3-4 min du métro Sherbrooke</t>
+          <t>Appartement meublé haut de gamme - avenue Henri-Julien (Rosemont), près marché Jean-Talon</t>
         </is>
       </c>
       <c r="D164" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t>3711 Rue Saint-Urbain, app. A, Montréal</t>
+          <t>6391 Avenue Henri-Julien, Montréal</t>
         </is>
       </c>
       <c r="F164" s="5" t="inlineStr">
         <is>
-          <t>2292</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="G164" s="5" t="inlineStr">
@@ -14677,17 +14677,17 @@
       </c>
       <c r="J164" s="5" t="inlineStr">
         <is>
-          <t>Sherbrooke</t>
+          <t>Jean-Talon (à vérifier)</t>
         </is>
       </c>
       <c r="K164" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>orange/bleue</t>
         </is>
       </c>
       <c r="L164" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M164" s="5" t="inlineStr">
@@ -14697,7 +14697,7 @@
       </c>
       <c r="N164" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/9588101</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/10049540</t>
         </is>
       </c>
       <c r="O164" s="5" t="inlineStr">
@@ -14707,19 +14707,19 @@
       </c>
       <c r="P164" s="6" t="inlineStr">
         <is>
-          <t>Cuisine et salle de bain rénovées, plafonds hauts, tous électros inclus, Walk Score 100, dispo 5 jours après acceptation, à 5 min de McGill</t>
+          <t>Meublé, finitions haut de gamme, pas d'animaux, Walk Score 98, proche marché Jean-Talon et cafés/restos, dispo 1er juin 2026, distance au métro estimée</t>
         </is>
       </c>
       <c r="Q164" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE6F28A2DDDDDDDDDDB&amp;t=pi&amp;w=1024&amp;h=640&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADB62FFDDDDDDDDDDD&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr">
@@ -14729,22 +14729,22 @@
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>Appartement meublé haut de gamme - avenue Henri-Julien (Rosemont), près marché Jean-Talon</t>
+          <t>Superbe 2 chambres rénové, rue Beaubien - Petite-Italie</t>
         </is>
       </c>
       <c r="D165" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>La Petite-Patrie</t>
         </is>
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t>6391 Avenue Henri-Julien, Montréal</t>
+          <t>Rue Beaubien (Montréal, QC)</t>
         </is>
       </c>
       <c r="F165" s="5" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="G165" s="5" t="inlineStr">
@@ -14764,27 +14764,27 @@
       </c>
       <c r="J165" s="5" t="inlineStr">
         <is>
-          <t>Jean-Talon (à vérifier)</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K165" s="5" t="inlineStr">
         <is>
-          <t>orange/bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L165" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M165" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N165" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/10049540</t>
+          <t>https://www.facebook.com/marketplace/item/2219881575422253</t>
         </is>
       </c>
       <c r="O165" s="5" t="inlineStr">
@@ -14794,19 +14794,19 @@
       </c>
       <c r="P165" s="6" t="inlineStr">
         <is>
-          <t>Meublé, finitions haut de gamme, pas d'animaux, Walk Score 98, proche marché Jean-Talon et cafés/restos, dispo 1er juin 2026, distance au métro estimée</t>
+          <t>Entièrement rénové, cour arrière privée, Walk Score 99, à quelques pas de cafés/restos/boulangeries/épiceries fines de la Petite-Italie, à environ 10 min du marché Jean-Talon. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q165" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADB62FFDDDDDDDDDDD&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/714823210_969706739294886_222709070726311984_n.jpg?stp=c134.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=111&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=Q4rmFfALvM0Q7kNvwH2W42u&amp;_nc_oc=AdpINKj09PPc8Re8DxGgY3chRB5RnttQl9NAS-AFL9O8KTqqt1dR9NYx_1WNt0O8lww&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=JqfxygLQ7LNnSdbCmwTgsw&amp;_nc_ss=7f2a8&amp;oh=00_AQDsARrJ7YHo6O-8Zg1v5X3ykFLojfdUxVqQy1Z7t2iyQg&amp;oe=6A5DC11E</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B166" s="5" t="inlineStr">
@@ -14816,22 +14816,22 @@
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>Superbe 2 chambres rénové, rue Beaubien - Petite-Italie</t>
+          <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
         </is>
       </c>
       <c r="D166" s="5" t="inlineStr">
         <is>
-          <t>La Petite-Patrie</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t>Rue Beaubien (Montréal, QC)</t>
+          <t>1889 Rue des Carrières, Montréal</t>
         </is>
       </c>
       <c r="F166" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2375</t>
         </is>
       </c>
       <c r="G166" s="5" t="inlineStr">
@@ -14841,7 +14841,7 @@
       </c>
       <c r="H166" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I166" s="5" t="inlineStr">
@@ -14851,27 +14851,27 @@
       </c>
       <c r="J166" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K166" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L166" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M166" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N166" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/2219881575422253</t>
+          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
         </is>
       </c>
       <c r="O166" s="5" t="inlineStr">
@@ -14881,19 +14881,19 @@
       </c>
       <c r="P166" s="6" t="inlineStr">
         <is>
-          <t>Entièrement rénové, cour arrière privée, Walk Score 99, à quelques pas de cafés/restos/boulangeries/épiceries fines de la Petite-Italie, à environ 10 min du marché Jean-Talon. Lien Facebook (connexion requise)</t>
+          <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
         </is>
       </c>
       <c r="Q166" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/714823210_969706739294886_222709070726311984_n.jpg?stp=c134.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=111&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=Q4rmFfALvM0Q7kNvwH2W42u&amp;_nc_oc=AdpINKj09PPc8Re8DxGgY3chRB5RnttQl9NAS-AFL9O8KTqqt1dR9NYx_1WNt0O8lww&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=JqfxygLQ7LNnSdbCmwTgsw&amp;_nc_ss=7f2a8&amp;oh=00_AQDsARrJ7YHo6O-8Zg1v5X3ykFLojfdUxVqQy1Z7t2iyQg&amp;oe=6A5DC11E</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE603764DDDDDDDDDDD&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
@@ -14903,22 +14903,22 @@
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
+          <t>Appartement 5 1/2, Plateau-Mont-Royal (Marketplace)</t>
         </is>
       </c>
       <c r="D167" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>1889 Rue des Carrières, Montréal</t>
+          <t>n/d (Montréal, QC)</t>
         </is>
       </c>
       <c r="F167" s="5" t="inlineStr">
         <is>
-          <t>2375</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G167" s="5" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="H167" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I167" s="5" t="inlineStr">
@@ -14953,34 +14953,34 @@
       </c>
       <c r="M167" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N167" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
+          <t>https://www.facebook.com/marketplace/item/1552904606229687</t>
         </is>
       </c>
       <c r="O167" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P167" s="6" t="inlineStr">
         <is>
-          <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
+          <t>Annonce titre seulement, description non disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails</t>
         </is>
       </c>
       <c r="Q167" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE603764DDDDDDDDDDD&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/720906013_1532570941905242_5666371068595538123_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=YEDvMBzBavUQ7kNvwEkVbXh&amp;_nc_oc=AdqtpC8qtzZHEdxPx9e94VcYtRcN6s4rYqZkBbexWTpuWv5UghDk5D0a0ySf9p9btAk&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=TJJlLcUljG48fNVcDPZJaA&amp;_nc_ss=7f2a8&amp;oh=00_AQBrJbOYbvchb0Tq-5jSsFppBFkZ2xgQOdjHrsx0FadLHQ&amp;oe=6A632614</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="5" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B168" s="5" t="inlineStr">
@@ -14990,22 +14990,22 @@
       </c>
       <c r="C168" s="6" t="inlineStr">
         <is>
-          <t>Appartement 5 1/2, Plateau-Mont-Royal (Marketplace)</t>
+          <t>Beau 5½ à Nouveau Rosemont (Marketplace)</t>
         </is>
       </c>
       <c r="D168" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC)</t>
+          <t>n/d (secteur Nouveau-Rosemont, Montréal)</t>
         </is>
       </c>
       <c r="F168" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G168" s="5" t="inlineStr">
@@ -15045,7 +15045,7 @@
       </c>
       <c r="N168" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1552904606229687</t>
+          <t>https://www.facebook.com/marketplace/item/771126382598215</t>
         </is>
       </c>
       <c r="O168" s="5" t="inlineStr">
@@ -15055,19 +15055,19 @@
       </c>
       <c r="P168" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement, description non disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails</t>
+          <t>Peu de détails disponibles dans l'annonce (pas d'adresse exacte ni de superficie). Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q168" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/720906013_1532570941905242_5666371068595538123_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=YEDvMBzBavUQ7kNvwEkVbXh&amp;_nc_oc=AdqtpC8qtzZHEdxPx9e94VcYtRcN6s4rYqZkBbexWTpuWv5UghDk5D0a0ySf9p9btAk&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=TJJlLcUljG48fNVcDPZJaA&amp;_nc_ss=7f2a8&amp;oh=00_AQBrJbOYbvchb0Tq-5jSsFppBFkZ2xgQOdjHrsx0FadLHQ&amp;oe=6A632614</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/674573089_942123441857660_1258864760862245194_n.jpg?stp=c89.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=-PqFDWdPNa8Q7kNvwG9FoYC&amp;_nc_oc=Adqy82S_lfHjbp4dkLyXqO9W2nrNBD-zKhYTIwlodmCwj46lhM9QhEG2rupuBRJOPVI&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=8ft2OWSslHjx1ccZ2nFb1w&amp;_nc_ss=7f2a8&amp;oh=00_AQDV5R2cb2f6avoKzX1khDbQ_SvUKiySFkJsux9T10Rmdg&amp;oe=6A6059BA</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B169" s="5" t="inlineStr">
@@ -15077,7 +15077,7 @@
       </c>
       <c r="C169" s="6" t="inlineStr">
         <is>
-          <t>Beau 5½ à Nouveau Rosemont (Marketplace)</t>
+          <t>5-1/2 Rosemont (La Petite-Patrie)</t>
         </is>
       </c>
       <c r="D169" s="5" t="inlineStr">
@@ -15087,12 +15087,12 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t>n/d (secteur Nouveau-Rosemont, Montréal)</t>
+          <t>n/d (Montréal, QC)</t>
         </is>
       </c>
       <c r="F169" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G169" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="N169" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/771126382598215</t>
+          <t>https://www.facebook.com/marketplace/item/1249775127316090</t>
         </is>
       </c>
       <c r="O169" s="5" t="inlineStr">
@@ -15142,12 +15142,12 @@
       </c>
       <c r="P169" s="6" t="inlineStr">
         <is>
-          <t>Peu de détails disponibles dans l'annonce (pas d'adresse exacte ni de superficie). Lien Facebook (connexion requise)</t>
+          <t>Annonce titre seulement, description non disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails</t>
         </is>
       </c>
       <c r="Q169" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/674573089_942123441857660_1258864760862245194_n.jpg?stp=c89.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=-PqFDWdPNa8Q7kNvwG9FoYC&amp;_nc_oc=Adqy82S_lfHjbp4dkLyXqO9W2nrNBD-zKhYTIwlodmCwj46lhM9QhEG2rupuBRJOPVI&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=8ft2OWSslHjx1ccZ2nFb1w&amp;_nc_ss=7f2a8&amp;oh=00_AQDV5R2cb2f6avoKzX1khDbQ_SvUKiySFkJsux9T10Rmdg&amp;oe=6A6059BA</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/671899528_1686294965723943_4545041476511987210_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=xqmMQDvhJyAQ7kNvwH2BiIA&amp;_nc_oc=Adrb6HhJ7AWRb5Vln_jWCEMjozYYhefbdIyqNV0qQcHSggRpyTjrMcklU7eB9de9Y0s&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=POnFrCwMzHXIAMbS8hYJRQ&amp;_nc_ss=7f2a8&amp;oh=00_AQBeKgxbGCX6t2QjecZXjpQL0PuubZ84LadG2I8Gj_1mug&amp;oe=6A5E87C9</t>
         </is>
       </c>
     </row>
@@ -15164,7 +15164,7 @@
       </c>
       <c r="C170" s="6" t="inlineStr">
         <is>
-          <t>5-1/2 Rosemont (La Petite-Patrie)</t>
+          <t>5 1/2 lumineux à Rosemont - 2 chambres - Masson / Pie-IX</t>
         </is>
       </c>
       <c r="D170" s="5" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC)</t>
+          <t>n/d (secteur Masson / Pie-IX, Montréal)</t>
         </is>
       </c>
       <c r="F170" s="5" t="inlineStr">
@@ -15199,19 +15199,19 @@
       </c>
       <c r="J170" s="5" t="inlineStr">
         <is>
+          <t>Pie-IX (mentionné dans le titre)</t>
+        </is>
+      </c>
+      <c r="K170" s="5" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L170" s="5" t="inlineStr">
+        <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="K170" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="L170" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
       <c r="M170" s="5" t="inlineStr">
         <is>
           <t>Marketplace</t>
@@ -15219,7 +15219,7 @@
       </c>
       <c r="N170" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1249775127316090</t>
+          <t>https://www.facebook.com/marketplace/item/2238212030311408</t>
         </is>
       </c>
       <c r="O170" s="5" t="inlineStr">
@@ -15229,12 +15229,12 @@
       </c>
       <c r="P170" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement, description non disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails</t>
+          <t>Annonce titre seulement, description non disponible via le scraper ; secteur Masson/Pie-IX mentionné dans le titre mais distance exacte inconnue. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q170" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/671899528_1686294965723943_4545041476511987210_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=xqmMQDvhJyAQ7kNvwH2BiIA&amp;_nc_oc=Adrb6HhJ7AWRb5Vln_jWCEMjozYYhefbdIyqNV0qQcHSggRpyTjrMcklU7eB9de9Y0s&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=POnFrCwMzHXIAMbS8hYJRQ&amp;_nc_ss=7f2a8&amp;oh=00_AQBeKgxbGCX6t2QjecZXjpQL0PuubZ84LadG2I8Gj_1mug&amp;oe=6A5E87C9</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/719804341_36311671888447568_3859659500532179340_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=vtlzBRqRSRoQ7kNvwHzTYPO&amp;_nc_oc=AdoFOL6FWNc1M9UybWVnYuEzJQJlAq6neF5rbnVhe9_6oLH2S29hP6IEKy2E7BpCLDg&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQB2Z-K5zeotniKSOg35MSVtER8_xPmH2m9kSVj-TPJ32A&amp;oe=6A5E8CF7</t>
         </is>
       </c>
     </row>
@@ -15251,22 +15251,22 @@
       </c>
       <c r="C171" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 lumineux à Rosemont - 2 chambres - Masson / Pie-IX</t>
+          <t>Location 4 et demi Plateau, pet friendly</t>
         </is>
       </c>
       <c r="D171" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>n/d (secteur Masson / Pie-IX, Montréal)</t>
+          <t>n/d (Montréal, QC)</t>
         </is>
       </c>
       <c r="F171" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G171" s="5" t="inlineStr">
@@ -15286,12 +15286,12 @@
       </c>
       <c r="J171" s="5" t="inlineStr">
         <is>
-          <t>Pie-IX (mentionné dans le titre)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K171" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L171" s="5" t="inlineStr">
@@ -15306,7 +15306,7 @@
       </c>
       <c r="N171" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/2238212030311408</t>
+          <t>https://www.facebook.com/marketplace/item/880670661257255</t>
         </is>
       </c>
       <c r="O171" s="5" t="inlineStr">
@@ -15316,12 +15316,12 @@
       </c>
       <c r="P171" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement, description non disponible via le scraper ; secteur Masson/Pie-IX mentionné dans le titre mais distance exacte inconnue. Lien Facebook (connexion requise)</t>
+          <t>Annonce titre seulement (prix affiché entre 2150$ et 2350$), description non disponible via le scraper, animaux acceptés. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q171" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/719804341_36311671888447568_3859659500532179340_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=vtlzBRqRSRoQ7kNvwHzTYPO&amp;_nc_oc=AdoFOL6FWNc1M9UybWVnYuEzJQJlAq6neF5rbnVhe9_6oLH2S29hP6IEKy2E7BpCLDg&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQB2Z-K5zeotniKSOg35MSVtER8_xPmH2m9kSVj-TPJ32A&amp;oe=6A5E8CF7</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/739200097_2136278627323814_3520943268052786943_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=103&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=gPcahdqySPYQ7kNvwGsYlqA&amp;_nc_oc=Adr3EDMhZojMTr_b6P1fzAVXVarO60w-XBK6dTJaEUmqMft4FzmSbchZ5AfV6DC3Usw&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQBgwOGHm1ihFR3tvhrAE6VDaZym-txS_aF6xIBAwy5A1Q&amp;oe=6A5EA1A8</t>
         </is>
       </c>
     </row>
@@ -15338,12 +15338,12 @@
       </c>
       <c r="C172" s="6" t="inlineStr">
         <is>
-          <t>Location 4 et demi Plateau, pet friendly</t>
+          <t>5 1/2 Rosemont avec cour privée</t>
         </is>
       </c>
       <c r="D172" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E172" s="5" t="inlineStr">
@@ -15353,7 +15353,7 @@
       </c>
       <c r="F172" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2215</t>
         </is>
       </c>
       <c r="G172" s="5" t="inlineStr">
@@ -15393,7 +15393,7 @@
       </c>
       <c r="N172" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/880670661257255</t>
+          <t>https://www.facebook.com/marketplace/item/1493110625829174</t>
         </is>
       </c>
       <c r="O172" s="5" t="inlineStr">
@@ -15403,104 +15403,17 @@
       </c>
       <c r="P172" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement (prix affiché entre 2150$ et 2350$), description non disponible via le scraper, animaux acceptés. Lien Facebook (connexion requise)</t>
+          <t>Annonce titre seulement, description non disponible via le scraper ; cour privée mentionnée. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q172" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/739200097_2136278627323814_3520943268052786943_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=103&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=gPcahdqySPYQ7kNvwGsYlqA&amp;_nc_oc=Adr3EDMhZojMTr_b6P1fzAVXVarO60w-XBK6dTJaEUmqMft4FzmSbchZ5AfV6DC3Usw&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQBgwOGHm1ihFR3tvhrAE6VDaZym-txS_aF6xIBAwy5A1Q&amp;oe=6A5EA1A8</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="B173" s="5" t="inlineStr">
-        <is>
-          <t>vu</t>
-        </is>
-      </c>
-      <c r="C173" s="6" t="inlineStr">
-        <is>
-          <t>5 1/2 Rosemont avec cour privée</t>
-        </is>
-      </c>
-      <c r="D173" s="5" t="inlineStr">
-        <is>
-          <t>Rosemont-La Petite-Patrie</t>
-        </is>
-      </c>
-      <c r="E173" s="5" t="inlineStr">
-        <is>
-          <t>n/d (Montréal, QC)</t>
-        </is>
-      </c>
-      <c r="F173" s="5" t="inlineStr">
-        <is>
-          <t>2215</t>
-        </is>
-      </c>
-      <c r="G173" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="H173" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I173" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J173" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="K173" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="L173" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M173" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N173" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1493110625829174</t>
-        </is>
-      </c>
-      <c r="O173" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="P173" s="6" t="inlineStr">
-        <is>
-          <t>Annonce titre seulement, description non disponible via le scraper ; cour privée mentionnée. Lien Facebook (connexion requise)</t>
-        </is>
-      </c>
-      <c r="Q173" s="5" t="inlineStr">
-        <is>
           <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t45.5328-4/730530074_1035539099460685_3801485303896565628_n.jpg?stp=c313.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=110&amp;ccb=1-7&amp;_nc_sid=247b10&amp;_nc_ohc=_9b7saLCWEUQ7kNvwHrw_2v&amp;_nc_oc=AdoqEj5UFxI4lgfrZP0kbf8mdi_MJO6fIO-zv3fvQ5DsX656NtR6Rf8AiVxw-oho-l4&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQDqhmwAH6WdMqAuOtshO7wqRdBG7RkedN25_yaUpz5ikg&amp;oe=6A5EB662</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q173"/>
+  <autoFilter ref="A1:Q172"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -15673,7 +15586,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N170" r:id="rId169"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N171" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N172" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N173" r:id="rId172"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>